<commit_message>
Implement MainWindowController for improved window management and integrate TitleBar widget
</commit_message>
<xml_diff>
--- a/app/data/BangGia.xlsx
+++ b/app/data/BangGia.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\mtms\app\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C88767-CE16-47B3-847D-91B229B88CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="7800"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tổng Quát" sheetId="1" r:id="rId1"/>
@@ -26,19 +32,6 @@
     <definedName name="YOKO_NAME">'Tổng Quát'!$I$2:$I$1048576</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -1563,15 +1556,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1698,156 +1688,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="12"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1886,198 +1732,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.39994506668294322"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -2314,250 +1974,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="50">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="18" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="10" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="10" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="11" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2565,31 +1986,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -2597,95 +2012,95 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="11" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="11" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="11" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="13" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="13" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="1" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="1" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="3" fillId="4" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="15" fillId="3" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="15" fillId="3" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="15" fillId="3" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="15" fillId="3" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="15" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2697,63 +2112,26 @@
     <xf numFmtId="3" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="3">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal 2" xfId="49"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -3011,49 +2389,50 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AD110"/>
-  <sheetFormatPr defaultColWidth="9.11111111111111" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="14.8888888888889" style="2" customWidth="1"/>
-    <col min="2" max="2" width="12.6666666666667" style="3" customWidth="1"/>
-    <col min="3" max="3" width="22.6666666666667" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10.6666666666667" style="4" customWidth="1"/>
-    <col min="5" max="5" width="34.6666666666667" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.6666666666667" style="3" customWidth="1"/>
-    <col min="7" max="7" width="25.3333333333333" style="2" customWidth="1"/>
-    <col min="8" max="8" width="10.6666666666667" style="3" customWidth="1"/>
-    <col min="9" max="9" width="31.5555555555556" style="2" customWidth="1"/>
+    <col min="1" max="1" width="14.88671875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="34.6640625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="25.33203125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="31.5546875" style="2" customWidth="1"/>
     <col min="10" max="10" width="13" style="5" customWidth="1"/>
-    <col min="11" max="11" width="28.1111111111111" style="2" customWidth="1"/>
-    <col min="12" max="12" width="10.6666666666667" style="3" customWidth="1"/>
-    <col min="13" max="13" width="29.5555555555556" style="2" customWidth="1"/>
-    <col min="14" max="14" width="10.6666666666667" style="3" customWidth="1"/>
-    <col min="15" max="15" width="17.3333333333333" style="2" customWidth="1"/>
-    <col min="16" max="16" width="10.6666666666667" style="3" customWidth="1"/>
-    <col min="17" max="17" width="19.6666666666667" style="2" customWidth="1"/>
-    <col min="18" max="18" width="10.6666666666667" style="3" customWidth="1"/>
-    <col min="19" max="19" width="28.3333333333333" style="2" customWidth="1"/>
-    <col min="20" max="20" width="10.6666666666667" style="3" customWidth="1"/>
-    <col min="21" max="21" width="20.5555555555556" style="2" customWidth="1"/>
-    <col min="22" max="22" width="10.6666666666667" style="3" customWidth="1"/>
-    <col min="23" max="23" width="21.5555555555556" style="2" customWidth="1"/>
-    <col min="24" max="24" width="10.6666666666667" style="3" customWidth="1"/>
-    <col min="25" max="25" width="26.6666666666667" style="2" customWidth="1"/>
-    <col min="26" max="26" width="10.6666666666667" style="3" customWidth="1"/>
-    <col min="27" max="27" width="33.4444444444444" style="2" customWidth="1"/>
-    <col min="28" max="28" width="22.5555555555556" style="3" customWidth="1"/>
-    <col min="29" max="29" width="19.4444444444444" style="2" customWidth="1"/>
+    <col min="11" max="11" width="28.109375" style="2" customWidth="1"/>
+    <col min="12" max="12" width="10.6640625" style="3" customWidth="1"/>
+    <col min="13" max="13" width="29.5546875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="10.6640625" style="3" customWidth="1"/>
+    <col min="15" max="15" width="17.33203125" style="2" customWidth="1"/>
+    <col min="16" max="16" width="10.6640625" style="3" customWidth="1"/>
+    <col min="17" max="17" width="19.6640625" style="2" customWidth="1"/>
+    <col min="18" max="18" width="10.6640625" style="3" customWidth="1"/>
+    <col min="19" max="19" width="28.33203125" style="2" customWidth="1"/>
+    <col min="20" max="20" width="10.6640625" style="3" customWidth="1"/>
+    <col min="21" max="21" width="20.5546875" style="2" customWidth="1"/>
+    <col min="22" max="22" width="10.6640625" style="3" customWidth="1"/>
+    <col min="23" max="23" width="21.5546875" style="2" customWidth="1"/>
+    <col min="24" max="24" width="10.6640625" style="3" customWidth="1"/>
+    <col min="25" max="25" width="26.6640625" style="2" customWidth="1"/>
+    <col min="26" max="26" width="10.6640625" style="3" customWidth="1"/>
+    <col min="27" max="27" width="33.44140625" style="2" customWidth="1"/>
+    <col min="28" max="28" width="22.5546875" style="3" customWidth="1"/>
+    <col min="29" max="29" width="19.44140625" style="2" customWidth="1"/>
     <col min="30" max="30" width="18" style="2" customWidth="1"/>
-    <col min="31" max="16384" width="9.11111111111111" style="2"/>
+    <col min="31" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="15.15" spans="1:30">
+    <row r="1" spans="1:30" s="1" customFormat="1">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -3110,22 +2489,22 @@
         <v>13</v>
       </c>
       <c r="AB1" s="9"/>
-      <c r="AC1" s="11" t="s">
+      <c r="AC1" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="AD1" s="12"/>
+      <c r="AD1" s="74"/>
     </row>
     <row r="2" spans="1:30">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="11" t="s">
         <v>15</v>
       </c>
       <c r="B2" s="3">
         <v>239000</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="14"/>
+      <c r="D2" s="12"/>
       <c r="E2" s="2" t="s">
         <v>17</v>
       </c>
@@ -3141,7 +2520,7 @@
       <c r="I2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="15">
+      <c r="J2" s="13">
         <v>152000</v>
       </c>
       <c r="K2" s="2" t="s">
@@ -3172,7 +2551,7 @@
         <v>25</v>
       </c>
       <c r="V2" s="3">
-        <v>222000</v>
+        <v>226000</v>
       </c>
       <c r="W2" s="2" t="s">
         <v>26</v>
@@ -3200,16 +2579,16 @@
       </c>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="11" t="s">
         <v>30</v>
       </c>
       <c r="B3" s="3">
         <v>252000</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="14"/>
+      <c r="D3" s="12"/>
       <c r="E3" s="2" t="s">
         <v>32</v>
       </c>
@@ -3225,7 +2604,7 @@
       <c r="I3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J3" s="16">
+      <c r="J3" s="14">
         <v>204000</v>
       </c>
       <c r="K3" s="2" t="s">
@@ -3256,7 +2635,7 @@
         <v>40</v>
       </c>
       <c r="V3" s="3">
-        <v>209000</v>
+        <v>212000</v>
       </c>
       <c r="W3" s="2" t="s">
         <v>41</v>
@@ -3284,16 +2663,16 @@
       </c>
     </row>
     <row r="4" spans="1:30">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="11" t="s">
         <v>45</v>
       </c>
       <c r="B4" s="3">
         <v>280000</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="14"/>
+      <c r="D4" s="12"/>
       <c r="E4" s="2" t="s">
         <v>47</v>
       </c>
@@ -3306,10 +2685,10 @@
       <c r="H4" s="3">
         <v>192000</v>
       </c>
-      <c r="I4" s="17" t="s">
+      <c r="I4" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="J4" s="18">
+      <c r="J4" s="16">
         <v>151000</v>
       </c>
       <c r="K4" s="2" t="s">
@@ -3340,7 +2719,7 @@
         <v>55</v>
       </c>
       <c r="V4" s="3">
-        <v>194000</v>
+        <v>198000</v>
       </c>
       <c r="W4" s="2" t="s">
         <v>56</v>
@@ -3368,16 +2747,16 @@
       </c>
     </row>
     <row r="5" spans="1:30">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="11" t="s">
         <v>60</v>
       </c>
       <c r="B5" s="3">
         <v>221000</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="14"/>
+      <c r="D5" s="12"/>
       <c r="E5" s="2" t="s">
         <v>62</v>
       </c>
@@ -3390,10 +2769,10 @@
       <c r="H5" s="3">
         <v>192000</v>
       </c>
-      <c r="I5" s="17" t="s">
+      <c r="I5" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="J5" s="19">
+      <c r="J5" s="17">
         <v>192000</v>
       </c>
       <c r="K5" s="2" t="s">
@@ -3424,7 +2803,7 @@
         <v>70</v>
       </c>
       <c r="V5" s="3">
-        <v>249000</v>
+        <v>254000</v>
       </c>
       <c r="W5" s="2" t="s">
         <v>71</v>
@@ -3452,16 +2831,16 @@
       </c>
     </row>
     <row r="6" spans="1:30">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="11" t="s">
         <v>75</v>
       </c>
       <c r="B6" s="3">
         <v>249000</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="D6" s="14"/>
+      <c r="D6" s="12"/>
       <c r="E6" s="2" t="s">
         <v>77</v>
       </c>
@@ -3477,7 +2856,7 @@
       <c r="I6" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="13">
         <v>177000</v>
       </c>
       <c r="K6" s="2" t="s">
@@ -3508,7 +2887,7 @@
         <v>85</v>
       </c>
       <c r="V6" s="3">
-        <v>316000</v>
+        <v>322000</v>
       </c>
       <c r="W6" s="2" t="s">
         <v>86</v>
@@ -3536,16 +2915,16 @@
       </c>
     </row>
     <row r="7" spans="1:30">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="11" t="s">
         <v>90</v>
       </c>
       <c r="B7" s="3">
         <v>382000</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="D7" s="14"/>
+      <c r="D7" s="12"/>
       <c r="E7" s="2" t="s">
         <v>92</v>
       </c>
@@ -3561,7 +2940,7 @@
       <c r="I7" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="J7" s="16">
+      <c r="J7" s="14">
         <v>228000</v>
       </c>
       <c r="K7" s="2" t="s">
@@ -3592,7 +2971,7 @@
         <v>100</v>
       </c>
       <c r="V7" s="3">
-        <v>348000</v>
+        <v>355000</v>
       </c>
       <c r="W7" s="2" t="s">
         <v>101</v>
@@ -3620,16 +2999,16 @@
       </c>
     </row>
     <row r="8" spans="1:30">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="11" t="s">
         <v>105</v>
       </c>
       <c r="B8" s="3">
         <v>412000</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="14"/>
+      <c r="D8" s="12"/>
       <c r="E8" s="2" t="s">
         <v>107</v>
       </c>
@@ -3639,13 +3018,13 @@
       <c r="G8" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="H8" s="20">
+      <c r="H8" s="18">
         <v>286000</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J8" s="15">
+      <c r="J8" s="13">
         <v>212000</v>
       </c>
       <c r="K8" s="2" t="s">
@@ -3676,7 +3055,7 @@
         <v>115</v>
       </c>
       <c r="V8" s="3">
-        <v>380000</v>
+        <v>387000</v>
       </c>
       <c r="W8" s="2" t="s">
         <v>116</v>
@@ -3704,16 +3083,16 @@
       </c>
     </row>
     <row r="9" spans="1:30">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="11" t="s">
         <v>120</v>
       </c>
       <c r="B9" s="3">
         <v>347000</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="D9" s="14"/>
+      <c r="D9" s="12"/>
       <c r="E9" s="2" t="s">
         <v>122</v>
       </c>
@@ -3729,7 +3108,7 @@
       <c r="I9" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="J9" s="16">
+      <c r="J9" s="14">
         <v>287000</v>
       </c>
       <c r="K9" s="2" t="s">
@@ -3753,14 +3132,14 @@
       <c r="S9" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="T9" s="21">
+      <c r="T9" s="19">
         <v>260000</v>
       </c>
       <c r="U9" s="2" t="s">
         <v>130</v>
       </c>
       <c r="V9" s="3">
-        <v>332000</v>
+        <v>338000</v>
       </c>
       <c r="W9" s="2" t="s">
         <v>131</v>
@@ -3788,32 +3167,32 @@
       </c>
     </row>
     <row r="10" spans="1:30">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="11" t="s">
         <v>135</v>
       </c>
       <c r="B10" s="3">
         <v>221000</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="D10" s="14"/>
+      <c r="D10" s="12"/>
       <c r="E10" s="2" t="s">
         <v>137</v>
       </c>
       <c r="F10" s="3">
         <v>282000</v>
       </c>
-      <c r="G10" s="22" t="s">
+      <c r="G10" s="20" t="s">
         <v>138</v>
       </c>
-      <c r="H10" s="23">
+      <c r="H10" s="21">
         <v>348000</v>
       </c>
-      <c r="I10" s="24" t="s">
+      <c r="I10" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="J10" s="25">
+      <c r="J10" s="23">
         <v>218000</v>
       </c>
       <c r="K10" s="2" t="s">
@@ -3844,7 +3223,7 @@
         <v>145</v>
       </c>
       <c r="V10" s="3">
-        <v>607000</v>
+        <v>620000</v>
       </c>
       <c r="W10" s="2" t="s">
         <v>146</v>
@@ -3878,26 +3257,26 @@
       <c r="B11" s="3">
         <v>332000</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="D11" s="14"/>
+      <c r="D11" s="12"/>
       <c r="E11" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F11" s="3">
         <v>235000</v>
       </c>
-      <c r="G11" s="22" t="s">
+      <c r="G11" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="21">
         <v>370000</v>
       </c>
-      <c r="I11" s="24" t="s">
+      <c r="I11" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="J11" s="26">
+      <c r="J11" s="24">
         <v>270000</v>
       </c>
       <c r="K11" s="2" t="s">
@@ -3962,26 +3341,26 @@
       <c r="B12" s="3">
         <v>800000</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="D12" s="14"/>
+      <c r="D12" s="12"/>
       <c r="E12" s="2" t="s">
         <v>167</v>
       </c>
       <c r="F12" s="3">
         <v>289000</v>
       </c>
-      <c r="G12" s="22" t="s">
+      <c r="G12" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="H12" s="27">
+      <c r="H12" s="25">
         <v>348000</v>
       </c>
-      <c r="I12" s="17" t="s">
+      <c r="I12" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="J12" s="28">
+      <c r="J12" s="26">
         <v>395000</v>
       </c>
       <c r="K12" s="2" t="s">
@@ -4040,29 +3419,29 @@
       </c>
     </row>
     <row r="13" spans="1:30">
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="27" t="s">
         <v>180</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="D13" s="14"/>
-      <c r="E13" s="24" t="s">
+      <c r="D13" s="12"/>
+      <c r="E13" s="22" t="s">
         <v>182</v>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="19">
         <v>254000</v>
       </c>
-      <c r="G13" s="22" t="s">
+      <c r="G13" s="20" t="s">
         <v>183</v>
       </c>
-      <c r="H13" s="27">
+      <c r="H13" s="25">
         <v>370000</v>
       </c>
-      <c r="I13" s="17" t="s">
+      <c r="I13" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="J13" s="30">
+      <c r="J13" s="28">
         <v>431000</v>
       </c>
       <c r="K13" s="2" t="s">
@@ -4121,26 +3500,26 @@
       </c>
     </row>
     <row r="14" spans="1:30">
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="D14" s="14"/>
-      <c r="E14" s="24" t="s">
+      <c r="D14" s="12"/>
+      <c r="E14" s="22" t="s">
         <v>195</v>
       </c>
-      <c r="F14" s="21">
+      <c r="F14" s="19">
         <v>291000</v>
       </c>
-      <c r="G14" s="31" t="s">
+      <c r="G14" s="29" t="s">
         <v>196</v>
       </c>
-      <c r="H14" s="32">
+      <c r="H14" s="30">
         <v>281000</v>
       </c>
-      <c r="I14" s="17" t="s">
+      <c r="I14" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="J14" s="19">
+      <c r="J14" s="17">
         <v>286000</v>
       </c>
       <c r="K14" s="2" t="s">
@@ -4199,26 +3578,26 @@
       </c>
     </row>
     <row r="15" spans="1:30">
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="D15" s="14"/>
+      <c r="D15" s="12"/>
       <c r="E15" s="3" t="s">
         <v>209</v>
       </c>
       <c r="F15" s="3">
         <v>214000</v>
       </c>
-      <c r="G15" s="31" t="s">
+      <c r="G15" s="29" t="s">
         <v>210</v>
       </c>
-      <c r="H15" s="32">
+      <c r="H15" s="30">
         <v>358000</v>
       </c>
-      <c r="I15" s="17" t="s">
+      <c r="I15" s="15" t="s">
         <v>211</v>
       </c>
-      <c r="J15" s="18">
+      <c r="J15" s="16">
         <v>334000</v>
       </c>
       <c r="K15" s="2" t="s">
@@ -4268,26 +3647,26 @@
       </c>
     </row>
     <row r="16" spans="1:30">
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="11" t="s">
         <v>220</v>
       </c>
-      <c r="D16" s="14"/>
+      <c r="D16" s="12"/>
       <c r="E16" s="2" t="s">
         <v>221</v>
       </c>
       <c r="F16" s="3">
         <v>266000</v>
       </c>
-      <c r="G16" s="31" t="s">
+      <c r="G16" s="29" t="s">
         <v>222</v>
       </c>
-      <c r="H16" s="32">
+      <c r="H16" s="30">
         <v>442000</v>
       </c>
-      <c r="I16" s="17" t="s">
+      <c r="I16" s="15" t="s">
         <v>223</v>
       </c>
-      <c r="J16" s="19">
+      <c r="J16" s="17">
         <v>269000</v>
       </c>
       <c r="K16" s="2" t="s">
@@ -4337,26 +3716,26 @@
       </c>
     </row>
     <row r="17" spans="3:30">
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="D17" s="14"/>
+      <c r="D17" s="12"/>
       <c r="E17" s="2" t="s">
         <v>233</v>
       </c>
       <c r="F17" s="3">
         <v>235000</v>
       </c>
-      <c r="G17" s="31" t="s">
+      <c r="G17" s="29" t="s">
         <v>234</v>
       </c>
-      <c r="H17" s="32">
+      <c r="H17" s="30">
         <v>374000</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="J17" s="15">
+      <c r="J17" s="13">
         <v>312000</v>
       </c>
       <c r="K17" s="2" t="s">
@@ -4406,26 +3785,26 @@
       </c>
     </row>
     <row r="18" spans="3:30">
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="D18" s="14"/>
+      <c r="D18" s="12"/>
       <c r="E18" s="2" t="s">
         <v>245</v>
       </c>
       <c r="F18" s="3">
         <v>293000</v>
       </c>
-      <c r="G18" s="31" t="s">
+      <c r="G18" s="29" t="s">
         <v>246</v>
       </c>
-      <c r="H18" s="32">
+      <c r="H18" s="30">
         <v>374000</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="J18" s="33">
+      <c r="J18" s="31">
         <v>375000</v>
       </c>
       <c r="K18" s="2" t="s">
@@ -4475,26 +3854,26 @@
       </c>
     </row>
     <row r="19" spans="3:30">
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="11" t="s">
         <v>256</v>
       </c>
-      <c r="D19" s="14"/>
+      <c r="D19" s="12"/>
       <c r="E19" s="2" t="s">
         <v>257</v>
       </c>
       <c r="F19" s="3">
         <v>267000</v>
       </c>
-      <c r="G19" s="31" t="s">
+      <c r="G19" s="29" t="s">
         <v>258</v>
       </c>
-      <c r="H19" s="32">
+      <c r="H19" s="30">
         <v>298000</v>
       </c>
-      <c r="I19" s="24" t="s">
+      <c r="I19" s="22" t="s">
         <v>259</v>
       </c>
-      <c r="J19" s="26">
+      <c r="J19" s="24">
         <v>317000</v>
       </c>
       <c r="K19" s="2" t="s">
@@ -4544,26 +3923,26 @@
       </c>
     </row>
     <row r="20" spans="3:30">
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="11" t="s">
         <v>268</v>
       </c>
-      <c r="D20" s="14"/>
+      <c r="D20" s="12"/>
       <c r="E20" s="2" t="s">
         <v>269</v>
       </c>
       <c r="F20" s="3">
         <v>340000</v>
       </c>
-      <c r="G20" s="31" t="s">
+      <c r="G20" s="29" t="s">
         <v>270</v>
       </c>
-      <c r="H20" s="32">
+      <c r="H20" s="30">
         <v>366000</v>
       </c>
-      <c r="I20" s="34" t="s">
+      <c r="I20" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="J20" s="35">
+      <c r="J20" s="33">
         <v>417000</v>
       </c>
       <c r="K20" s="2" t="s">
@@ -4584,7 +3963,7 @@
       <c r="S20" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="T20" s="21">
+      <c r="T20" s="19">
         <v>431000</v>
       </c>
       <c r="U20" s="2" t="s">
@@ -4616,26 +3995,26 @@
       </c>
     </row>
     <row r="21" spans="3:30">
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="11" t="s">
         <v>280</v>
       </c>
-      <c r="D21" s="14"/>
+      <c r="D21" s="12"/>
       <c r="E21" s="2" t="s">
         <v>281</v>
       </c>
       <c r="F21" s="3">
         <v>411000</v>
       </c>
-      <c r="G21" s="31" t="s">
+      <c r="G21" s="29" t="s">
         <v>282</v>
       </c>
-      <c r="H21" s="32">
+      <c r="H21" s="30">
         <v>330000</v>
       </c>
-      <c r="I21" s="34" t="s">
+      <c r="I21" s="32" t="s">
         <v>283</v>
       </c>
-      <c r="J21" s="36">
+      <c r="J21" s="34">
         <v>373000</v>
       </c>
       <c r="K21" s="2" t="s">
@@ -4667,26 +4046,26 @@
       </c>
     </row>
     <row r="22" spans="3:30">
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="11" t="s">
         <v>289</v>
       </c>
-      <c r="D22" s="14"/>
+      <c r="D22" s="12"/>
       <c r="E22" s="2" t="s">
         <v>290</v>
       </c>
       <c r="F22" s="3">
         <v>320000</v>
       </c>
-      <c r="G22" s="31" t="s">
+      <c r="G22" s="29" t="s">
         <v>291</v>
       </c>
-      <c r="H22" s="32">
+      <c r="H22" s="30">
         <v>340000</v>
       </c>
-      <c r="I22" s="34" t="s">
+      <c r="I22" s="32" t="s">
         <v>292</v>
       </c>
-      <c r="J22" s="37">
+      <c r="J22" s="35">
         <v>467000</v>
       </c>
       <c r="K22" s="2" t="s">
@@ -4712,26 +4091,26 @@
       </c>
     </row>
     <row r="23" spans="3:30">
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="11" t="s">
         <v>298</v>
       </c>
-      <c r="D23" s="14"/>
+      <c r="D23" s="12"/>
       <c r="E23" s="2" t="s">
         <v>299</v>
       </c>
       <c r="F23" s="3">
         <v>345000</v>
       </c>
-      <c r="G23" s="31" t="s">
+      <c r="G23" s="29" t="s">
         <v>300</v>
       </c>
-      <c r="H23" s="32">
+      <c r="H23" s="30">
         <v>360000</v>
       </c>
-      <c r="I23" s="38" t="s">
+      <c r="I23" s="36" t="s">
         <v>301</v>
       </c>
-      <c r="J23" s="39">
+      <c r="J23" s="37">
         <v>299000</v>
       </c>
       <c r="K23" s="2" t="s">
@@ -4757,26 +4136,26 @@
       </c>
     </row>
     <row r="24" spans="3:30">
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="11" t="s">
         <v>306</v>
       </c>
-      <c r="D24" s="14"/>
-      <c r="E24" s="22" t="s">
+      <c r="D24" s="12"/>
+      <c r="E24" s="20" t="s">
         <v>307</v>
       </c>
-      <c r="F24" s="27">
+      <c r="F24" s="25">
         <v>309000</v>
       </c>
-      <c r="G24" s="40" t="s">
+      <c r="G24" s="38" t="s">
         <v>308</v>
       </c>
-      <c r="H24" s="41">
+      <c r="H24" s="39">
         <v>269000</v>
       </c>
-      <c r="I24" s="38" t="s">
+      <c r="I24" s="36" t="s">
         <v>309</v>
       </c>
-      <c r="J24" s="42">
+      <c r="J24" s="40">
         <v>321000</v>
       </c>
       <c r="K24" s="2" t="s">
@@ -4802,26 +4181,26 @@
       </c>
     </row>
     <row r="25" spans="3:30">
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="11" t="s">
         <v>314</v>
       </c>
-      <c r="D25" s="14"/>
-      <c r="E25" s="22" t="s">
+      <c r="D25" s="12"/>
+      <c r="E25" s="20" t="s">
         <v>315</v>
       </c>
-      <c r="F25" s="27">
+      <c r="F25" s="25">
         <v>369000</v>
       </c>
-      <c r="G25" s="31" t="s">
+      <c r="G25" s="29" t="s">
         <v>316</v>
       </c>
-      <c r="H25" s="32">
+      <c r="H25" s="30">
         <v>396000</v>
       </c>
-      <c r="I25" s="43" t="s">
+      <c r="I25" s="41" t="s">
         <v>317</v>
       </c>
-      <c r="J25" s="44">
+      <c r="J25" s="42">
         <v>329000</v>
       </c>
       <c r="K25" s="2" t="s">
@@ -4846,27 +4225,27 @@
         <v>17000</v>
       </c>
     </row>
-    <row r="26" ht="15.15" spans="3:30">
+    <row r="26" spans="3:30">
       <c r="C26" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="D26" s="14"/>
-      <c r="E26" s="22" t="s">
+      <c r="D26" s="12"/>
+      <c r="E26" s="20" t="s">
         <v>323</v>
       </c>
-      <c r="F26" s="27">
+      <c r="F26" s="25">
         <v>372000</v>
       </c>
-      <c r="G26" s="31" t="s">
+      <c r="G26" s="29" t="s">
         <v>324</v>
       </c>
-      <c r="H26" s="32">
+      <c r="H26" s="30">
         <v>441000</v>
       </c>
-      <c r="I26" s="43" t="s">
+      <c r="I26" s="41" t="s">
         <v>325</v>
       </c>
-      <c r="J26" s="45">
+      <c r="J26" s="43">
         <v>349000</v>
       </c>
       <c r="K26" s="2" t="s">
@@ -4886,26 +4265,26 @@
       </c>
     </row>
     <row r="27" spans="3:30">
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="11" t="s">
         <v>329</v>
       </c>
-      <c r="D27" s="14"/>
-      <c r="E27" s="22" t="s">
+      <c r="D27" s="12"/>
+      <c r="E27" s="20" t="s">
         <v>330</v>
       </c>
-      <c r="F27" s="27">
+      <c r="F27" s="25">
         <v>425000</v>
       </c>
-      <c r="G27" s="31" t="s">
+      <c r="G27" s="29" t="s">
         <v>331</v>
       </c>
-      <c r="H27" s="32">
+      <c r="H27" s="30">
         <v>697000</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="J27" s="46">
+      <c r="J27" s="44">
         <v>280000</v>
       </c>
       <c r="K27" s="2" t="s">
@@ -4918,27 +4297,27 @@
         <v>334</v>
       </c>
     </row>
-    <row r="28" ht="15.15" spans="3:30">
+    <row r="28" spans="3:30">
       <c r="C28" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="D28" s="14"/>
-      <c r="E28" s="22" t="s">
+      <c r="D28" s="12"/>
+      <c r="E28" s="20" t="s">
         <v>336</v>
       </c>
-      <c r="F28" s="27">
+      <c r="F28" s="25">
         <v>522000</v>
       </c>
-      <c r="G28" s="31" t="s">
+      <c r="G28" s="29" t="s">
         <v>337</v>
       </c>
-      <c r="H28" s="32">
+      <c r="H28" s="30">
         <v>494000</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="J28" s="47">
+      <c r="J28" s="45">
         <v>426000</v>
       </c>
       <c r="K28" s="2" t="s">
@@ -4952,26 +4331,26 @@
       </c>
     </row>
     <row r="29" spans="3:30">
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="11" t="s">
         <v>341</v>
       </c>
-      <c r="D29" s="14"/>
-      <c r="E29" s="31" t="s">
+      <c r="D29" s="12"/>
+      <c r="E29" s="29" t="s">
         <v>342</v>
       </c>
-      <c r="F29" s="32">
+      <c r="F29" s="30">
         <v>398000</v>
       </c>
-      <c r="G29" s="31" t="s">
+      <c r="G29" s="29" t="s">
         <v>343</v>
       </c>
-      <c r="H29" s="32">
+      <c r="H29" s="30">
         <v>173000</v>
       </c>
-      <c r="I29" s="22" t="s">
+      <c r="I29" s="20" t="s">
         <v>344</v>
       </c>
-      <c r="J29" s="48">
+      <c r="J29" s="46">
         <v>207000</v>
       </c>
       <c r="K29" s="2" t="s">
@@ -4988,23 +4367,23 @@
       <c r="C30" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="D30" s="14"/>
-      <c r="E30" s="31" t="s">
+      <c r="D30" s="12"/>
+      <c r="E30" s="29" t="s">
         <v>348</v>
       </c>
-      <c r="F30" s="32">
+      <c r="F30" s="30">
         <v>777000</v>
       </c>
-      <c r="G30" s="31" t="s">
+      <c r="G30" s="29" t="s">
         <v>349</v>
       </c>
-      <c r="H30" s="32">
+      <c r="H30" s="30">
         <v>207000</v>
       </c>
-      <c r="I30" s="22" t="s">
+      <c r="I30" s="20" t="s">
         <v>350</v>
       </c>
-      <c r="J30" s="48">
+      <c r="J30" s="46">
         <v>257000</v>
       </c>
       <c r="K30" s="2" t="s">
@@ -5021,23 +4400,23 @@
       <c r="C31" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="D31" s="14"/>
-      <c r="E31" s="49" t="s">
+      <c r="D31" s="12"/>
+      <c r="E31" s="47" t="s">
         <v>354</v>
       </c>
-      <c r="F31" s="50">
+      <c r="F31" s="48">
         <v>341000</v>
       </c>
-      <c r="G31" s="31" t="s">
+      <c r="G31" s="29" t="s">
         <v>355</v>
       </c>
-      <c r="H31" s="32">
+      <c r="H31" s="30">
         <v>302000</v>
       </c>
-      <c r="I31" s="51" t="s">
+      <c r="I31" s="49" t="s">
         <v>356</v>
       </c>
-      <c r="J31" s="52">
+      <c r="J31" s="50">
         <v>295000</v>
       </c>
       <c r="K31" s="2" t="s">
@@ -5054,23 +4433,23 @@
       <c r="C32" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="D32" s="14"/>
-      <c r="E32" s="49" t="s">
+      <c r="D32" s="12"/>
+      <c r="E32" s="47" t="s">
         <v>360</v>
       </c>
-      <c r="F32" s="50">
+      <c r="F32" s="48">
         <v>388000</v>
       </c>
-      <c r="G32" s="40" t="s">
+      <c r="G32" s="38" t="s">
         <v>361</v>
       </c>
-      <c r="H32" s="41">
+      <c r="H32" s="39">
         <v>381000</v>
       </c>
-      <c r="I32" s="51" t="s">
+      <c r="I32" s="49" t="s">
         <v>362</v>
       </c>
-      <c r="J32" s="52">
+      <c r="J32" s="50">
         <v>405000</v>
       </c>
       <c r="K32" s="2" t="s">
@@ -5083,27 +4462,27 @@
         <v>364</v>
       </c>
     </row>
-    <row r="33" ht="15.15" spans="3:13">
+    <row r="33" spans="3:13">
       <c r="C33" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="D33" s="53"/>
-      <c r="E33" s="31" t="s">
+      <c r="D33" s="51"/>
+      <c r="E33" s="29" t="s">
         <v>366</v>
       </c>
-      <c r="F33" s="32">
+      <c r="F33" s="30">
         <v>648000</v>
       </c>
-      <c r="G33" s="31" t="s">
+      <c r="G33" s="29" t="s">
         <v>367</v>
       </c>
-      <c r="H33" s="50">
+      <c r="H33" s="48">
         <v>388000</v>
       </c>
-      <c r="I33" s="31" t="s">
+      <c r="I33" s="29" t="s">
         <v>368</v>
       </c>
-      <c r="J33" s="54">
+      <c r="J33" s="52">
         <v>641000</v>
       </c>
       <c r="K33" s="2" t="s">
@@ -5117,25 +4496,25 @@
       </c>
     </row>
     <row r="34" spans="3:13">
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="11" t="s">
         <v>371</v>
       </c>
-      <c r="E34" s="31" t="s">
+      <c r="E34" s="29" t="s">
         <v>372</v>
       </c>
-      <c r="F34" s="32">
+      <c r="F34" s="30">
         <v>793000</v>
       </c>
-      <c r="G34" s="31" t="s">
+      <c r="G34" s="29" t="s">
         <v>373</v>
       </c>
-      <c r="H34" s="50">
+      <c r="H34" s="48">
         <v>413000</v>
       </c>
-      <c r="I34" s="31" t="s">
+      <c r="I34" s="29" t="s">
         <v>374</v>
       </c>
-      <c r="J34" s="55">
+      <c r="J34" s="53">
         <v>754000</v>
       </c>
       <c r="K34" s="2" t="s">
@@ -5152,22 +4531,22 @@
       <c r="C35" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="E35" s="31" t="s">
+      <c r="E35" s="29" t="s">
         <v>378</v>
       </c>
-      <c r="F35" s="56">
+      <c r="F35" s="54">
         <v>747000</v>
       </c>
-      <c r="G35" s="31" t="s">
+      <c r="G35" s="29" t="s">
         <v>379</v>
       </c>
-      <c r="H35" s="32">
+      <c r="H35" s="30">
         <v>309000</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="J35" s="57">
+      <c r="J35" s="55">
         <v>312000</v>
       </c>
       <c r="K35" s="2" t="s">
@@ -5184,22 +4563,22 @@
       <c r="C36" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="E36" s="31" t="s">
+      <c r="E36" s="29" t="s">
         <v>384</v>
       </c>
-      <c r="F36" s="56">
+      <c r="F36" s="54">
         <v>882000</v>
       </c>
-      <c r="G36" s="31" t="s">
+      <c r="G36" s="29" t="s">
         <v>385</v>
       </c>
-      <c r="H36" s="32">
+      <c r="H36" s="30">
         <v>411000</v>
       </c>
-      <c r="I36" s="17" t="s">
+      <c r="I36" s="15" t="s">
         <v>386</v>
       </c>
-      <c r="J36" s="57">
+      <c r="J36" s="55">
         <v>381000</v>
       </c>
       <c r="K36" s="2" t="s">
@@ -5213,25 +4592,25 @@
       </c>
     </row>
     <row r="37" spans="3:13">
-      <c r="C37" s="13" t="s">
+      <c r="C37" s="11" t="s">
         <v>389</v>
       </c>
-      <c r="E37" s="31" t="s">
+      <c r="E37" s="29" t="s">
         <v>390</v>
       </c>
-      <c r="F37" s="32">
+      <c r="F37" s="30">
         <v>356000</v>
       </c>
-      <c r="G37" s="31" t="s">
+      <c r="G37" s="29" t="s">
         <v>391</v>
       </c>
-      <c r="H37" s="32">
+      <c r="H37" s="30">
         <v>473000</v>
       </c>
-      <c r="I37" s="24" t="s">
+      <c r="I37" s="22" t="s">
         <v>392</v>
       </c>
-      <c r="J37" s="58">
+      <c r="J37" s="56">
         <v>365000</v>
       </c>
       <c r="K37" s="2" t="s">
@@ -5242,117 +4621,117 @@
       </c>
     </row>
     <row r="38" spans="3:13">
-      <c r="C38" s="13" t="s">
+      <c r="C38" s="11" t="s">
         <v>394</v>
       </c>
-      <c r="E38" s="31" t="s">
+      <c r="E38" s="29" t="s">
         <v>395</v>
       </c>
-      <c r="F38" s="32">
+      <c r="F38" s="30">
         <v>369000</v>
       </c>
-      <c r="G38" s="31" t="s">
+      <c r="G38" s="29" t="s">
         <v>396</v>
       </c>
-      <c r="H38" s="32">
+      <c r="H38" s="30">
         <v>329000</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="J38" s="59">
+      <c r="J38" s="57">
         <v>501000</v>
       </c>
     </row>
     <row r="39" spans="3:13">
-      <c r="C39" s="13" t="s">
+      <c r="C39" s="11" t="s">
         <v>398</v>
       </c>
-      <c r="E39" s="31" t="s">
+      <c r="E39" s="29" t="s">
         <v>399</v>
       </c>
-      <c r="F39" s="32">
+      <c r="F39" s="30">
         <v>465000</v>
       </c>
-      <c r="G39" s="31" t="s">
+      <c r="G39" s="29" t="s">
         <v>400</v>
       </c>
-      <c r="H39" s="32">
+      <c r="H39" s="30">
         <v>385000</v>
       </c>
-      <c r="I39" s="31" t="s">
+      <c r="I39" s="29" t="s">
         <v>401</v>
       </c>
-      <c r="J39" s="60">
+      <c r="J39" s="58">
         <v>740000</v>
       </c>
     </row>
     <row r="40" spans="3:13">
-      <c r="C40" s="13" t="s">
+      <c r="C40" s="11" t="s">
         <v>402</v>
       </c>
-      <c r="E40" s="31" t="s">
+      <c r="E40" s="29" t="s">
         <v>403</v>
       </c>
-      <c r="F40" s="32">
+      <c r="F40" s="30">
         <v>543000</v>
       </c>
-      <c r="G40" s="31" t="s">
+      <c r="G40" s="29" t="s">
         <v>404</v>
       </c>
-      <c r="H40" s="32">
+      <c r="H40" s="30">
         <v>437000</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="J40" s="61">
+      <c r="J40" s="59">
         <v>278000</v>
       </c>
     </row>
     <row r="41" spans="3:13">
-      <c r="C41" s="13" t="s">
+      <c r="C41" s="11" t="s">
         <v>406</v>
       </c>
-      <c r="E41" s="31" t="s">
+      <c r="E41" s="29" t="s">
         <v>407</v>
       </c>
-      <c r="F41" s="32">
+      <c r="F41" s="30">
         <v>778000</v>
       </c>
-      <c r="G41" s="31" t="s">
+      <c r="G41" s="29" t="s">
         <v>408</v>
       </c>
-      <c r="H41" s="32">
+      <c r="H41" s="30">
         <v>566000</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="J41" s="33">
+      <c r="J41" s="31">
         <v>351000</v>
       </c>
     </row>
     <row r="42" spans="3:13">
-      <c r="C42" s="13" t="s">
+      <c r="C42" s="11" t="s">
         <v>410</v>
       </c>
-      <c r="E42" s="31" t="s">
+      <c r="E42" s="29" t="s">
         <v>411</v>
       </c>
-      <c r="F42" s="32">
+      <c r="F42" s="30">
         <v>337000</v>
       </c>
-      <c r="G42" s="31" t="s">
+      <c r="G42" s="29" t="s">
         <v>412</v>
       </c>
-      <c r="H42" s="32">
+      <c r="H42" s="30">
         <v>636000</v>
       </c>
-      <c r="I42" s="22" t="s">
+      <c r="I42" s="20" t="s">
         <v>413</v>
       </c>
-      <c r="J42" s="62">
+      <c r="J42" s="60">
         <v>300000</v>
       </c>
     </row>
@@ -5360,22 +4739,22 @@
       <c r="C43" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E43" s="31" t="s">
+      <c r="E43" s="29" t="s">
         <v>415</v>
       </c>
-      <c r="F43" s="56">
+      <c r="F43" s="54">
         <v>440000</v>
       </c>
-      <c r="G43" s="31" t="s">
+      <c r="G43" s="29" t="s">
         <v>416</v>
       </c>
-      <c r="H43" s="32">
+      <c r="H43" s="30">
         <v>707000</v>
       </c>
-      <c r="I43" s="22" t="s">
+      <c r="I43" s="20" t="s">
         <v>417</v>
       </c>
-      <c r="J43" s="63">
+      <c r="J43" s="61">
         <v>322000</v>
       </c>
     </row>
@@ -5389,16 +4768,16 @@
       <c r="F44" s="3">
         <v>335000</v>
       </c>
-      <c r="G44" s="31" t="s">
+      <c r="G44" s="29" t="s">
         <v>420</v>
       </c>
-      <c r="H44" s="32">
+      <c r="H44" s="30">
         <v>420000</v>
       </c>
-      <c r="I44" s="64" t="s">
+      <c r="I44" s="62" t="s">
         <v>421</v>
       </c>
-      <c r="J44" s="65">
+      <c r="J44" s="63">
         <v>329000</v>
       </c>
     </row>
@@ -5412,16 +4791,16 @@
       <c r="F45" s="3">
         <v>448000</v>
       </c>
-      <c r="G45" s="31" t="s">
+      <c r="G45" s="29" t="s">
         <v>424</v>
       </c>
-      <c r="H45" s="32">
+      <c r="H45" s="30">
         <v>430000</v>
       </c>
-      <c r="I45" s="64" t="s">
+      <c r="I45" s="62" t="s">
         <v>425</v>
       </c>
-      <c r="J45" s="65">
+      <c r="J45" s="63">
         <v>445000</v>
       </c>
     </row>
@@ -5435,14 +4814,14 @@
       <c r="F46" s="3">
         <v>402000</v>
       </c>
-      <c r="G46" s="31" t="s">
+      <c r="G46" s="29" t="s">
         <v>428</v>
       </c>
-      <c r="H46" s="32">
+      <c r="H46" s="30">
         <v>400000</v>
       </c>
-      <c r="I46" s="64"/>
-      <c r="J46" s="65"/>
+      <c r="I46" s="62"/>
+      <c r="J46" s="63"/>
     </row>
     <row r="47" spans="3:13">
       <c r="C47" s="2" t="s">
@@ -5454,15 +4833,15 @@
       <c r="F47" s="3">
         <v>469000</v>
       </c>
-      <c r="G47" s="31" t="s">
+      <c r="G47" s="29" t="s">
         <v>431</v>
       </c>
-      <c r="H47" s="32">
+      <c r="H47" s="30">
         <v>382000</v>
       </c>
     </row>
     <row r="48" spans="3:13">
-      <c r="C48" s="13" t="s">
+      <c r="C48" s="11" t="s">
         <v>432</v>
       </c>
       <c r="E48" s="2" t="s">
@@ -5479,10 +4858,10 @@
       </c>
     </row>
     <row r="49" spans="5:8">
-      <c r="E49" s="22" t="s">
+      <c r="E49" s="20" t="s">
         <v>435</v>
       </c>
-      <c r="F49" s="27">
+      <c r="F49" s="25">
         <v>180000</v>
       </c>
       <c r="G49" s="2" t="s">
@@ -5493,10 +4872,10 @@
       </c>
     </row>
     <row r="50" spans="5:8">
-      <c r="E50" s="22" t="s">
+      <c r="E50" s="20" t="s">
         <v>437</v>
       </c>
-      <c r="F50" s="27">
+      <c r="F50" s="25">
         <v>230000</v>
       </c>
       <c r="G50" s="2" t="s">
@@ -5513,10 +4892,10 @@
       <c r="F51" s="3">
         <v>46000</v>
       </c>
-      <c r="G51" s="31" t="s">
+      <c r="G51" s="29" t="s">
         <v>440</v>
       </c>
-      <c r="H51" s="32">
+      <c r="H51" s="30">
         <v>446000</v>
       </c>
     </row>
@@ -5611,10 +4990,10 @@
       <c r="F58" s="3">
         <v>358000</v>
       </c>
-      <c r="G58" s="31" t="s">
+      <c r="G58" s="29" t="s">
         <v>454</v>
       </c>
-      <c r="H58" s="32">
+      <c r="H58" s="30">
         <v>541000</v>
       </c>
     </row>
@@ -5625,42 +5004,42 @@
       <c r="F59" s="3">
         <v>320000</v>
       </c>
-      <c r="G59" s="49" t="s">
+      <c r="G59" s="47" t="s">
         <v>456</v>
       </c>
-      <c r="H59" s="50">
+      <c r="H59" s="48">
         <v>515000</v>
       </c>
     </row>
     <row r="60" spans="5:8">
-      <c r="G60" s="66" t="s">
+      <c r="G60" s="64" t="s">
         <v>457</v>
       </c>
-      <c r="H60" s="67">
+      <c r="H60" s="65">
         <v>701000</v>
       </c>
     </row>
     <row r="61" spans="5:8">
-      <c r="G61" s="66" t="s">
+      <c r="G61" s="64" t="s">
         <v>458</v>
       </c>
-      <c r="H61" s="67">
+      <c r="H61" s="65">
         <v>794000</v>
       </c>
     </row>
     <row r="62" spans="5:8">
-      <c r="G62" s="40" t="s">
+      <c r="G62" s="38" t="s">
         <v>459</v>
       </c>
-      <c r="H62" s="41">
+      <c r="H62" s="39">
         <v>628000</v>
       </c>
     </row>
     <row r="63" spans="5:8">
-      <c r="G63" s="40" t="s">
+      <c r="G63" s="38" t="s">
         <v>460</v>
       </c>
-      <c r="H63" s="41">
+      <c r="H63" s="39">
         <v>747000</v>
       </c>
     </row>
@@ -5716,7 +5095,7 @@
       <c r="G70" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="H70" s="20">
+      <c r="H70" s="18">
         <v>903000</v>
       </c>
     </row>
@@ -5729,290 +5108,290 @@
       </c>
     </row>
     <row r="72" spans="7:8">
-      <c r="G72" s="51" t="s">
+      <c r="G72" s="49" t="s">
         <v>469</v>
       </c>
-      <c r="H72" s="68">
+      <c r="H72" s="66">
         <v>268000</v>
       </c>
     </row>
     <row r="73" spans="7:8">
-      <c r="G73" s="51" t="s">
+      <c r="G73" s="49" t="s">
         <v>470</v>
       </c>
-      <c r="H73" s="68">
+      <c r="H73" s="66">
         <v>325000</v>
       </c>
     </row>
     <row r="74" spans="7:8">
-      <c r="G74" s="69" t="s">
+      <c r="G74" s="67" t="s">
         <v>471</v>
       </c>
-      <c r="H74" s="68">
+      <c r="H74" s="66">
         <v>297000</v>
       </c>
     </row>
     <row r="75" spans="7:8">
-      <c r="G75" s="69" t="s">
+      <c r="G75" s="67" t="s">
         <v>472</v>
       </c>
-      <c r="H75" s="68">
+      <c r="H75" s="66">
         <v>359000</v>
       </c>
     </row>
     <row r="76" spans="7:8">
-      <c r="G76" s="31" t="s">
+      <c r="G76" s="29" t="s">
         <v>473</v>
       </c>
-      <c r="H76" s="32">
+      <c r="H76" s="30">
         <v>297000</v>
       </c>
     </row>
     <row r="77" spans="7:8">
-      <c r="G77" s="31" t="s">
+      <c r="G77" s="29" t="s">
         <v>474</v>
       </c>
-      <c r="H77" s="32">
+      <c r="H77" s="30">
         <v>394000</v>
       </c>
     </row>
     <row r="78" spans="7:8">
-      <c r="G78" s="70" t="s">
+      <c r="G78" s="68" t="s">
         <v>475</v>
       </c>
-      <c r="H78" s="20">
+      <c r="H78" s="18">
         <v>446000</v>
       </c>
     </row>
     <row r="79" spans="7:8">
-      <c r="G79" s="40" t="s">
+      <c r="G79" s="38" t="s">
         <v>476</v>
       </c>
-      <c r="H79" s="41">
+      <c r="H79" s="39">
         <v>337000</v>
       </c>
     </row>
     <row r="80" spans="7:8">
-      <c r="G80" s="40" t="s">
+      <c r="G80" s="38" t="s">
         <v>477</v>
       </c>
-      <c r="H80" s="41">
+      <c r="H80" s="39">
         <v>358000</v>
       </c>
     </row>
     <row r="81" spans="7:8">
-      <c r="G81" s="40" t="s">
+      <c r="G81" s="38" t="s">
         <v>478</v>
       </c>
-      <c r="H81" s="41">
+      <c r="H81" s="39">
         <v>435000</v>
       </c>
     </row>
     <row r="82" spans="7:8">
-      <c r="G82" s="40" t="s">
+      <c r="G82" s="38" t="s">
         <v>479</v>
       </c>
-      <c r="H82" s="41">
+      <c r="H82" s="39">
         <v>497000</v>
       </c>
     </row>
     <row r="83" spans="7:8">
-      <c r="G83" s="49" t="s">
+      <c r="G83" s="47" t="s">
         <v>480</v>
       </c>
-      <c r="H83" s="50">
+      <c r="H83" s="48">
         <v>433000</v>
       </c>
     </row>
     <row r="84" spans="7:8">
-      <c r="G84" s="49" t="s">
+      <c r="G84" s="47" t="s">
         <v>481</v>
       </c>
-      <c r="H84" s="50">
+      <c r="H84" s="48">
         <v>610000</v>
       </c>
     </row>
     <row r="85" spans="7:8">
-      <c r="G85" s="49" t="s">
+      <c r="G85" s="47" t="s">
         <v>482</v>
       </c>
-      <c r="H85" s="50">
+      <c r="H85" s="48">
         <v>145000</v>
       </c>
     </row>
     <row r="86" spans="7:8">
-      <c r="G86" s="49" t="s">
+      <c r="G86" s="47" t="s">
         <v>483</v>
       </c>
-      <c r="H86" s="50">
+      <c r="H86" s="48">
         <v>178000</v>
       </c>
     </row>
     <row r="87" spans="7:8">
-      <c r="G87" s="49" t="s">
+      <c r="G87" s="47" t="s">
         <v>484</v>
       </c>
-      <c r="H87" s="50">
+      <c r="H87" s="48">
         <v>259000</v>
       </c>
     </row>
     <row r="88" spans="7:8">
-      <c r="G88" s="49" t="s">
+      <c r="G88" s="47" t="s">
         <v>485</v>
       </c>
-      <c r="H88" s="50">
+      <c r="H88" s="48">
         <v>176000</v>
       </c>
     </row>
     <row r="89" spans="7:8">
-      <c r="G89" s="49" t="s">
+      <c r="G89" s="47" t="s">
         <v>486</v>
       </c>
-      <c r="H89" s="50">
+      <c r="H89" s="48">
         <v>180000</v>
       </c>
     </row>
     <row r="90" spans="7:8">
-      <c r="G90" s="49" t="s">
+      <c r="G90" s="47" t="s">
         <v>487</v>
       </c>
-      <c r="H90" s="50">
+      <c r="H90" s="48">
         <v>240000</v>
       </c>
     </row>
     <row r="91" spans="7:8">
-      <c r="G91" s="49" t="s">
+      <c r="G91" s="47" t="s">
         <v>488</v>
       </c>
-      <c r="H91" s="50">
+      <c r="H91" s="48">
         <v>288000</v>
       </c>
     </row>
     <row r="92" spans="7:8">
-      <c r="G92" s="49" t="s">
+      <c r="G92" s="47" t="s">
         <v>489</v>
       </c>
-      <c r="H92" s="50">
+      <c r="H92" s="48">
         <v>568000</v>
       </c>
     </row>
     <row r="93" spans="7:8">
-      <c r="G93" s="49" t="s">
+      <c r="G93" s="47" t="s">
         <v>490</v>
       </c>
-      <c r="H93" s="50">
+      <c r="H93" s="48">
         <v>579000</v>
       </c>
     </row>
     <row r="94" spans="7:8">
-      <c r="G94" s="49" t="s">
+      <c r="G94" s="47" t="s">
         <v>491</v>
       </c>
-      <c r="H94" s="50">
+      <c r="H94" s="48">
         <v>473000</v>
       </c>
     </row>
     <row r="95" spans="7:8">
-      <c r="G95" s="71" t="s">
+      <c r="G95" s="69" t="s">
         <v>492</v>
       </c>
-      <c r="H95" s="72">
+      <c r="H95" s="70">
         <v>43000</v>
       </c>
     </row>
     <row r="96" spans="7:8">
-      <c r="G96" s="71" t="s">
+      <c r="G96" s="69" t="s">
         <v>493</v>
       </c>
-      <c r="H96" s="72">
+      <c r="H96" s="70">
         <v>48000</v>
       </c>
     </row>
     <row r="97" spans="2:8">
-      <c r="G97" s="73" t="s">
+      <c r="G97" s="71" t="s">
         <v>494</v>
       </c>
-      <c r="H97" s="74">
+      <c r="H97" s="72">
         <v>47000</v>
       </c>
     </row>
     <row r="98" spans="2:8">
-      <c r="G98" s="71" t="s">
+      <c r="G98" s="69" t="s">
         <v>495</v>
       </c>
-      <c r="H98" s="72">
+      <c r="H98" s="70">
         <v>53000</v>
       </c>
     </row>
     <row r="99" spans="2:8">
-      <c r="G99" s="71" t="s">
+      <c r="G99" s="69" t="s">
         <v>496</v>
       </c>
-      <c r="H99" s="72">
+      <c r="H99" s="70">
         <v>54000</v>
       </c>
     </row>
     <row r="100" spans="2:8">
-      <c r="G100" s="71" t="s">
+      <c r="G100" s="69" t="s">
         <v>497</v>
       </c>
-      <c r="H100" s="72">
+      <c r="H100" s="70">
         <v>56000</v>
       </c>
     </row>
     <row r="101" spans="2:8">
-      <c r="G101" s="71" t="s">
+      <c r="G101" s="69" t="s">
         <v>498</v>
       </c>
-      <c r="H101" s="72">
+      <c r="H101" s="70">
         <v>54000</v>
       </c>
     </row>
     <row r="102" spans="2:8">
-      <c r="G102" s="40" t="s">
+      <c r="G102" s="38" t="s">
         <v>499</v>
       </c>
-      <c r="H102" s="41">
+      <c r="H102" s="39">
         <v>250000</v>
       </c>
     </row>
     <row r="103" spans="2:8">
-      <c r="G103" s="40" t="s">
+      <c r="G103" s="38" t="s">
         <v>500</v>
       </c>
-      <c r="H103" s="41">
+      <c r="H103" s="39">
         <v>303000</v>
       </c>
     </row>
     <row r="104" spans="2:8">
-      <c r="G104" s="40" t="s">
+      <c r="G104" s="38" t="s">
         <v>501</v>
       </c>
-      <c r="H104" s="41">
+      <c r="H104" s="39">
         <v>330000</v>
       </c>
     </row>
     <row r="105" spans="2:8">
-      <c r="G105" s="40" t="s">
+      <c r="G105" s="38" t="s">
         <v>502</v>
       </c>
-      <c r="H105" s="41">
+      <c r="H105" s="39">
         <v>387000</v>
       </c>
     </row>
     <row r="106" spans="2:8">
-      <c r="G106" s="40" t="s">
+      <c r="G106" s="38" t="s">
         <v>503</v>
       </c>
-      <c r="H106" s="41">
+      <c r="H106" s="39">
         <v>578000</v>
       </c>
     </row>
     <row r="107" spans="2:8">
-      <c r="G107" s="40" t="s">
+      <c r="G107" s="38" t="s">
         <v>504</v>
       </c>
-      <c r="H107" s="41">
+      <c r="H107" s="39">
         <v>722000</v>
       </c>
     </row>
@@ -6027,6 +5406,5 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update BangGia.xlsx with new data
</commit_message>
<xml_diff>
--- a/app/data/BangGia.xlsx
+++ b/app/data/BangGia.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\mtms\app\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C88767-CE16-47B3-847D-91B229B88CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="23040" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="Tổng Quát" sheetId="1" r:id="rId1"/>
@@ -32,6 +26,19 @@
     <definedName name="YOKO_NAME">'Tổng Quát'!$I$2:$I$1048576</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1556,12 +1563,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="5">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="37">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1681,10 +1691,147 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1693,7 +1840,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1732,12 +1879,198 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39994506668294322"/>
+        <fgColor theme="7" tint="0.399945066682943"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -1974,11 +2307,250 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1986,25 +2558,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="177" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="177" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -2012,95 +2590,95 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="11" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="11" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="11" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="11" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="11" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="13" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="13" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="177" fontId="1" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="1" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="177" fontId="1" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="3" fillId="4" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="3" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="3" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="3" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="15" fillId="3" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="3" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="15" fillId="3" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="15" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2112,26 +2690,63 @@
     <xf numFmtId="3" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="50">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal 2" xfId="49"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -2389,50 +3004,49 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AD110"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.11111111111111" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="14.88671875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="34.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="25.33203125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="31.5546875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="14.8888888888889" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.6666666666667" style="3" customWidth="1"/>
+    <col min="3" max="3" width="22.6666666666667" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.6666666666667" style="4" customWidth="1"/>
+    <col min="5" max="5" width="34.6666666666667" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.6666666666667" style="3" customWidth="1"/>
+    <col min="7" max="7" width="25.3333333333333" style="2" customWidth="1"/>
+    <col min="8" max="8" width="10.6666666666667" style="3" customWidth="1"/>
+    <col min="9" max="9" width="31.5555555555556" style="2" customWidth="1"/>
     <col min="10" max="10" width="13" style="5" customWidth="1"/>
-    <col min="11" max="11" width="28.109375" style="2" customWidth="1"/>
-    <col min="12" max="12" width="10.6640625" style="3" customWidth="1"/>
-    <col min="13" max="13" width="29.5546875" style="2" customWidth="1"/>
-    <col min="14" max="14" width="10.6640625" style="3" customWidth="1"/>
-    <col min="15" max="15" width="17.33203125" style="2" customWidth="1"/>
-    <col min="16" max="16" width="10.6640625" style="3" customWidth="1"/>
-    <col min="17" max="17" width="19.6640625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="10.6640625" style="3" customWidth="1"/>
-    <col min="19" max="19" width="28.33203125" style="2" customWidth="1"/>
-    <col min="20" max="20" width="10.6640625" style="3" customWidth="1"/>
-    <col min="21" max="21" width="20.5546875" style="2" customWidth="1"/>
-    <col min="22" max="22" width="10.6640625" style="3" customWidth="1"/>
-    <col min="23" max="23" width="21.5546875" style="2" customWidth="1"/>
-    <col min="24" max="24" width="10.6640625" style="3" customWidth="1"/>
-    <col min="25" max="25" width="26.6640625" style="2" customWidth="1"/>
-    <col min="26" max="26" width="10.6640625" style="3" customWidth="1"/>
-    <col min="27" max="27" width="33.44140625" style="2" customWidth="1"/>
-    <col min="28" max="28" width="22.5546875" style="3" customWidth="1"/>
-    <col min="29" max="29" width="19.44140625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="28.1111111111111" style="2" customWidth="1"/>
+    <col min="12" max="12" width="10.6666666666667" style="3" customWidth="1"/>
+    <col min="13" max="13" width="29.5555555555556" style="2" customWidth="1"/>
+    <col min="14" max="14" width="10.6666666666667" style="3" customWidth="1"/>
+    <col min="15" max="15" width="17.3333333333333" style="2" customWidth="1"/>
+    <col min="16" max="16" width="10.6666666666667" style="3" customWidth="1"/>
+    <col min="17" max="17" width="19.6666666666667" style="2" customWidth="1"/>
+    <col min="18" max="18" width="10.6666666666667" style="3" customWidth="1"/>
+    <col min="19" max="19" width="28.3333333333333" style="2" customWidth="1"/>
+    <col min="20" max="20" width="10.6666666666667" style="3" customWidth="1"/>
+    <col min="21" max="21" width="20.5555555555556" style="2" customWidth="1"/>
+    <col min="22" max="22" width="10.6666666666667" style="3" customWidth="1"/>
+    <col min="23" max="23" width="21.5555555555556" style="2" customWidth="1"/>
+    <col min="24" max="24" width="10.6666666666667" style="3" customWidth="1"/>
+    <col min="25" max="25" width="26.6666666666667" style="2" customWidth="1"/>
+    <col min="26" max="26" width="10.6666666666667" style="3" customWidth="1"/>
+    <col min="27" max="27" width="33.4444444444444" style="2" customWidth="1"/>
+    <col min="28" max="28" width="22.5555555555556" style="3" customWidth="1"/>
+    <col min="29" max="29" width="19.4444444444444" style="2" customWidth="1"/>
     <col min="30" max="30" width="18" style="2" customWidth="1"/>
-    <col min="31" max="16384" width="9.109375" style="2"/>
+    <col min="31" max="16384" width="9.11111111111111" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1">
+    <row r="1" s="1" customFormat="1" ht="15.15" spans="1:30">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -2489,22 +3103,22 @@
         <v>13</v>
       </c>
       <c r="AB1" s="9"/>
-      <c r="AC1" s="73" t="s">
+      <c r="AC1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="AD1" s="74"/>
+      <c r="AD1" s="12"/>
     </row>
     <row r="2" spans="1:30">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="13" t="s">
         <v>15</v>
       </c>
       <c r="B2" s="3">
         <v>239000</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="12"/>
+      <c r="D2" s="14"/>
       <c r="E2" s="2" t="s">
         <v>17</v>
       </c>
@@ -2520,7 +3134,7 @@
       <c r="I2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="13">
+      <c r="J2" s="15">
         <v>152000</v>
       </c>
       <c r="K2" s="2" t="s">
@@ -2578,17 +3192,17 @@
         <v>319000</v>
       </c>
     </row>
-    <row r="3" spans="1:30">
-      <c r="A3" s="11" t="s">
+    <row r="3" ht="15.15" spans="1:30">
+      <c r="A3" s="13" t="s">
         <v>30</v>
       </c>
       <c r="B3" s="3">
         <v>252000</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="12"/>
+      <c r="D3" s="14"/>
       <c r="E3" s="2" t="s">
         <v>32</v>
       </c>
@@ -2604,7 +3218,7 @@
       <c r="I3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J3" s="14">
+      <c r="J3" s="16">
         <v>204000</v>
       </c>
       <c r="K3" s="2" t="s">
@@ -2663,16 +3277,16 @@
       </c>
     </row>
     <row r="4" spans="1:30">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="13" t="s">
         <v>45</v>
       </c>
       <c r="B4" s="3">
         <v>280000</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="12"/>
+      <c r="D4" s="14"/>
       <c r="E4" s="2" t="s">
         <v>47</v>
       </c>
@@ -2685,10 +3299,10 @@
       <c r="H4" s="3">
         <v>192000</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="I4" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="J4" s="16">
+      <c r="J4" s="18">
         <v>151000</v>
       </c>
       <c r="K4" s="2" t="s">
@@ -2747,16 +3361,16 @@
       </c>
     </row>
     <row r="5" spans="1:30">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="13" t="s">
         <v>60</v>
       </c>
       <c r="B5" s="3">
         <v>221000</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="12"/>
+      <c r="D5" s="14"/>
       <c r="E5" s="2" t="s">
         <v>62</v>
       </c>
@@ -2769,10 +3383,10 @@
       <c r="H5" s="3">
         <v>192000</v>
       </c>
-      <c r="I5" s="15" t="s">
+      <c r="I5" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="J5" s="17">
+      <c r="J5" s="19">
         <v>192000</v>
       </c>
       <c r="K5" s="2" t="s">
@@ -2809,7 +3423,7 @@
         <v>71</v>
       </c>
       <c r="X5" s="3">
-        <v>66000</v>
+        <v>81000</v>
       </c>
       <c r="Y5" s="2" t="s">
         <v>72</v>
@@ -2831,16 +3445,16 @@
       </c>
     </row>
     <row r="6" spans="1:30">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="13" t="s">
         <v>75</v>
       </c>
       <c r="B6" s="3">
         <v>249000</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="D6" s="12"/>
+      <c r="D6" s="14"/>
       <c r="E6" s="2" t="s">
         <v>77</v>
       </c>
@@ -2856,7 +3470,7 @@
       <c r="I6" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="J6" s="13">
+      <c r="J6" s="15">
         <v>177000</v>
       </c>
       <c r="K6" s="2" t="s">
@@ -2893,7 +3507,7 @@
         <v>86</v>
       </c>
       <c r="X6" s="3">
-        <v>82000</v>
+        <v>102000</v>
       </c>
       <c r="Y6" s="2" t="s">
         <v>87</v>
@@ -2915,16 +3529,16 @@
       </c>
     </row>
     <row r="7" spans="1:30">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="13" t="s">
         <v>90</v>
       </c>
       <c r="B7" s="3">
         <v>382000</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="14"/>
       <c r="E7" s="2" t="s">
         <v>92</v>
       </c>
@@ -2940,7 +3554,7 @@
       <c r="I7" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="J7" s="14">
+      <c r="J7" s="16">
         <v>228000</v>
       </c>
       <c r="K7" s="2" t="s">
@@ -2977,7 +3591,7 @@
         <v>101</v>
       </c>
       <c r="X7" s="3">
-        <v>77000</v>
+        <v>96000</v>
       </c>
       <c r="Y7" s="2" t="s">
         <v>102</v>
@@ -2999,16 +3613,16 @@
       </c>
     </row>
     <row r="8" spans="1:30">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="13" t="s">
         <v>105</v>
       </c>
       <c r="B8" s="3">
         <v>412000</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="12"/>
+      <c r="D8" s="14"/>
       <c r="E8" s="2" t="s">
         <v>107</v>
       </c>
@@ -3018,13 +3632,13 @@
       <c r="G8" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="H8" s="18">
+      <c r="H8" s="20">
         <v>286000</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J8" s="13">
+      <c r="J8" s="15">
         <v>212000</v>
       </c>
       <c r="K8" s="2" t="s">
@@ -3082,17 +3696,17 @@
         <v>269000</v>
       </c>
     </row>
-    <row r="9" spans="1:30">
-      <c r="A9" s="11" t="s">
+    <row r="9" ht="15.15" spans="1:30">
+      <c r="A9" s="13" t="s">
         <v>120</v>
       </c>
       <c r="B9" s="3">
         <v>347000</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="D9" s="12"/>
+      <c r="D9" s="14"/>
       <c r="E9" s="2" t="s">
         <v>122</v>
       </c>
@@ -3108,7 +3722,7 @@
       <c r="I9" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="J9" s="14">
+      <c r="J9" s="16">
         <v>287000</v>
       </c>
       <c r="K9" s="2" t="s">
@@ -3132,7 +3746,7 @@
       <c r="S9" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="T9" s="19">
+      <c r="T9" s="21">
         <v>260000</v>
       </c>
       <c r="U9" s="2" t="s">
@@ -3167,32 +3781,32 @@
       </c>
     </row>
     <row r="10" spans="1:30">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="13" t="s">
         <v>135</v>
       </c>
       <c r="B10" s="3">
         <v>221000</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="D10" s="12"/>
+      <c r="D10" s="14"/>
       <c r="E10" s="2" t="s">
         <v>137</v>
       </c>
       <c r="F10" s="3">
         <v>282000</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="H10" s="21">
+      <c r="H10" s="23">
         <v>348000</v>
       </c>
-      <c r="I10" s="22" t="s">
+      <c r="I10" s="24" t="s">
         <v>139</v>
       </c>
-      <c r="J10" s="23">
+      <c r="J10" s="25">
         <v>218000</v>
       </c>
       <c r="K10" s="2" t="s">
@@ -3250,33 +3864,33 @@
         <v>290000</v>
       </c>
     </row>
-    <row r="11" spans="1:30">
+    <row r="11" ht="15.15" spans="1:30">
       <c r="A11" s="2" t="s">
         <v>150</v>
       </c>
       <c r="B11" s="3">
         <v>332000</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11" s="14"/>
       <c r="E11" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F11" s="3">
         <v>235000</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="G11" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="H11" s="21">
+      <c r="H11" s="23">
         <v>370000</v>
       </c>
-      <c r="I11" s="22" t="s">
+      <c r="I11" s="24" t="s">
         <v>154</v>
       </c>
-      <c r="J11" s="24">
+      <c r="J11" s="26">
         <v>270000</v>
       </c>
       <c r="K11" s="2" t="s">
@@ -3341,26 +3955,26 @@
       <c r="B12" s="3">
         <v>800000</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="D12" s="12"/>
+      <c r="D12" s="14"/>
       <c r="E12" s="2" t="s">
         <v>167</v>
       </c>
       <c r="F12" s="3">
         <v>289000</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="27">
         <v>348000</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="I12" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="J12" s="26">
+      <c r="J12" s="28">
         <v>395000</v>
       </c>
       <c r="K12" s="2" t="s">
@@ -3419,29 +4033,29 @@
       </c>
     </row>
     <row r="13" spans="1:30">
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="29" t="s">
         <v>180</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="D13" s="12"/>
-      <c r="E13" s="22" t="s">
+      <c r="D13" s="14"/>
+      <c r="E13" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="F13" s="19">
+      <c r="F13" s="21">
         <v>254000</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="G13" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="H13" s="25">
+      <c r="H13" s="27">
         <v>370000</v>
       </c>
-      <c r="I13" s="15" t="s">
+      <c r="I13" s="17" t="s">
         <v>184</v>
       </c>
-      <c r="J13" s="28">
+      <c r="J13" s="30">
         <v>431000</v>
       </c>
       <c r="K13" s="2" t="s">
@@ -3499,27 +4113,27 @@
         <v>32000</v>
       </c>
     </row>
-    <row r="14" spans="1:30">
-      <c r="C14" s="11" t="s">
+    <row r="14" ht="15.15" spans="1:30">
+      <c r="C14" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="D14" s="12"/>
-      <c r="E14" s="22" t="s">
+      <c r="D14" s="14"/>
+      <c r="E14" s="24" t="s">
         <v>195</v>
       </c>
-      <c r="F14" s="19">
+      <c r="F14" s="21">
         <v>291000</v>
       </c>
-      <c r="G14" s="29" t="s">
+      <c r="G14" s="31" t="s">
         <v>196</v>
       </c>
-      <c r="H14" s="30">
+      <c r="H14" s="32">
         <v>281000</v>
       </c>
-      <c r="I14" s="15" t="s">
+      <c r="I14" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="J14" s="17">
+      <c r="J14" s="19">
         <v>286000</v>
       </c>
       <c r="K14" s="2" t="s">
@@ -3578,26 +4192,26 @@
       </c>
     </row>
     <row r="15" spans="1:30">
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="D15" s="12"/>
+      <c r="D15" s="14"/>
       <c r="E15" s="3" t="s">
         <v>209</v>
       </c>
       <c r="F15" s="3">
         <v>214000</v>
       </c>
-      <c r="G15" s="29" t="s">
+      <c r="G15" s="31" t="s">
         <v>210</v>
       </c>
-      <c r="H15" s="30">
+      <c r="H15" s="32">
         <v>358000</v>
       </c>
-      <c r="I15" s="15" t="s">
+      <c r="I15" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="J15" s="16">
+      <c r="J15" s="18">
         <v>334000</v>
       </c>
       <c r="K15" s="2" t="s">
@@ -3646,27 +4260,27 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="16" spans="1:30">
-      <c r="C16" s="11" t="s">
+    <row r="16" ht="15.15" spans="1:30">
+      <c r="C16" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="D16" s="12"/>
+      <c r="D16" s="14"/>
       <c r="E16" s="2" t="s">
         <v>221</v>
       </c>
       <c r="F16" s="3">
         <v>266000</v>
       </c>
-      <c r="G16" s="29" t="s">
+      <c r="G16" s="31" t="s">
         <v>222</v>
       </c>
-      <c r="H16" s="30">
+      <c r="H16" s="32">
         <v>442000</v>
       </c>
-      <c r="I16" s="15" t="s">
+      <c r="I16" s="17" t="s">
         <v>223</v>
       </c>
-      <c r="J16" s="17">
+      <c r="J16" s="19">
         <v>269000</v>
       </c>
       <c r="K16" s="2" t="s">
@@ -3716,26 +4330,26 @@
       </c>
     </row>
     <row r="17" spans="3:30">
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="D17" s="12"/>
+      <c r="D17" s="14"/>
       <c r="E17" s="2" t="s">
         <v>233</v>
       </c>
       <c r="F17" s="3">
         <v>235000</v>
       </c>
-      <c r="G17" s="29" t="s">
+      <c r="G17" s="31" t="s">
         <v>234</v>
       </c>
-      <c r="H17" s="30">
+      <c r="H17" s="32">
         <v>374000</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="J17" s="13">
+      <c r="J17" s="15">
         <v>312000</v>
       </c>
       <c r="K17" s="2" t="s">
@@ -3785,26 +4399,26 @@
       </c>
     </row>
     <row r="18" spans="3:30">
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="13" t="s">
         <v>244</v>
       </c>
-      <c r="D18" s="12"/>
+      <c r="D18" s="14"/>
       <c r="E18" s="2" t="s">
         <v>245</v>
       </c>
       <c r="F18" s="3">
         <v>293000</v>
       </c>
-      <c r="G18" s="29" t="s">
+      <c r="G18" s="31" t="s">
         <v>246</v>
       </c>
-      <c r="H18" s="30">
+      <c r="H18" s="32">
         <v>374000</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="J18" s="31">
+      <c r="J18" s="33">
         <v>375000</v>
       </c>
       <c r="K18" s="2" t="s">
@@ -3853,27 +4467,27 @@
         <v>1120000</v>
       </c>
     </row>
-    <row r="19" spans="3:30">
-      <c r="C19" s="11" t="s">
+    <row r="19" ht="15.15" spans="3:30">
+      <c r="C19" s="13" t="s">
         <v>256</v>
       </c>
-      <c r="D19" s="12"/>
+      <c r="D19" s="14"/>
       <c r="E19" s="2" t="s">
         <v>257</v>
       </c>
       <c r="F19" s="3">
         <v>267000</v>
       </c>
-      <c r="G19" s="29" t="s">
+      <c r="G19" s="31" t="s">
         <v>258</v>
       </c>
-      <c r="H19" s="30">
+      <c r="H19" s="32">
         <v>298000</v>
       </c>
-      <c r="I19" s="22" t="s">
+      <c r="I19" s="24" t="s">
         <v>259</v>
       </c>
-      <c r="J19" s="24">
+      <c r="J19" s="26">
         <v>317000</v>
       </c>
       <c r="K19" s="2" t="s">
@@ -3923,26 +4537,26 @@
       </c>
     </row>
     <row r="20" spans="3:30">
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="13" t="s">
         <v>268</v>
       </c>
-      <c r="D20" s="12"/>
+      <c r="D20" s="14"/>
       <c r="E20" s="2" t="s">
         <v>269</v>
       </c>
       <c r="F20" s="3">
         <v>340000</v>
       </c>
-      <c r="G20" s="29" t="s">
+      <c r="G20" s="31" t="s">
         <v>270</v>
       </c>
-      <c r="H20" s="30">
+      <c r="H20" s="32">
         <v>366000</v>
       </c>
-      <c r="I20" s="32" t="s">
+      <c r="I20" s="34" t="s">
         <v>271</v>
       </c>
-      <c r="J20" s="33">
+      <c r="J20" s="35">
         <v>417000</v>
       </c>
       <c r="K20" s="2" t="s">
@@ -3963,7 +4577,7 @@
       <c r="S20" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="T20" s="19">
+      <c r="T20" s="21">
         <v>431000</v>
       </c>
       <c r="U20" s="2" t="s">
@@ -3995,26 +4609,26 @@
       </c>
     </row>
     <row r="21" spans="3:30">
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="13" t="s">
         <v>280</v>
       </c>
-      <c r="D21" s="12"/>
+      <c r="D21" s="14"/>
       <c r="E21" s="2" t="s">
         <v>281</v>
       </c>
       <c r="F21" s="3">
         <v>411000</v>
       </c>
-      <c r="G21" s="29" t="s">
+      <c r="G21" s="31" t="s">
         <v>282</v>
       </c>
-      <c r="H21" s="30">
+      <c r="H21" s="32">
         <v>330000</v>
       </c>
-      <c r="I21" s="32" t="s">
+      <c r="I21" s="34" t="s">
         <v>283</v>
       </c>
-      <c r="J21" s="34">
+      <c r="J21" s="36">
         <v>373000</v>
       </c>
       <c r="K21" s="2" t="s">
@@ -4046,26 +4660,26 @@
       </c>
     </row>
     <row r="22" spans="3:30">
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="13" t="s">
         <v>289</v>
       </c>
-      <c r="D22" s="12"/>
+      <c r="D22" s="14"/>
       <c r="E22" s="2" t="s">
         <v>290</v>
       </c>
       <c r="F22" s="3">
         <v>320000</v>
       </c>
-      <c r="G22" s="29" t="s">
+      <c r="G22" s="31" t="s">
         <v>291</v>
       </c>
-      <c r="H22" s="30">
+      <c r="H22" s="32">
         <v>340000</v>
       </c>
-      <c r="I22" s="32" t="s">
+      <c r="I22" s="34" t="s">
         <v>292</v>
       </c>
-      <c r="J22" s="35">
+      <c r="J22" s="37">
         <v>467000</v>
       </c>
       <c r="K22" s="2" t="s">
@@ -4091,26 +4705,26 @@
       </c>
     </row>
     <row r="23" spans="3:30">
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="13" t="s">
         <v>298</v>
       </c>
-      <c r="D23" s="12"/>
+      <c r="D23" s="14"/>
       <c r="E23" s="2" t="s">
         <v>299</v>
       </c>
       <c r="F23" s="3">
         <v>345000</v>
       </c>
-      <c r="G23" s="29" t="s">
+      <c r="G23" s="31" t="s">
         <v>300</v>
       </c>
-      <c r="H23" s="30">
+      <c r="H23" s="32">
         <v>360000</v>
       </c>
-      <c r="I23" s="36" t="s">
+      <c r="I23" s="38" t="s">
         <v>301</v>
       </c>
-      <c r="J23" s="37">
+      <c r="J23" s="39">
         <v>299000</v>
       </c>
       <c r="K23" s="2" t="s">
@@ -4136,26 +4750,26 @@
       </c>
     </row>
     <row r="24" spans="3:30">
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="13" t="s">
         <v>306</v>
       </c>
-      <c r="D24" s="12"/>
-      <c r="E24" s="20" t="s">
+      <c r="D24" s="14"/>
+      <c r="E24" s="22" t="s">
         <v>307</v>
       </c>
-      <c r="F24" s="25">
+      <c r="F24" s="27">
         <v>309000</v>
       </c>
-      <c r="G24" s="38" t="s">
+      <c r="G24" s="40" t="s">
         <v>308</v>
       </c>
-      <c r="H24" s="39">
+      <c r="H24" s="41">
         <v>269000</v>
       </c>
-      <c r="I24" s="36" t="s">
+      <c r="I24" s="38" t="s">
         <v>309</v>
       </c>
-      <c r="J24" s="40">
+      <c r="J24" s="42">
         <v>321000</v>
       </c>
       <c r="K24" s="2" t="s">
@@ -4181,26 +4795,26 @@
       </c>
     </row>
     <row r="25" spans="3:30">
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="13" t="s">
         <v>314</v>
       </c>
-      <c r="D25" s="12"/>
-      <c r="E25" s="20" t="s">
+      <c r="D25" s="14"/>
+      <c r="E25" s="22" t="s">
         <v>315</v>
       </c>
-      <c r="F25" s="25">
+      <c r="F25" s="27">
         <v>369000</v>
       </c>
-      <c r="G25" s="29" t="s">
+      <c r="G25" s="31" t="s">
         <v>316</v>
       </c>
-      <c r="H25" s="30">
+      <c r="H25" s="32">
         <v>396000</v>
       </c>
-      <c r="I25" s="41" t="s">
+      <c r="I25" s="43" t="s">
         <v>317</v>
       </c>
-      <c r="J25" s="42">
+      <c r="J25" s="44">
         <v>329000</v>
       </c>
       <c r="K25" s="2" t="s">
@@ -4225,27 +4839,27 @@
         <v>17000</v>
       </c>
     </row>
-    <row r="26" spans="3:30">
+    <row r="26" ht="15.15" spans="3:30">
       <c r="C26" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="D26" s="12"/>
-      <c r="E26" s="20" t="s">
+      <c r="D26" s="14"/>
+      <c r="E26" s="22" t="s">
         <v>323</v>
       </c>
-      <c r="F26" s="25">
+      <c r="F26" s="27">
         <v>372000</v>
       </c>
-      <c r="G26" s="29" t="s">
+      <c r="G26" s="31" t="s">
         <v>324</v>
       </c>
-      <c r="H26" s="30">
+      <c r="H26" s="32">
         <v>441000</v>
       </c>
-      <c r="I26" s="41" t="s">
+      <c r="I26" s="43" t="s">
         <v>325</v>
       </c>
-      <c r="J26" s="43">
+      <c r="J26" s="45">
         <v>349000</v>
       </c>
       <c r="K26" s="2" t="s">
@@ -4265,26 +4879,26 @@
       </c>
     </row>
     <row r="27" spans="3:30">
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="13" t="s">
         <v>329</v>
       </c>
-      <c r="D27" s="12"/>
-      <c r="E27" s="20" t="s">
+      <c r="D27" s="14"/>
+      <c r="E27" s="22" t="s">
         <v>330</v>
       </c>
-      <c r="F27" s="25">
+      <c r="F27" s="27">
         <v>425000</v>
       </c>
-      <c r="G27" s="29" t="s">
+      <c r="G27" s="31" t="s">
         <v>331</v>
       </c>
-      <c r="H27" s="30">
+      <c r="H27" s="32">
         <v>697000</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="J27" s="44">
+      <c r="J27" s="46">
         <v>280000</v>
       </c>
       <c r="K27" s="2" t="s">
@@ -4297,27 +4911,27 @@
         <v>334</v>
       </c>
     </row>
-    <row r="28" spans="3:30">
+    <row r="28" ht="15.15" spans="3:30">
       <c r="C28" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="D28" s="12"/>
-      <c r="E28" s="20" t="s">
+      <c r="D28" s="14"/>
+      <c r="E28" s="22" t="s">
         <v>336</v>
       </c>
-      <c r="F28" s="25">
+      <c r="F28" s="27">
         <v>522000</v>
       </c>
-      <c r="G28" s="29" t="s">
+      <c r="G28" s="31" t="s">
         <v>337</v>
       </c>
-      <c r="H28" s="30">
+      <c r="H28" s="32">
         <v>494000</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="J28" s="45">
+      <c r="J28" s="47">
         <v>426000</v>
       </c>
       <c r="K28" s="2" t="s">
@@ -4331,26 +4945,26 @@
       </c>
     </row>
     <row r="29" spans="3:30">
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="13" t="s">
         <v>341</v>
       </c>
-      <c r="D29" s="12"/>
-      <c r="E29" s="29" t="s">
+      <c r="D29" s="14"/>
+      <c r="E29" s="31" t="s">
         <v>342</v>
       </c>
-      <c r="F29" s="30">
+      <c r="F29" s="32">
         <v>398000</v>
       </c>
-      <c r="G29" s="29" t="s">
+      <c r="G29" s="31" t="s">
         <v>343</v>
       </c>
-      <c r="H29" s="30">
+      <c r="H29" s="32">
         <v>173000</v>
       </c>
-      <c r="I29" s="20" t="s">
+      <c r="I29" s="22" t="s">
         <v>344</v>
       </c>
-      <c r="J29" s="46">
+      <c r="J29" s="48">
         <v>207000</v>
       </c>
       <c r="K29" s="2" t="s">
@@ -4367,23 +4981,23 @@
       <c r="C30" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="D30" s="12"/>
-      <c r="E30" s="29" t="s">
+      <c r="D30" s="14"/>
+      <c r="E30" s="31" t="s">
         <v>348</v>
       </c>
-      <c r="F30" s="30">
+      <c r="F30" s="32">
         <v>777000</v>
       </c>
-      <c r="G30" s="29" t="s">
+      <c r="G30" s="31" t="s">
         <v>349</v>
       </c>
-      <c r="H30" s="30">
+      <c r="H30" s="32">
         <v>207000</v>
       </c>
-      <c r="I30" s="20" t="s">
+      <c r="I30" s="22" t="s">
         <v>350</v>
       </c>
-      <c r="J30" s="46">
+      <c r="J30" s="48">
         <v>257000</v>
       </c>
       <c r="K30" s="2" t="s">
@@ -4400,23 +5014,23 @@
       <c r="C31" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="D31" s="12"/>
-      <c r="E31" s="47" t="s">
+      <c r="D31" s="14"/>
+      <c r="E31" s="49" t="s">
         <v>354</v>
       </c>
-      <c r="F31" s="48">
+      <c r="F31" s="50">
         <v>341000</v>
       </c>
-      <c r="G31" s="29" t="s">
+      <c r="G31" s="31" t="s">
         <v>355</v>
       </c>
-      <c r="H31" s="30">
+      <c r="H31" s="32">
         <v>302000</v>
       </c>
-      <c r="I31" s="49" t="s">
+      <c r="I31" s="51" t="s">
         <v>356</v>
       </c>
-      <c r="J31" s="50">
+      <c r="J31" s="52">
         <v>295000</v>
       </c>
       <c r="K31" s="2" t="s">
@@ -4433,23 +5047,23 @@
       <c r="C32" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="D32" s="12"/>
-      <c r="E32" s="47" t="s">
+      <c r="D32" s="14"/>
+      <c r="E32" s="49" t="s">
         <v>360</v>
       </c>
-      <c r="F32" s="48">
+      <c r="F32" s="50">
         <v>388000</v>
       </c>
-      <c r="G32" s="38" t="s">
+      <c r="G32" s="40" t="s">
         <v>361</v>
       </c>
-      <c r="H32" s="39">
+      <c r="H32" s="41">
         <v>381000</v>
       </c>
-      <c r="I32" s="49" t="s">
+      <c r="I32" s="51" t="s">
         <v>362</v>
       </c>
-      <c r="J32" s="50">
+      <c r="J32" s="52">
         <v>405000</v>
       </c>
       <c r="K32" s="2" t="s">
@@ -4462,27 +5076,27 @@
         <v>364</v>
       </c>
     </row>
-    <row r="33" spans="3:13">
+    <row r="33" ht="15.15" spans="3:13">
       <c r="C33" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="D33" s="51"/>
-      <c r="E33" s="29" t="s">
+      <c r="D33" s="53"/>
+      <c r="E33" s="31" t="s">
         <v>366</v>
       </c>
-      <c r="F33" s="30">
+      <c r="F33" s="32">
         <v>648000</v>
       </c>
-      <c r="G33" s="29" t="s">
+      <c r="G33" s="31" t="s">
         <v>367</v>
       </c>
-      <c r="H33" s="48">
+      <c r="H33" s="50">
         <v>388000</v>
       </c>
-      <c r="I33" s="29" t="s">
+      <c r="I33" s="31" t="s">
         <v>368</v>
       </c>
-      <c r="J33" s="52">
+      <c r="J33" s="54">
         <v>641000</v>
       </c>
       <c r="K33" s="2" t="s">
@@ -4496,25 +5110,25 @@
       </c>
     </row>
     <row r="34" spans="3:13">
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="13" t="s">
         <v>371</v>
       </c>
-      <c r="E34" s="29" t="s">
+      <c r="E34" s="31" t="s">
         <v>372</v>
       </c>
-      <c r="F34" s="30">
+      <c r="F34" s="32">
         <v>793000</v>
       </c>
-      <c r="G34" s="29" t="s">
+      <c r="G34" s="31" t="s">
         <v>373</v>
       </c>
-      <c r="H34" s="48">
+      <c r="H34" s="50">
         <v>413000</v>
       </c>
-      <c r="I34" s="29" t="s">
+      <c r="I34" s="31" t="s">
         <v>374</v>
       </c>
-      <c r="J34" s="53">
+      <c r="J34" s="55">
         <v>754000</v>
       </c>
       <c r="K34" s="2" t="s">
@@ -4531,22 +5145,22 @@
       <c r="C35" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="E35" s="29" t="s">
+      <c r="E35" s="31" t="s">
         <v>378</v>
       </c>
-      <c r="F35" s="54">
+      <c r="F35" s="56">
         <v>747000</v>
       </c>
-      <c r="G35" s="29" t="s">
+      <c r="G35" s="31" t="s">
         <v>379</v>
       </c>
-      <c r="H35" s="30">
+      <c r="H35" s="32">
         <v>309000</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="J35" s="55">
+      <c r="J35" s="57">
         <v>312000</v>
       </c>
       <c r="K35" s="2" t="s">
@@ -4563,22 +5177,22 @@
       <c r="C36" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="E36" s="29" t="s">
+      <c r="E36" s="31" t="s">
         <v>384</v>
       </c>
-      <c r="F36" s="54">
+      <c r="F36" s="56">
         <v>882000</v>
       </c>
-      <c r="G36" s="29" t="s">
+      <c r="G36" s="31" t="s">
         <v>385</v>
       </c>
-      <c r="H36" s="30">
+      <c r="H36" s="32">
         <v>411000</v>
       </c>
-      <c r="I36" s="15" t="s">
+      <c r="I36" s="17" t="s">
         <v>386</v>
       </c>
-      <c r="J36" s="55">
+      <c r="J36" s="57">
         <v>381000</v>
       </c>
       <c r="K36" s="2" t="s">
@@ -4592,25 +5206,25 @@
       </c>
     </row>
     <row r="37" spans="3:13">
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="13" t="s">
         <v>389</v>
       </c>
-      <c r="E37" s="29" t="s">
+      <c r="E37" s="31" t="s">
         <v>390</v>
       </c>
-      <c r="F37" s="30">
+      <c r="F37" s="32">
         <v>356000</v>
       </c>
-      <c r="G37" s="29" t="s">
+      <c r="G37" s="31" t="s">
         <v>391</v>
       </c>
-      <c r="H37" s="30">
+      <c r="H37" s="32">
         <v>473000</v>
       </c>
-      <c r="I37" s="22" t="s">
+      <c r="I37" s="24" t="s">
         <v>392</v>
       </c>
-      <c r="J37" s="56">
+      <c r="J37" s="58">
         <v>365000</v>
       </c>
       <c r="K37" s="2" t="s">
@@ -4621,117 +5235,117 @@
       </c>
     </row>
     <row r="38" spans="3:13">
-      <c r="C38" s="11" t="s">
+      <c r="C38" s="13" t="s">
         <v>394</v>
       </c>
-      <c r="E38" s="29" t="s">
+      <c r="E38" s="31" t="s">
         <v>395</v>
       </c>
-      <c r="F38" s="30">
+      <c r="F38" s="32">
         <v>369000</v>
       </c>
-      <c r="G38" s="29" t="s">
+      <c r="G38" s="31" t="s">
         <v>396</v>
       </c>
-      <c r="H38" s="30">
+      <c r="H38" s="32">
         <v>329000</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="J38" s="57">
+      <c r="J38" s="59">
         <v>501000</v>
       </c>
     </row>
     <row r="39" spans="3:13">
-      <c r="C39" s="11" t="s">
+      <c r="C39" s="13" t="s">
         <v>398</v>
       </c>
-      <c r="E39" s="29" t="s">
+      <c r="E39" s="31" t="s">
         <v>399</v>
       </c>
-      <c r="F39" s="30">
+      <c r="F39" s="32">
         <v>465000</v>
       </c>
-      <c r="G39" s="29" t="s">
+      <c r="G39" s="31" t="s">
         <v>400</v>
       </c>
-      <c r="H39" s="30">
+      <c r="H39" s="32">
         <v>385000</v>
       </c>
-      <c r="I39" s="29" t="s">
+      <c r="I39" s="31" t="s">
         <v>401</v>
       </c>
-      <c r="J39" s="58">
+      <c r="J39" s="60">
         <v>740000</v>
       </c>
     </row>
     <row r="40" spans="3:13">
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="13" t="s">
         <v>402</v>
       </c>
-      <c r="E40" s="29" t="s">
+      <c r="E40" s="31" t="s">
         <v>403</v>
       </c>
-      <c r="F40" s="30">
+      <c r="F40" s="32">
         <v>543000</v>
       </c>
-      <c r="G40" s="29" t="s">
+      <c r="G40" s="31" t="s">
         <v>404</v>
       </c>
-      <c r="H40" s="30">
+      <c r="H40" s="32">
         <v>437000</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="J40" s="59">
+      <c r="J40" s="61">
         <v>278000</v>
       </c>
     </row>
     <row r="41" spans="3:13">
-      <c r="C41" s="11" t="s">
+      <c r="C41" s="13" t="s">
         <v>406</v>
       </c>
-      <c r="E41" s="29" t="s">
+      <c r="E41" s="31" t="s">
         <v>407</v>
       </c>
-      <c r="F41" s="30">
+      <c r="F41" s="32">
         <v>778000</v>
       </c>
-      <c r="G41" s="29" t="s">
+      <c r="G41" s="31" t="s">
         <v>408</v>
       </c>
-      <c r="H41" s="30">
+      <c r="H41" s="32">
         <v>566000</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="J41" s="31">
+      <c r="J41" s="33">
         <v>351000</v>
       </c>
     </row>
     <row r="42" spans="3:13">
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="13" t="s">
         <v>410</v>
       </c>
-      <c r="E42" s="29" t="s">
+      <c r="E42" s="31" t="s">
         <v>411</v>
       </c>
-      <c r="F42" s="30">
+      <c r="F42" s="32">
         <v>337000</v>
       </c>
-      <c r="G42" s="29" t="s">
+      <c r="G42" s="31" t="s">
         <v>412</v>
       </c>
-      <c r="H42" s="30">
+      <c r="H42" s="32">
         <v>636000</v>
       </c>
-      <c r="I42" s="20" t="s">
+      <c r="I42" s="22" t="s">
         <v>413</v>
       </c>
-      <c r="J42" s="60">
+      <c r="J42" s="62">
         <v>300000</v>
       </c>
     </row>
@@ -4739,22 +5353,22 @@
       <c r="C43" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E43" s="29" t="s">
+      <c r="E43" s="31" t="s">
         <v>415</v>
       </c>
-      <c r="F43" s="54">
+      <c r="F43" s="56">
         <v>440000</v>
       </c>
-      <c r="G43" s="29" t="s">
+      <c r="G43" s="31" t="s">
         <v>416</v>
       </c>
-      <c r="H43" s="30">
+      <c r="H43" s="32">
         <v>707000</v>
       </c>
-      <c r="I43" s="20" t="s">
+      <c r="I43" s="22" t="s">
         <v>417</v>
       </c>
-      <c r="J43" s="61">
+      <c r="J43" s="63">
         <v>322000</v>
       </c>
     </row>
@@ -4768,16 +5382,16 @@
       <c r="F44" s="3">
         <v>335000</v>
       </c>
-      <c r="G44" s="29" t="s">
+      <c r="G44" s="31" t="s">
         <v>420</v>
       </c>
-      <c r="H44" s="30">
+      <c r="H44" s="32">
         <v>420000</v>
       </c>
-      <c r="I44" s="62" t="s">
+      <c r="I44" s="64" t="s">
         <v>421</v>
       </c>
-      <c r="J44" s="63">
+      <c r="J44" s="65">
         <v>329000</v>
       </c>
     </row>
@@ -4791,16 +5405,16 @@
       <c r="F45" s="3">
         <v>448000</v>
       </c>
-      <c r="G45" s="29" t="s">
+      <c r="G45" s="31" t="s">
         <v>424</v>
       </c>
-      <c r="H45" s="30">
+      <c r="H45" s="32">
         <v>430000</v>
       </c>
-      <c r="I45" s="62" t="s">
+      <c r="I45" s="64" t="s">
         <v>425</v>
       </c>
-      <c r="J45" s="63">
+      <c r="J45" s="65">
         <v>445000</v>
       </c>
     </row>
@@ -4814,14 +5428,14 @@
       <c r="F46" s="3">
         <v>402000</v>
       </c>
-      <c r="G46" s="29" t="s">
+      <c r="G46" s="31" t="s">
         <v>428</v>
       </c>
-      <c r="H46" s="30">
+      <c r="H46" s="32">
         <v>400000</v>
       </c>
-      <c r="I46" s="62"/>
-      <c r="J46" s="63"/>
+      <c r="I46" s="64"/>
+      <c r="J46" s="65"/>
     </row>
     <row r="47" spans="3:13">
       <c r="C47" s="2" t="s">
@@ -4833,15 +5447,15 @@
       <c r="F47" s="3">
         <v>469000</v>
       </c>
-      <c r="G47" s="29" t="s">
+      <c r="G47" s="31" t="s">
         <v>431</v>
       </c>
-      <c r="H47" s="30">
+      <c r="H47" s="32">
         <v>382000</v>
       </c>
     </row>
     <row r="48" spans="3:13">
-      <c r="C48" s="11" t="s">
+      <c r="C48" s="13" t="s">
         <v>432</v>
       </c>
       <c r="E48" s="2" t="s">
@@ -4858,10 +5472,10 @@
       </c>
     </row>
     <row r="49" spans="5:8">
-      <c r="E49" s="20" t="s">
+      <c r="E49" s="22" t="s">
         <v>435</v>
       </c>
-      <c r="F49" s="25">
+      <c r="F49" s="27">
         <v>180000</v>
       </c>
       <c r="G49" s="2" t="s">
@@ -4872,10 +5486,10 @@
       </c>
     </row>
     <row r="50" spans="5:8">
-      <c r="E50" s="20" t="s">
+      <c r="E50" s="22" t="s">
         <v>437</v>
       </c>
-      <c r="F50" s="25">
+      <c r="F50" s="27">
         <v>230000</v>
       </c>
       <c r="G50" s="2" t="s">
@@ -4892,10 +5506,10 @@
       <c r="F51" s="3">
         <v>46000</v>
       </c>
-      <c r="G51" s="29" t="s">
+      <c r="G51" s="31" t="s">
         <v>440</v>
       </c>
-      <c r="H51" s="30">
+      <c r="H51" s="32">
         <v>446000</v>
       </c>
     </row>
@@ -4990,10 +5604,10 @@
       <c r="F58" s="3">
         <v>358000</v>
       </c>
-      <c r="G58" s="29" t="s">
+      <c r="G58" s="31" t="s">
         <v>454</v>
       </c>
-      <c r="H58" s="30">
+      <c r="H58" s="32">
         <v>541000</v>
       </c>
     </row>
@@ -5004,42 +5618,42 @@
       <c r="F59" s="3">
         <v>320000</v>
       </c>
-      <c r="G59" s="47" t="s">
+      <c r="G59" s="49" t="s">
         <v>456</v>
       </c>
-      <c r="H59" s="48">
+      <c r="H59" s="50">
         <v>515000</v>
       </c>
     </row>
     <row r="60" spans="5:8">
-      <c r="G60" s="64" t="s">
+      <c r="G60" s="66" t="s">
         <v>457</v>
       </c>
-      <c r="H60" s="65">
+      <c r="H60" s="67">
         <v>701000</v>
       </c>
     </row>
     <row r="61" spans="5:8">
-      <c r="G61" s="64" t="s">
+      <c r="G61" s="66" t="s">
         <v>458</v>
       </c>
-      <c r="H61" s="65">
+      <c r="H61" s="67">
         <v>794000</v>
       </c>
     </row>
     <row r="62" spans="5:8">
-      <c r="G62" s="38" t="s">
+      <c r="G62" s="40" t="s">
         <v>459</v>
       </c>
-      <c r="H62" s="39">
+      <c r="H62" s="41">
         <v>628000</v>
       </c>
     </row>
     <row r="63" spans="5:8">
-      <c r="G63" s="38" t="s">
+      <c r="G63" s="40" t="s">
         <v>460</v>
       </c>
-      <c r="H63" s="39">
+      <c r="H63" s="41">
         <v>747000</v>
       </c>
     </row>
@@ -5095,7 +5709,7 @@
       <c r="G70" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="H70" s="18">
+      <c r="H70" s="20">
         <v>903000</v>
       </c>
     </row>
@@ -5108,290 +5722,290 @@
       </c>
     </row>
     <row r="72" spans="7:8">
-      <c r="G72" s="49" t="s">
+      <c r="G72" s="51" t="s">
         <v>469</v>
       </c>
-      <c r="H72" s="66">
+      <c r="H72" s="68">
         <v>268000</v>
       </c>
     </row>
     <row r="73" spans="7:8">
-      <c r="G73" s="49" t="s">
+      <c r="G73" s="51" t="s">
         <v>470</v>
       </c>
-      <c r="H73" s="66">
+      <c r="H73" s="68">
         <v>325000</v>
       </c>
     </row>
     <row r="74" spans="7:8">
-      <c r="G74" s="67" t="s">
+      <c r="G74" s="69" t="s">
         <v>471</v>
       </c>
-      <c r="H74" s="66">
+      <c r="H74" s="68">
         <v>297000</v>
       </c>
     </row>
     <row r="75" spans="7:8">
-      <c r="G75" s="67" t="s">
+      <c r="G75" s="69" t="s">
         <v>472</v>
       </c>
-      <c r="H75" s="66">
+      <c r="H75" s="68">
         <v>359000</v>
       </c>
     </row>
     <row r="76" spans="7:8">
-      <c r="G76" s="29" t="s">
+      <c r="G76" s="31" t="s">
         <v>473</v>
       </c>
-      <c r="H76" s="30">
+      <c r="H76" s="32">
         <v>297000</v>
       </c>
     </row>
     <row r="77" spans="7:8">
-      <c r="G77" s="29" t="s">
+      <c r="G77" s="31" t="s">
         <v>474</v>
       </c>
-      <c r="H77" s="30">
+      <c r="H77" s="32">
         <v>394000</v>
       </c>
     </row>
     <row r="78" spans="7:8">
-      <c r="G78" s="68" t="s">
+      <c r="G78" s="70" t="s">
         <v>475</v>
       </c>
-      <c r="H78" s="18">
+      <c r="H78" s="20">
         <v>446000</v>
       </c>
     </row>
     <row r="79" spans="7:8">
-      <c r="G79" s="38" t="s">
+      <c r="G79" s="40" t="s">
         <v>476</v>
       </c>
-      <c r="H79" s="39">
+      <c r="H79" s="41">
         <v>337000</v>
       </c>
     </row>
     <row r="80" spans="7:8">
-      <c r="G80" s="38" t="s">
+      <c r="G80" s="40" t="s">
         <v>477</v>
       </c>
-      <c r="H80" s="39">
+      <c r="H80" s="41">
         <v>358000</v>
       </c>
     </row>
     <row r="81" spans="7:8">
-      <c r="G81" s="38" t="s">
+      <c r="G81" s="40" t="s">
         <v>478</v>
       </c>
-      <c r="H81" s="39">
+      <c r="H81" s="41">
         <v>435000</v>
       </c>
     </row>
     <row r="82" spans="7:8">
-      <c r="G82" s="38" t="s">
+      <c r="G82" s="40" t="s">
         <v>479</v>
       </c>
-      <c r="H82" s="39">
+      <c r="H82" s="41">
         <v>497000</v>
       </c>
     </row>
     <row r="83" spans="7:8">
-      <c r="G83" s="47" t="s">
+      <c r="G83" s="49" t="s">
         <v>480</v>
       </c>
-      <c r="H83" s="48">
+      <c r="H83" s="50">
         <v>433000</v>
       </c>
     </row>
     <row r="84" spans="7:8">
-      <c r="G84" s="47" t="s">
+      <c r="G84" s="49" t="s">
         <v>481</v>
       </c>
-      <c r="H84" s="48">
+      <c r="H84" s="50">
         <v>610000</v>
       </c>
     </row>
     <row r="85" spans="7:8">
-      <c r="G85" s="47" t="s">
+      <c r="G85" s="49" t="s">
         <v>482</v>
       </c>
-      <c r="H85" s="48">
+      <c r="H85" s="50">
         <v>145000</v>
       </c>
     </row>
     <row r="86" spans="7:8">
-      <c r="G86" s="47" t="s">
+      <c r="G86" s="49" t="s">
         <v>483</v>
       </c>
-      <c r="H86" s="48">
+      <c r="H86" s="50">
         <v>178000</v>
       </c>
     </row>
     <row r="87" spans="7:8">
-      <c r="G87" s="47" t="s">
+      <c r="G87" s="49" t="s">
         <v>484</v>
       </c>
-      <c r="H87" s="48">
+      <c r="H87" s="50">
         <v>259000</v>
       </c>
     </row>
     <row r="88" spans="7:8">
-      <c r="G88" s="47" t="s">
+      <c r="G88" s="49" t="s">
         <v>485</v>
       </c>
-      <c r="H88" s="48">
+      <c r="H88" s="50">
         <v>176000</v>
       </c>
     </row>
     <row r="89" spans="7:8">
-      <c r="G89" s="47" t="s">
+      <c r="G89" s="49" t="s">
         <v>486</v>
       </c>
-      <c r="H89" s="48">
+      <c r="H89" s="50">
         <v>180000</v>
       </c>
     </row>
     <row r="90" spans="7:8">
-      <c r="G90" s="47" t="s">
+      <c r="G90" s="49" t="s">
         <v>487</v>
       </c>
-      <c r="H90" s="48">
+      <c r="H90" s="50">
         <v>240000</v>
       </c>
     </row>
     <row r="91" spans="7:8">
-      <c r="G91" s="47" t="s">
+      <c r="G91" s="49" t="s">
         <v>488</v>
       </c>
-      <c r="H91" s="48">
+      <c r="H91" s="50">
         <v>288000</v>
       </c>
     </row>
     <row r="92" spans="7:8">
-      <c r="G92" s="47" t="s">
+      <c r="G92" s="49" t="s">
         <v>489</v>
       </c>
-      <c r="H92" s="48">
+      <c r="H92" s="50">
         <v>568000</v>
       </c>
     </row>
     <row r="93" spans="7:8">
-      <c r="G93" s="47" t="s">
+      <c r="G93" s="49" t="s">
         <v>490</v>
       </c>
-      <c r="H93" s="48">
+      <c r="H93" s="50">
         <v>579000</v>
       </c>
     </row>
     <row r="94" spans="7:8">
-      <c r="G94" s="47" t="s">
+      <c r="G94" s="49" t="s">
         <v>491</v>
       </c>
-      <c r="H94" s="48">
+      <c r="H94" s="50">
         <v>473000</v>
       </c>
     </row>
     <row r="95" spans="7:8">
-      <c r="G95" s="69" t="s">
+      <c r="G95" s="71" t="s">
         <v>492</v>
       </c>
-      <c r="H95" s="70">
+      <c r="H95" s="72">
         <v>43000</v>
       </c>
     </row>
     <row r="96" spans="7:8">
-      <c r="G96" s="69" t="s">
+      <c r="G96" s="71" t="s">
         <v>493</v>
       </c>
-      <c r="H96" s="70">
+      <c r="H96" s="72">
         <v>48000</v>
       </c>
     </row>
     <row r="97" spans="2:8">
-      <c r="G97" s="71" t="s">
+      <c r="G97" s="73" t="s">
         <v>494</v>
       </c>
-      <c r="H97" s="72">
+      <c r="H97" s="74">
         <v>47000</v>
       </c>
     </row>
     <row r="98" spans="2:8">
-      <c r="G98" s="69" t="s">
+      <c r="G98" s="71" t="s">
         <v>495</v>
       </c>
-      <c r="H98" s="70">
+      <c r="H98" s="72">
         <v>53000</v>
       </c>
     </row>
     <row r="99" spans="2:8">
-      <c r="G99" s="69" t="s">
+      <c r="G99" s="71" t="s">
         <v>496</v>
       </c>
-      <c r="H99" s="70">
+      <c r="H99" s="72">
         <v>54000</v>
       </c>
     </row>
     <row r="100" spans="2:8">
-      <c r="G100" s="69" t="s">
+      <c r="G100" s="71" t="s">
         <v>497</v>
       </c>
-      <c r="H100" s="70">
+      <c r="H100" s="72">
         <v>56000</v>
       </c>
     </row>
     <row r="101" spans="2:8">
-      <c r="G101" s="69" t="s">
+      <c r="G101" s="71" t="s">
         <v>498</v>
       </c>
-      <c r="H101" s="70">
+      <c r="H101" s="72">
         <v>54000</v>
       </c>
     </row>
     <row r="102" spans="2:8">
-      <c r="G102" s="38" t="s">
+      <c r="G102" s="40" t="s">
         <v>499</v>
       </c>
-      <c r="H102" s="39">
+      <c r="H102" s="41">
         <v>250000</v>
       </c>
     </row>
     <row r="103" spans="2:8">
-      <c r="G103" s="38" t="s">
+      <c r="G103" s="40" t="s">
         <v>500</v>
       </c>
-      <c r="H103" s="39">
+      <c r="H103" s="41">
         <v>303000</v>
       </c>
     </row>
     <row r="104" spans="2:8">
-      <c r="G104" s="38" t="s">
+      <c r="G104" s="40" t="s">
         <v>501</v>
       </c>
-      <c r="H104" s="39">
+      <c r="H104" s="41">
         <v>330000</v>
       </c>
     </row>
     <row r="105" spans="2:8">
-      <c r="G105" s="38" t="s">
+      <c r="G105" s="40" t="s">
         <v>502</v>
       </c>
-      <c r="H105" s="39">
+      <c r="H105" s="41">
         <v>387000</v>
       </c>
     </row>
     <row r="106" spans="2:8">
-      <c r="G106" s="38" t="s">
+      <c r="G106" s="40" t="s">
         <v>503</v>
       </c>
-      <c r="H106" s="39">
+      <c r="H106" s="41">
         <v>578000</v>
       </c>
     </row>
     <row r="107" spans="2:8">
-      <c r="G107" s="38" t="s">
+      <c r="G107" s="40" t="s">
         <v>504</v>
       </c>
-      <c r="H107" s="39">
+      <c r="H107" s="41">
         <v>722000</v>
       </c>
     </row>
@@ -5406,5 +6020,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor main window service, add autosave feature, and implement update check worker; enhance error handling in print functionality and update version management
</commit_message>
<xml_diff>
--- a/app/data/BangGia.xlsx
+++ b/app/data/BangGia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thotr\OneDrive\Desktop\Toa Hang\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4863E3AD-2897-4A7F-8B85-4741BC7A0747}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB6A82C-6513-4991-AB5D-34D9FDB5ED72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="510">
   <si>
     <t>GS</t>
   </si>
@@ -1557,22 +1557,37 @@
   </si>
   <si>
     <t>110/17 DURO Thái</t>
+  </si>
+  <si>
+    <t>120/70-12 DURO</t>
+  </si>
+  <si>
+    <t>90/80-14 DURO</t>
+  </si>
+  <si>
+    <t>90/80-17 DURO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1592,37 +1607,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1635,25 +1621,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF00B0F0"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF00B0F0"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1663,23 +1635,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF92D050"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1702,6 +1661,70 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF00B0F0"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF92D050"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1991,148 +2014,151 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="13" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="21" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="12" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="21" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="21" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="12" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="12" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="13" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="13" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="11" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="18" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="11" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="18" fillId="3" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="19" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="19" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="1" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="12" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="12" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="15" fillId="4" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="15" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="15" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="3" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="20" fillId="3" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="3" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="20" fillId="3" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="19" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2415,133 +2441,133 @@
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.88671875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" style="28" customWidth="1"/>
     <col min="3" max="3" width="22.6640625" style="2" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" style="4" customWidth="1"/>
     <col min="5" max="5" width="34.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" style="28" customWidth="1"/>
     <col min="7" max="7" width="25.33203125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="28" customWidth="1"/>
     <col min="9" max="9" width="31.5546875" style="2" customWidth="1"/>
-    <col min="10" max="10" width="13" style="5" customWidth="1"/>
+    <col min="10" max="10" width="13" style="78" customWidth="1"/>
     <col min="11" max="11" width="28.109375" style="2" customWidth="1"/>
-    <col min="12" max="12" width="10.6640625" style="3" customWidth="1"/>
+    <col min="12" max="12" width="10.6640625" style="28" customWidth="1"/>
     <col min="13" max="13" width="29.5546875" style="2" customWidth="1"/>
     <col min="14" max="14" width="10.6640625" style="3" customWidth="1"/>
     <col min="15" max="15" width="17.33203125" style="2" customWidth="1"/>
     <col min="16" max="16" width="10.6640625" style="3" customWidth="1"/>
     <col min="17" max="17" width="19.6640625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="10.6640625" style="3" customWidth="1"/>
+    <col min="18" max="18" width="10.6640625" style="28" customWidth="1"/>
     <col min="19" max="19" width="28.33203125" style="2" customWidth="1"/>
-    <col min="20" max="20" width="10.6640625" style="3" customWidth="1"/>
+    <col min="20" max="20" width="10.6640625" style="28" customWidth="1"/>
     <col min="21" max="21" width="20.5546875" style="2" customWidth="1"/>
-    <col min="22" max="22" width="10.6640625" style="3" customWidth="1"/>
+    <col min="22" max="22" width="10.6640625" style="28" customWidth="1"/>
     <col min="23" max="23" width="21.5546875" style="2" customWidth="1"/>
-    <col min="24" max="24" width="10.6640625" style="3" customWidth="1"/>
+    <col min="24" max="24" width="10.6640625" style="28" customWidth="1"/>
     <col min="25" max="25" width="26.6640625" style="2" customWidth="1"/>
-    <col min="26" max="26" width="10.6640625" style="3" customWidth="1"/>
+    <col min="26" max="26" width="10.6640625" style="28" customWidth="1"/>
     <col min="27" max="27" width="33.44140625" style="2" customWidth="1"/>
-    <col min="28" max="28" width="22.5546875" style="3" customWidth="1"/>
+    <col min="28" max="28" width="22.5546875" style="28" customWidth="1"/>
     <col min="29" max="29" width="19.44140625" style="2" customWidth="1"/>
-    <col min="30" max="30" width="18" style="2" customWidth="1"/>
+    <col min="30" max="30" width="18" style="28" customWidth="1"/>
     <col min="31" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="1" customFormat="1">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="6" t="s">
+      <c r="B1" s="45"/>
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="7"/>
-      <c r="E1" s="8" t="s">
+      <c r="D1" s="6"/>
+      <c r="E1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="9"/>
-      <c r="G1" s="8" t="s">
+      <c r="F1" s="32"/>
+      <c r="G1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="9"/>
-      <c r="I1" s="8" t="s">
+      <c r="H1" s="32"/>
+      <c r="I1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="10"/>
-      <c r="K1" s="8" t="s">
+      <c r="J1" s="47"/>
+      <c r="K1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="9"/>
-      <c r="M1" s="8" t="s">
+      <c r="L1" s="32"/>
+      <c r="M1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="9"/>
-      <c r="O1" s="8" t="s">
+      <c r="N1" s="8"/>
+      <c r="O1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="8" t="s">
+      <c r="P1" s="8"/>
+      <c r="Q1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="R1" s="9"/>
-      <c r="S1" s="8" t="s">
+      <c r="R1" s="32"/>
+      <c r="S1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="T1" s="9"/>
-      <c r="U1" s="8" t="s">
+      <c r="T1" s="32"/>
+      <c r="U1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="V1" s="9"/>
-      <c r="W1" s="8" t="s">
+      <c r="V1" s="32"/>
+      <c r="W1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="X1" s="9"/>
-      <c r="Y1" s="8" t="s">
+      <c r="X1" s="32"/>
+      <c r="Y1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="Z1" s="9"/>
-      <c r="AA1" s="8" t="s">
+      <c r="Z1" s="32"/>
+      <c r="AA1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="AB1" s="9"/>
-      <c r="AC1" s="73" t="s">
+      <c r="AB1" s="32"/>
+      <c r="AC1" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="AD1" s="74"/>
+      <c r="AD1" s="30"/>
     </row>
     <row r="2" spans="1:30">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="28">
         <v>239000</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="12"/>
+      <c r="D2" s="10"/>
       <c r="E2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="28">
         <v>160000</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="28">
         <v>158000</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="13">
+      <c r="J2" s="48">
         <v>152000</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="L2" s="3">
+      <c r="L2" s="28">
         <v>730000</v>
       </c>
       <c r="M2" s="2" t="s">
@@ -2553,79 +2579,79 @@
       <c r="Q2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="R2" s="3">
+      <c r="R2" s="28">
         <v>400000</v>
       </c>
       <c r="S2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="T2" s="3">
+      <c r="T2" s="28">
         <v>154000</v>
       </c>
       <c r="U2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="V2" s="3">
+      <c r="V2" s="28">
         <v>226000</v>
       </c>
       <c r="W2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="X2" s="3">
+      <c r="X2" s="28">
         <v>91000</v>
       </c>
       <c r="Y2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="Z2" s="3">
+      <c r="Z2" s="28">
         <v>163000</v>
       </c>
       <c r="AA2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AB2" s="3">
+      <c r="AB2" s="28">
         <v>315000</v>
       </c>
       <c r="AC2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AD2" s="3">
+      <c r="AD2" s="28">
         <v>319000</v>
       </c>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="28">
         <v>252000</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="12"/>
+      <c r="D3" s="10"/>
       <c r="E3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="28">
         <v>202000</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="28">
         <v>158000</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J3" s="14">
+      <c r="J3" s="49">
         <v>204000</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" s="28">
         <v>670000</v>
       </c>
       <c r="M3" s="2" t="s">
@@ -2637,79 +2663,79 @@
       <c r="Q3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="R3" s="3">
+      <c r="R3" s="28">
         <v>505000</v>
       </c>
       <c r="S3" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="T3" s="3">
+      <c r="T3" s="28">
         <v>154000</v>
       </c>
       <c r="U3" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V3" s="3">
+      <c r="V3" s="28">
         <v>212000</v>
       </c>
       <c r="W3" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="X3" s="3">
+      <c r="X3" s="28">
         <v>103000</v>
       </c>
       <c r="Y3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="Z3" s="3">
+      <c r="Z3" s="28">
         <v>163000</v>
       </c>
       <c r="AA3" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AB3" s="3">
+      <c r="AB3" s="28">
         <v>315000</v>
       </c>
       <c r="AC3" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AD3" s="3">
+      <c r="AD3" s="28">
         <v>225000</v>
       </c>
     </row>
     <row r="4" spans="1:30">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="28">
         <v>280000</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="12"/>
+      <c r="D4" s="10"/>
       <c r="E4" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="28">
         <v>171000</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="28">
         <v>192000</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="I4" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="J4" s="16">
+      <c r="J4" s="50">
         <v>151000</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="L4" s="3">
+      <c r="L4" s="28">
         <v>495000</v>
       </c>
       <c r="M4" s="2" t="s">
@@ -2721,79 +2747,79 @@
       <c r="Q4" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="R4" s="3">
+      <c r="R4" s="28">
         <v>545000</v>
       </c>
       <c r="S4" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="T4" s="3">
+      <c r="T4" s="28">
         <v>198000</v>
       </c>
       <c r="U4" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="V4" s="3">
+      <c r="V4" s="28">
         <v>198000</v>
       </c>
       <c r="W4" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="X4" s="3">
+      <c r="X4" s="28">
         <v>134000</v>
       </c>
       <c r="Y4" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="Z4" s="3">
+      <c r="Z4" s="28">
         <v>205000</v>
       </c>
       <c r="AA4" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="AB4" s="3">
+      <c r="AB4" s="28">
         <v>315000</v>
       </c>
       <c r="AC4" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="AD4" s="3">
+      <c r="AD4" s="28">
         <v>165000</v>
       </c>
     </row>
     <row r="5" spans="1:30">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="28">
         <v>221000</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="12"/>
+      <c r="D5" s="10"/>
       <c r="E5" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="28">
         <v>216000</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="28">
         <v>192000</v>
       </c>
-      <c r="I5" s="15" t="s">
+      <c r="I5" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="J5" s="17">
+      <c r="J5" s="51">
         <v>192000</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="L5" s="3">
+      <c r="L5" s="28">
         <v>530000</v>
       </c>
       <c r="M5" s="2" t="s">
@@ -2805,79 +2831,79 @@
       <c r="Q5" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="R5" s="3">
+      <c r="R5" s="28">
         <v>800000</v>
       </c>
       <c r="S5" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="T5" s="3">
+      <c r="T5" s="28">
         <v>198000</v>
       </c>
       <c r="U5" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="V5" s="3">
+      <c r="V5" s="28">
         <v>254000</v>
       </c>
       <c r="W5" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="X5" s="3">
+      <c r="X5" s="28">
         <v>81000</v>
       </c>
       <c r="Y5" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="Z5" s="3">
+      <c r="Z5" s="28">
         <v>206000</v>
       </c>
       <c r="AA5" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AB5" s="3">
+      <c r="AB5" s="28">
         <v>345000</v>
       </c>
       <c r="AC5" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AD5" s="3">
+      <c r="AD5" s="28">
         <v>168000</v>
       </c>
     </row>
     <row r="6" spans="1:30">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="28">
         <v>249000</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D6" s="12"/>
+      <c r="D6" s="10"/>
       <c r="E6" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="28">
         <v>210000</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="28">
         <v>271000</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="J6" s="13">
+      <c r="J6" s="48">
         <v>177000</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L6" s="3">
+      <c r="L6" s="28">
         <v>616000</v>
       </c>
       <c r="M6" s="2" t="s">
@@ -2889,79 +2915,79 @@
       <c r="Q6" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="R6" s="3">
+      <c r="R6" s="28">
         <v>820000</v>
       </c>
       <c r="S6" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="T6" s="3">
+      <c r="T6" s="28">
         <v>220000</v>
       </c>
       <c r="U6" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="V6" s="3">
+      <c r="V6" s="28">
         <v>322000</v>
       </c>
       <c r="W6" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="X6" s="3">
+      <c r="X6" s="28">
         <v>102000</v>
       </c>
       <c r="Y6" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="Z6" s="3">
+      <c r="Z6" s="28">
         <v>194000</v>
       </c>
       <c r="AA6" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AB6" s="3">
+      <c r="AB6" s="28">
         <v>435000</v>
       </c>
       <c r="AC6" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="AD6" s="3">
+      <c r="AD6" s="28">
         <v>180000</v>
       </c>
     </row>
     <row r="7" spans="1:30">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="28">
         <v>382000</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="D7" s="12"/>
+      <c r="D7" s="10"/>
       <c r="E7" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="28">
         <v>264000</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="28">
         <v>231000</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="J7" s="14">
+      <c r="J7" s="49">
         <v>228000</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="L7" s="3">
+      <c r="L7" s="28">
         <v>720000</v>
       </c>
       <c r="M7" s="2" t="s">
@@ -2973,79 +2999,79 @@
       <c r="Q7" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="R7" s="3">
+      <c r="R7" s="28">
         <v>990000</v>
       </c>
       <c r="S7" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="T7" s="3">
+      <c r="T7" s="28">
         <v>220000</v>
       </c>
       <c r="U7" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="V7" s="3">
+      <c r="V7" s="28">
         <v>355000</v>
       </c>
       <c r="W7" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="X7" s="3">
+      <c r="X7" s="28">
         <v>96000</v>
       </c>
       <c r="Y7" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="Z7" s="3">
+      <c r="Z7" s="28">
         <v>163000</v>
       </c>
       <c r="AA7" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="AB7" s="3">
+      <c r="AB7" s="28">
         <v>380000</v>
       </c>
       <c r="AC7" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="AD7" s="3">
+      <c r="AD7" s="28">
         <v>215000</v>
       </c>
     </row>
     <row r="8" spans="1:30">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="28">
         <v>412000</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="12"/>
+      <c r="D8" s="10"/>
       <c r="E8" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="28">
         <v>226000</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="H8" s="18">
+      <c r="H8" s="34">
         <v>286000</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J8" s="13">
+      <c r="J8" s="48">
         <v>212000</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="L8" s="3">
+      <c r="L8" s="28">
         <v>672000</v>
       </c>
       <c r="M8" s="2" t="s">
@@ -3057,79 +3083,79 @@
       <c r="Q8" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="R8" s="3">
+      <c r="R8" s="28">
         <v>690000</v>
       </c>
       <c r="S8" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="T8" s="3">
+      <c r="T8" s="28">
         <v>249000</v>
       </c>
       <c r="U8" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="V8" s="3">
+      <c r="V8" s="28">
         <v>387000</v>
       </c>
       <c r="W8" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="X8" s="3">
+      <c r="X8" s="28">
         <v>128000</v>
       </c>
       <c r="Y8" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="Z8" s="3">
+      <c r="Z8" s="28">
         <v>247000</v>
       </c>
       <c r="AA8" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="AB8" s="3">
+      <c r="AB8" s="28">
         <v>400000</v>
       </c>
       <c r="AC8" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="AD8" s="3">
+      <c r="AD8" s="28">
         <v>269000</v>
       </c>
     </row>
     <row r="9" spans="1:30">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="28">
         <v>347000</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="D9" s="12"/>
+      <c r="D9" s="10"/>
       <c r="E9" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="28">
         <v>228000</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="28">
         <v>275000</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="J9" s="14">
+      <c r="J9" s="49">
         <v>287000</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="L9" s="3">
+      <c r="L9" s="28">
         <v>454000</v>
       </c>
       <c r="M9" s="2" t="s">
@@ -3141,79 +3167,79 @@
       <c r="Q9" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="R9" s="3">
+      <c r="R9" s="28">
         <v>920000</v>
       </c>
       <c r="S9" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="T9" s="19">
+      <c r="T9" s="33">
         <v>260000</v>
       </c>
       <c r="U9" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="V9" s="3">
+      <c r="V9" s="28">
         <v>338000</v>
       </c>
       <c r="W9" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="X9" s="3">
+      <c r="X9" s="28">
         <v>122000</v>
       </c>
       <c r="Y9" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="Z9" s="3">
+      <c r="Z9" s="28">
         <v>174000</v>
       </c>
       <c r="AA9" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="AB9" s="3">
+      <c r="AB9" s="28">
         <v>385000</v>
       </c>
       <c r="AC9" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="AD9" s="3">
+      <c r="AD9" s="28">
         <v>280000</v>
       </c>
     </row>
     <row r="10" spans="1:30">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="28">
         <v>221000</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="D10" s="12"/>
+      <c r="D10" s="10"/>
       <c r="E10" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="28">
         <v>282000</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="H10" s="21">
+      <c r="H10" s="35">
         <v>348000</v>
       </c>
-      <c r="I10" s="22" t="s">
+      <c r="I10" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="J10" s="23">
+      <c r="J10" s="52">
         <v>218000</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="L10" s="3">
+      <c r="L10" s="28">
         <v>550000</v>
       </c>
       <c r="M10" s="2" t="s">
@@ -3225,43 +3251,43 @@
       <c r="Q10" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="R10" s="3">
+      <c r="R10" s="28">
         <v>1140000</v>
       </c>
       <c r="S10" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="T10" s="3">
+      <c r="T10" s="28">
         <v>332000</v>
       </c>
       <c r="U10" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="V10" s="3">
+      <c r="V10" s="28">
         <v>620000</v>
       </c>
       <c r="W10" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="X10" s="3">
+      <c r="X10" s="28">
         <v>128000</v>
       </c>
       <c r="Y10" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="Z10" s="3">
+      <c r="Z10" s="28">
         <v>220000</v>
       </c>
       <c r="AA10" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="AB10" s="3">
+      <c r="AB10" s="28">
         <v>440000</v>
       </c>
       <c r="AC10" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="AD10" s="3">
+      <c r="AD10" s="28">
         <v>290000</v>
       </c>
     </row>
@@ -3269,35 +3295,35 @@
       <c r="A11" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="28">
         <v>332000</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11" s="10"/>
       <c r="E11" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="28">
         <v>235000</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="G11" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="H11" s="21">
+      <c r="H11" s="35">
         <v>370000</v>
       </c>
-      <c r="I11" s="22" t="s">
+      <c r="I11" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="J11" s="24">
+      <c r="J11" s="53">
         <v>270000</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="L11" s="3">
+      <c r="L11" s="28">
         <v>739000</v>
       </c>
       <c r="M11" s="2" t="s">
@@ -3309,43 +3335,43 @@
       <c r="Q11" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="R11" s="3">
+      <c r="R11" s="28">
         <v>545000</v>
       </c>
       <c r="S11" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="T11" s="3">
+      <c r="T11" s="28">
         <v>275000</v>
       </c>
       <c r="U11" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="V11" s="3">
+      <c r="V11" s="28">
         <v>95000</v>
       </c>
       <c r="W11" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="X11" s="3">
+      <c r="X11" s="28">
         <v>101000</v>
       </c>
       <c r="Y11" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="Z11" s="3">
+      <c r="Z11" s="28">
         <v>220000</v>
       </c>
       <c r="AA11" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="AB11" s="3">
+      <c r="AB11" s="28">
         <v>435000</v>
       </c>
       <c r="AC11" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="AD11" s="3">
+      <c r="AD11" s="28">
         <v>470000</v>
       </c>
     </row>
@@ -3353,35 +3379,35 @@
       <c r="A12" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="28">
         <v>800000</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="D12" s="12"/>
+      <c r="D12" s="10"/>
       <c r="E12" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="28">
         <v>289000</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="36">
         <v>348000</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="I12" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="J12" s="26">
+      <c r="J12" s="54">
         <v>395000</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="L12" s="3">
+      <c r="L12" s="28">
         <v>774000</v>
       </c>
       <c r="M12" s="2" t="s">
@@ -3393,76 +3419,76 @@
       <c r="Q12" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="R12" s="3">
+      <c r="R12" s="28">
         <v>570000</v>
       </c>
       <c r="S12" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="T12" s="3">
+      <c r="T12" s="28">
         <v>311000</v>
       </c>
       <c r="U12" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="V12" s="3">
+      <c r="V12" s="28">
         <v>87000</v>
       </c>
       <c r="W12" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="X12" s="3">
+      <c r="X12" s="28">
         <v>113000</v>
       </c>
       <c r="Y12" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="Z12" s="3">
+      <c r="Z12" s="28">
         <v>220000</v>
       </c>
       <c r="AA12" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AB12" s="3">
+      <c r="AB12" s="28">
         <v>695000</v>
       </c>
       <c r="AC12" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="AD12" s="3">
+      <c r="AD12" s="28">
         <v>340000</v>
       </c>
     </row>
     <row r="13" spans="1:30">
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="46" t="s">
         <v>180</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="D13" s="12"/>
-      <c r="E13" s="22" t="s">
+      <c r="D13" s="10"/>
+      <c r="E13" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="F13" s="19">
+      <c r="F13" s="33">
         <v>254000</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="G13" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="H13" s="25">
+      <c r="H13" s="36">
         <v>370000</v>
       </c>
-      <c r="I13" s="15" t="s">
+      <c r="I13" s="11" t="s">
         <v>184</v>
       </c>
-      <c r="J13" s="28">
+      <c r="J13" s="55">
         <v>431000</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="L13" s="3">
+      <c r="L13" s="28">
         <v>865000</v>
       </c>
       <c r="M13" s="2" t="s">
@@ -3474,73 +3500,73 @@
       <c r="Q13" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="R13" s="3">
+      <c r="R13" s="28">
         <v>600000</v>
       </c>
       <c r="S13" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="T13" s="3">
+      <c r="T13" s="28">
         <v>220000</v>
       </c>
       <c r="U13" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="V13" s="3">
+      <c r="V13" s="28">
         <v>232000</v>
       </c>
       <c r="W13" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="X13" s="3">
+      <c r="X13" s="28">
         <v>89000</v>
       </c>
       <c r="Y13" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="Z13" s="3">
+      <c r="Z13" s="28">
         <v>207000</v>
       </c>
       <c r="AA13" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="AB13" s="3">
+      <c r="AB13" s="28">
         <v>695000</v>
       </c>
       <c r="AC13" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="AD13" s="3">
+      <c r="AD13" s="28">
         <v>32000</v>
       </c>
     </row>
     <row r="14" spans="1:30">
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="D14" s="12"/>
-      <c r="E14" s="22" t="s">
+      <c r="D14" s="10"/>
+      <c r="E14" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="F14" s="19">
+      <c r="F14" s="33">
         <v>291000</v>
       </c>
-      <c r="G14" s="29" t="s">
+      <c r="G14" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="H14" s="30">
+      <c r="H14" s="37">
         <v>281000</v>
       </c>
-      <c r="I14" s="15" t="s">
+      <c r="I14" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="J14" s="17">
+      <c r="J14" s="51">
         <v>286000</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="L14" s="3">
+      <c r="L14" s="28">
         <v>1070000</v>
       </c>
       <c r="M14" s="2" t="s">
@@ -3552,73 +3578,73 @@
       <c r="Q14" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="R14" s="3">
+      <c r="R14" s="28">
         <v>640000</v>
       </c>
       <c r="S14" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="T14" s="3">
+      <c r="T14" s="28">
         <v>249000</v>
       </c>
       <c r="U14" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="V14" s="3">
+      <c r="V14" s="28">
         <v>372000</v>
       </c>
       <c r="W14" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="X14" s="3">
+      <c r="X14" s="28">
         <v>89000</v>
       </c>
       <c r="Y14" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="Z14" s="3">
+      <c r="Z14" s="28">
         <v>247000</v>
       </c>
       <c r="AA14" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="AB14" s="3">
+      <c r="AB14" s="28">
         <v>500000</v>
       </c>
       <c r="AC14" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="AD14" s="3">
+      <c r="AD14" s="28">
         <v>210000</v>
       </c>
     </row>
     <row r="15" spans="1:30">
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="D15" s="12"/>
+      <c r="D15" s="10"/>
       <c r="E15" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="28">
         <v>214000</v>
       </c>
-      <c r="G15" s="29" t="s">
+      <c r="G15" s="14" t="s">
         <v>210</v>
       </c>
-      <c r="H15" s="30">
+      <c r="H15" s="37">
         <v>358000</v>
       </c>
-      <c r="I15" s="15" t="s">
+      <c r="I15" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="J15" s="16">
+      <c r="J15" s="50">
         <v>334000</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="L15" s="3">
+      <c r="L15" s="28">
         <v>1280000</v>
       </c>
       <c r="M15" s="2" t="s">
@@ -3627,67 +3653,67 @@
       <c r="Q15" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="R15" s="3">
+      <c r="R15" s="28">
         <v>800000</v>
       </c>
       <c r="S15" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="T15" s="3">
+      <c r="T15" s="28">
         <v>287000</v>
       </c>
       <c r="U15" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="V15" s="3">
+      <c r="V15" s="28">
         <v>392000</v>
       </c>
       <c r="W15" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="X15" s="3">
+      <c r="X15" s="28">
         <v>35000</v>
       </c>
       <c r="AA15" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="AB15" s="3">
+      <c r="AB15" s="28">
         <v>385000</v>
       </c>
       <c r="AC15" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="AD15" s="3">
+      <c r="AD15" s="28">
         <v>30000</v>
       </c>
     </row>
     <row r="16" spans="1:30">
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="D16" s="12"/>
+      <c r="D16" s="10"/>
       <c r="E16" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="28">
         <v>266000</v>
       </c>
-      <c r="G16" s="29" t="s">
+      <c r="G16" s="14" t="s">
         <v>222</v>
       </c>
-      <c r="H16" s="30">
+      <c r="H16" s="37">
         <v>442000</v>
       </c>
-      <c r="I16" s="15" t="s">
+      <c r="I16" s="11" t="s">
         <v>223</v>
       </c>
-      <c r="J16" s="17">
+      <c r="J16" s="51">
         <v>269000</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="L16" s="3">
+      <c r="L16" s="28">
         <v>1365000</v>
       </c>
       <c r="M16" s="2" t="s">
@@ -3696,67 +3722,67 @@
       <c r="Q16" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="R16" s="3">
+      <c r="R16" s="28">
         <v>880000</v>
       </c>
       <c r="S16" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="T16" s="3">
+      <c r="T16" s="28">
         <v>299000</v>
       </c>
       <c r="U16" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="V16" s="3">
+      <c r="V16" s="28">
         <v>662000</v>
       </c>
       <c r="W16" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="X16" s="3">
+      <c r="X16" s="28">
         <v>29000</v>
       </c>
       <c r="AA16" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="AB16" s="3">
+      <c r="AB16" s="28">
         <v>17000</v>
       </c>
       <c r="AC16" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="AD16" s="3">
+      <c r="AD16" s="28">
         <v>38000</v>
       </c>
     </row>
     <row r="17" spans="3:30">
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="D17" s="12"/>
+      <c r="D17" s="10"/>
       <c r="E17" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="F17" s="3">
+      <c r="F17" s="28">
         <v>235000</v>
       </c>
-      <c r="G17" s="29" t="s">
+      <c r="G17" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="H17" s="30">
+      <c r="H17" s="37">
         <v>374000</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="J17" s="13">
+      <c r="J17" s="48">
         <v>312000</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="L17" s="3">
+      <c r="L17" s="28">
         <v>1385000</v>
       </c>
       <c r="M17" s="2" t="s">
@@ -3765,67 +3791,67 @@
       <c r="Q17" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="R17" s="3">
+      <c r="R17" s="28">
         <v>950000</v>
       </c>
       <c r="S17" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="T17" s="3">
+      <c r="T17" s="28">
         <v>371000</v>
       </c>
       <c r="U17" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="V17" s="3">
+      <c r="V17" s="28">
         <v>662000</v>
       </c>
       <c r="W17" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="X17" s="3">
+      <c r="X17" s="28">
         <v>33000</v>
       </c>
       <c r="AA17" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="AB17" s="3">
+      <c r="AB17" s="28">
         <v>17000</v>
       </c>
       <c r="AC17" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="AD17" s="3">
+      <c r="AD17" s="28">
         <v>1120000</v>
       </c>
     </row>
     <row r="18" spans="3:30">
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="D18" s="12"/>
+      <c r="D18" s="10"/>
       <c r="E18" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="28">
         <v>293000</v>
       </c>
-      <c r="G18" s="29" t="s">
+      <c r="G18" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="H18" s="30">
+      <c r="H18" s="37">
         <v>374000</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="J18" s="31">
+      <c r="J18" s="56">
         <v>375000</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="L18" s="3">
+      <c r="L18" s="28">
         <v>1610000</v>
       </c>
       <c r="M18" s="2" t="s">
@@ -3834,67 +3860,67 @@
       <c r="Q18" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="R18" s="3">
+      <c r="R18" s="28">
         <v>1290000</v>
       </c>
       <c r="S18" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="T18" s="3">
+      <c r="T18" s="28">
         <v>243000</v>
       </c>
       <c r="U18" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="V18" s="3">
+      <c r="V18" s="28">
         <v>272000</v>
       </c>
       <c r="W18" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="X18" s="3">
+      <c r="X18" s="28">
         <v>47000</v>
       </c>
       <c r="AA18" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="AB18" s="3">
+      <c r="AB18" s="28">
         <v>29000</v>
       </c>
       <c r="AC18" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="AD18" s="3">
+      <c r="AD18" s="28">
         <v>1120000</v>
       </c>
     </row>
     <row r="19" spans="3:30">
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="D19" s="12"/>
+      <c r="D19" s="10"/>
       <c r="E19" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="28">
         <v>267000</v>
       </c>
-      <c r="G19" s="29" t="s">
+      <c r="G19" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="H19" s="30">
+      <c r="H19" s="37">
         <v>298000</v>
       </c>
-      <c r="I19" s="22" t="s">
+      <c r="I19" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="J19" s="24">
+      <c r="J19" s="53">
         <v>317000</v>
       </c>
       <c r="K19" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="L19" s="3">
+      <c r="L19" s="28">
         <v>1234000</v>
       </c>
       <c r="M19" s="2" t="s">
@@ -3903,67 +3929,67 @@
       <c r="Q19" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="R19" s="3">
+      <c r="R19" s="28">
         <v>1250000</v>
       </c>
       <c r="S19" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="T19" s="3">
+      <c r="T19" s="28">
         <v>287000</v>
       </c>
       <c r="U19" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="V19" s="3">
+      <c r="V19" s="28">
         <v>390000</v>
       </c>
       <c r="W19" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="X19" s="3">
+      <c r="X19" s="28">
         <v>45000</v>
       </c>
       <c r="AA19" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="AB19" s="3">
+      <c r="AB19" s="28">
         <v>34000</v>
       </c>
       <c r="AC19" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="AD19" s="3">
+      <c r="AD19" s="28">
         <v>1220000</v>
       </c>
     </row>
     <row r="20" spans="3:30">
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="D20" s="12"/>
+      <c r="D20" s="10"/>
       <c r="E20" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="28">
         <v>340000</v>
       </c>
-      <c r="G20" s="29" t="s">
+      <c r="G20" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="H20" s="30">
+      <c r="H20" s="37">
         <v>366000</v>
       </c>
-      <c r="I20" s="32" t="s">
+      <c r="I20" s="15" t="s">
         <v>271</v>
       </c>
-      <c r="J20" s="33">
+      <c r="J20" s="57">
         <v>417000</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="L20" s="3">
+      <c r="L20" s="28">
         <v>1510000</v>
       </c>
       <c r="M20" s="2" t="s">
@@ -3972,25 +3998,25 @@
       <c r="Q20" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="R20" s="3">
+      <c r="R20" s="28">
         <v>830000</v>
       </c>
       <c r="S20" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="T20" s="19">
+      <c r="T20" s="33">
         <v>431000</v>
       </c>
       <c r="U20" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="V20" s="3">
+      <c r="V20" s="28">
         <v>430000</v>
       </c>
       <c r="W20" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="X20" s="3">
+      <c r="X20" s="28">
         <v>50000</v>
       </c>
       <c r="Y20" s="2" t="s">
@@ -3999,43 +4025,43 @@
       <c r="AA20" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="AB20" s="3">
+      <c r="AB20" s="28">
         <v>60000</v>
       </c>
       <c r="AC20" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="AD20" s="3">
+      <c r="AD20" s="28">
         <v>1220000</v>
       </c>
     </row>
     <row r="21" spans="3:30">
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="9" t="s">
         <v>280</v>
       </c>
-      <c r="D21" s="12"/>
+      <c r="D21" s="10"/>
       <c r="E21" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="28">
         <v>411000</v>
       </c>
-      <c r="G21" s="29" t="s">
+      <c r="G21" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="H21" s="30">
+      <c r="H21" s="37">
         <v>330000</v>
       </c>
-      <c r="I21" s="32" t="s">
+      <c r="I21" s="15" t="s">
         <v>283</v>
       </c>
-      <c r="J21" s="34">
+      <c r="J21" s="58">
         <v>373000</v>
       </c>
       <c r="K21" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="L21" s="3">
+      <c r="L21" s="28">
         <v>1350000</v>
       </c>
       <c r="M21" s="2" t="s">
@@ -4044,55 +4070,55 @@
       <c r="S21" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="T21" s="3">
+      <c r="T21" s="28">
         <v>495000</v>
       </c>
       <c r="W21" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="X21" s="3">
+      <c r="X21" s="28">
         <v>20000</v>
       </c>
       <c r="AA21" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="AB21" s="3">
+      <c r="AB21" s="28">
         <v>104000</v>
       </c>
       <c r="AC21" s="2" t="s">
         <v>505</v>
       </c>
-      <c r="AD21" s="75">
+      <c r="AD21" s="28">
         <v>350000</v>
       </c>
     </row>
     <row r="22" spans="3:30">
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="9" t="s">
         <v>289</v>
       </c>
-      <c r="D22" s="12"/>
+      <c r="D22" s="10"/>
       <c r="E22" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="F22" s="3">
+      <c r="F22" s="28">
         <v>320000</v>
       </c>
-      <c r="G22" s="29" t="s">
+      <c r="G22" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="H22" s="30">
+      <c r="H22" s="37">
         <v>340000</v>
       </c>
-      <c r="I22" s="32" t="s">
+      <c r="I22" s="15" t="s">
         <v>292</v>
       </c>
-      <c r="J22" s="35">
+      <c r="J22" s="59">
         <v>467000</v>
       </c>
       <c r="K22" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="L22" s="3" t="s">
+      <c r="L22" s="28" t="s">
         <v>294</v>
       </c>
       <c r="M22" s="2" t="s">
@@ -4101,49 +4127,49 @@
       <c r="S22" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="T22" s="3">
+      <c r="T22" s="28">
         <v>257000</v>
       </c>
       <c r="AA22" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="AB22" s="3">
+      <c r="AB22" s="28">
         <v>91000</v>
       </c>
       <c r="AC22" s="2" t="s">
         <v>506</v>
       </c>
-      <c r="AD22" s="75">
+      <c r="AD22" s="28">
         <v>480000</v>
       </c>
     </row>
     <row r="23" spans="3:30">
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="9" t="s">
         <v>298</v>
       </c>
-      <c r="D23" s="12"/>
+      <c r="D23" s="10"/>
       <c r="E23" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="F23" s="3">
+      <c r="F23" s="28">
         <v>345000</v>
       </c>
-      <c r="G23" s="29" t="s">
+      <c r="G23" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="H23" s="30">
+      <c r="H23" s="37">
         <v>360000</v>
       </c>
-      <c r="I23" s="36" t="s">
+      <c r="I23" s="16" t="s">
         <v>301</v>
       </c>
-      <c r="J23" s="37">
+      <c r="J23" s="60">
         <v>299000</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="L23" s="3">
+      <c r="L23" s="28">
         <v>472000</v>
       </c>
       <c r="M23" s="2" t="s">
@@ -4152,43 +4178,49 @@
       <c r="S23" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="T23" s="3">
+      <c r="T23" s="28">
         <v>299000</v>
       </c>
       <c r="AA23" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="AB23" s="3">
+      <c r="AB23" s="28">
         <v>25000</v>
       </c>
+      <c r="AC23" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="AD23" s="28">
+        <v>380000</v>
+      </c>
     </row>
     <row r="24" spans="3:30">
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="9" t="s">
         <v>306</v>
       </c>
-      <c r="D24" s="12"/>
-      <c r="E24" s="20" t="s">
+      <c r="D24" s="10"/>
+      <c r="E24" s="12" t="s">
         <v>307</v>
       </c>
-      <c r="F24" s="25">
+      <c r="F24" s="36">
         <v>309000</v>
       </c>
-      <c r="G24" s="38" t="s">
+      <c r="G24" s="17" t="s">
         <v>308</v>
       </c>
-      <c r="H24" s="39">
+      <c r="H24" s="38">
         <v>269000</v>
       </c>
-      <c r="I24" s="36" t="s">
+      <c r="I24" s="16" t="s">
         <v>309</v>
       </c>
-      <c r="J24" s="40">
+      <c r="J24" s="61">
         <v>321000</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="L24" s="3">
+      <c r="L24" s="28">
         <v>518000</v>
       </c>
       <c r="M24" s="2" t="s">
@@ -4197,43 +4229,49 @@
       <c r="S24" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="T24" s="3">
+      <c r="T24" s="28">
         <v>344000</v>
       </c>
       <c r="AA24" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="AB24" s="3">
+      <c r="AB24" s="28">
         <v>30000</v>
       </c>
+      <c r="AC24" s="31" t="s">
+        <v>508</v>
+      </c>
+      <c r="AD24" s="28">
+        <v>330000</v>
+      </c>
     </row>
     <row r="25" spans="3:30">
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="9" t="s">
         <v>314</v>
       </c>
-      <c r="D25" s="12"/>
-      <c r="E25" s="20" t="s">
+      <c r="D25" s="10"/>
+      <c r="E25" s="12" t="s">
         <v>315</v>
       </c>
-      <c r="F25" s="25">
+      <c r="F25" s="36">
         <v>369000</v>
       </c>
-      <c r="G25" s="29" t="s">
+      <c r="G25" s="14" t="s">
         <v>316</v>
       </c>
-      <c r="H25" s="30">
+      <c r="H25" s="37">
         <v>396000</v>
       </c>
-      <c r="I25" s="41" t="s">
+      <c r="I25" s="18" t="s">
         <v>317</v>
       </c>
-      <c r="J25" s="42">
+      <c r="J25" s="62">
         <v>329000</v>
       </c>
       <c r="K25" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="L25" s="3">
+      <c r="L25" s="28">
         <v>603000</v>
       </c>
       <c r="M25" s="2" t="s">
@@ -4242,43 +4280,49 @@
       <c r="S25" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="T25" s="3">
+      <c r="T25" s="28">
         <v>489000</v>
       </c>
       <c r="AA25" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="AB25" s="3">
+      <c r="AB25" s="28">
         <v>17000</v>
+      </c>
+      <c r="AC25" s="31" t="s">
+        <v>509</v>
+      </c>
+      <c r="AD25" s="28">
+        <v>380000</v>
       </c>
     </row>
     <row r="26" spans="3:30">
       <c r="C26" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="D26" s="12"/>
-      <c r="E26" s="20" t="s">
+      <c r="D26" s="10"/>
+      <c r="E26" s="12" t="s">
         <v>323</v>
       </c>
-      <c r="F26" s="25">
+      <c r="F26" s="36">
         <v>372000</v>
       </c>
-      <c r="G26" s="29" t="s">
+      <c r="G26" s="14" t="s">
         <v>324</v>
       </c>
-      <c r="H26" s="30">
+      <c r="H26" s="37">
         <v>441000</v>
       </c>
-      <c r="I26" s="41" t="s">
+      <c r="I26" s="18" t="s">
         <v>325</v>
       </c>
-      <c r="J26" s="43">
+      <c r="J26" s="63">
         <v>349000</v>
       </c>
       <c r="K26" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="L26" s="3">
+      <c r="L26" s="28">
         <v>670000</v>
       </c>
       <c r="M26" s="2" t="s">
@@ -4287,37 +4331,37 @@
       <c r="S26" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="T26" s="3">
+      <c r="T26" s="28">
         <v>453000</v>
       </c>
     </row>
     <row r="27" spans="3:30">
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="9" t="s">
         <v>329</v>
       </c>
-      <c r="D27" s="12"/>
-      <c r="E27" s="20" t="s">
+      <c r="D27" s="10"/>
+      <c r="E27" s="12" t="s">
         <v>330</v>
       </c>
-      <c r="F27" s="25">
+      <c r="F27" s="36">
         <v>425000</v>
       </c>
-      <c r="G27" s="29" t="s">
+      <c r="G27" s="14" t="s">
         <v>331</v>
       </c>
-      <c r="H27" s="30">
+      <c r="H27" s="37">
         <v>697000</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="J27" s="44">
+      <c r="J27" s="64">
         <v>280000</v>
       </c>
       <c r="K27" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="L27" s="3">
+      <c r="L27" s="28">
         <v>440000</v>
       </c>
       <c r="M27" s="2" t="s">
@@ -4328,29 +4372,29 @@
       <c r="C28" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="D28" s="12"/>
-      <c r="E28" s="20" t="s">
+      <c r="D28" s="10"/>
+      <c r="E28" s="12" t="s">
         <v>336</v>
       </c>
-      <c r="F28" s="25">
+      <c r="F28" s="36">
         <v>522000</v>
       </c>
-      <c r="G28" s="29" t="s">
+      <c r="G28" s="14" t="s">
         <v>337</v>
       </c>
-      <c r="H28" s="30">
+      <c r="H28" s="37">
         <v>494000</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="J28" s="45">
+      <c r="J28" s="65">
         <v>426000</v>
       </c>
       <c r="K28" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="L28" s="3">
+      <c r="L28" s="28">
         <v>536000</v>
       </c>
       <c r="M28" s="2" t="s">
@@ -4358,32 +4402,32 @@
       </c>
     </row>
     <row r="29" spans="3:30">
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="9" t="s">
         <v>341</v>
       </c>
-      <c r="D29" s="12"/>
-      <c r="E29" s="29" t="s">
+      <c r="D29" s="10"/>
+      <c r="E29" s="14" t="s">
         <v>342</v>
       </c>
-      <c r="F29" s="30">
+      <c r="F29" s="37">
         <v>398000</v>
       </c>
-      <c r="G29" s="29" t="s">
+      <c r="G29" s="14" t="s">
         <v>343</v>
       </c>
-      <c r="H29" s="30">
+      <c r="H29" s="37">
         <v>173000</v>
       </c>
-      <c r="I29" s="20" t="s">
+      <c r="I29" s="12" t="s">
         <v>344</v>
       </c>
-      <c r="J29" s="46">
+      <c r="J29" s="66">
         <v>207000</v>
       </c>
       <c r="K29" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="L29" s="3">
+      <c r="L29" s="28">
         <v>675000</v>
       </c>
       <c r="M29" s="2" t="s">
@@ -4394,29 +4438,29 @@
       <c r="C30" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="D30" s="12"/>
-      <c r="E30" s="29" t="s">
+      <c r="D30" s="10"/>
+      <c r="E30" s="14" t="s">
         <v>348</v>
       </c>
-      <c r="F30" s="30">
+      <c r="F30" s="37">
         <v>777000</v>
       </c>
-      <c r="G30" s="29" t="s">
+      <c r="G30" s="14" t="s">
         <v>349</v>
       </c>
-      <c r="H30" s="30">
+      <c r="H30" s="37">
         <v>207000</v>
       </c>
-      <c r="I30" s="20" t="s">
+      <c r="I30" s="12" t="s">
         <v>350</v>
       </c>
-      <c r="J30" s="46">
+      <c r="J30" s="66">
         <v>257000</v>
       </c>
       <c r="K30" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="L30" s="3">
+      <c r="L30" s="28">
         <v>486000</v>
       </c>
       <c r="M30" s="2" t="s">
@@ -4427,29 +4471,29 @@
       <c r="C31" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="D31" s="12"/>
-      <c r="E31" s="47" t="s">
+      <c r="D31" s="10"/>
+      <c r="E31" s="19" t="s">
         <v>354</v>
       </c>
-      <c r="F31" s="48">
+      <c r="F31" s="39">
         <v>341000</v>
       </c>
-      <c r="G31" s="29" t="s">
+      <c r="G31" s="14" t="s">
         <v>355</v>
       </c>
-      <c r="H31" s="30">
+      <c r="H31" s="37">
         <v>302000</v>
       </c>
-      <c r="I31" s="49" t="s">
+      <c r="I31" s="20" t="s">
         <v>356</v>
       </c>
-      <c r="J31" s="50">
+      <c r="J31" s="67">
         <v>295000</v>
       </c>
       <c r="K31" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="L31" s="3">
+      <c r="L31" s="28">
         <v>590000</v>
       </c>
       <c r="M31" s="2" t="s">
@@ -4460,29 +4504,29 @@
       <c r="C32" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="D32" s="12"/>
-      <c r="E32" s="47" t="s">
+      <c r="D32" s="10"/>
+      <c r="E32" s="19" t="s">
         <v>360</v>
       </c>
-      <c r="F32" s="48">
+      <c r="F32" s="39">
         <v>388000</v>
       </c>
-      <c r="G32" s="38" t="s">
+      <c r="G32" s="17" t="s">
         <v>361</v>
       </c>
-      <c r="H32" s="39">
+      <c r="H32" s="38">
         <v>381000</v>
       </c>
-      <c r="I32" s="49" t="s">
+      <c r="I32" s="20" t="s">
         <v>362</v>
       </c>
-      <c r="J32" s="50">
+      <c r="J32" s="67">
         <v>405000</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="L32" s="3">
+      <c r="L32" s="28">
         <v>747000</v>
       </c>
       <c r="M32" s="2" t="s">
@@ -4493,29 +4537,29 @@
       <c r="C33" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="D33" s="51"/>
-      <c r="E33" s="29" t="s">
+      <c r="D33" s="21"/>
+      <c r="E33" s="14" t="s">
         <v>366</v>
       </c>
-      <c r="F33" s="30">
+      <c r="F33" s="37">
         <v>648000</v>
       </c>
-      <c r="G33" s="29" t="s">
+      <c r="G33" s="14" t="s">
         <v>367</v>
       </c>
-      <c r="H33" s="48">
+      <c r="H33" s="39">
         <v>388000</v>
       </c>
-      <c r="I33" s="29" t="s">
+      <c r="I33" s="14" t="s">
         <v>368</v>
       </c>
-      <c r="J33" s="52">
+      <c r="J33" s="68">
         <v>641000</v>
       </c>
       <c r="K33" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="L33" s="3">
+      <c r="L33" s="28">
         <v>586000</v>
       </c>
       <c r="M33" s="2" t="s">
@@ -4523,31 +4567,31 @@
       </c>
     </row>
     <row r="34" spans="3:13">
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="9" t="s">
         <v>371</v>
       </c>
-      <c r="E34" s="29" t="s">
+      <c r="E34" s="14" t="s">
         <v>372</v>
       </c>
-      <c r="F34" s="30">
+      <c r="F34" s="37">
         <v>793000</v>
       </c>
-      <c r="G34" s="29" t="s">
+      <c r="G34" s="14" t="s">
         <v>373</v>
       </c>
-      <c r="H34" s="48">
+      <c r="H34" s="39">
         <v>413000</v>
       </c>
-      <c r="I34" s="29" t="s">
+      <c r="I34" s="14" t="s">
         <v>374</v>
       </c>
-      <c r="J34" s="53">
+      <c r="J34" s="69">
         <v>754000</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="L34" s="3">
+      <c r="L34" s="28">
         <v>603000</v>
       </c>
       <c r="M34" s="2" t="s">
@@ -4558,28 +4602,28 @@
       <c r="C35" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="E35" s="29" t="s">
+      <c r="E35" s="14" t="s">
         <v>378</v>
       </c>
-      <c r="F35" s="54">
+      <c r="F35" s="44">
         <v>747000</v>
       </c>
-      <c r="G35" s="29" t="s">
+      <c r="G35" s="14" t="s">
         <v>379</v>
       </c>
-      <c r="H35" s="30">
+      <c r="H35" s="37">
         <v>309000</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="J35" s="55">
+      <c r="J35" s="70">
         <v>312000</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="L35" s="3">
+      <c r="L35" s="28">
         <v>620000</v>
       </c>
       <c r="M35" s="2" t="s">
@@ -4590,28 +4634,28 @@
       <c r="C36" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="E36" s="29" t="s">
+      <c r="E36" s="14" t="s">
         <v>384</v>
       </c>
-      <c r="F36" s="54">
+      <c r="F36" s="44">
         <v>882000</v>
       </c>
-      <c r="G36" s="29" t="s">
+      <c r="G36" s="14" t="s">
         <v>385</v>
       </c>
-      <c r="H36" s="30">
+      <c r="H36" s="37">
         <v>411000</v>
       </c>
-      <c r="I36" s="15" t="s">
+      <c r="I36" s="11" t="s">
         <v>386</v>
       </c>
-      <c r="J36" s="55">
+      <c r="J36" s="70">
         <v>381000</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="L36" s="3">
+      <c r="L36" s="28">
         <v>1460000</v>
       </c>
       <c r="M36" s="2" t="s">
@@ -4619,146 +4663,146 @@
       </c>
     </row>
     <row r="37" spans="3:13">
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="9" t="s">
         <v>389</v>
       </c>
-      <c r="E37" s="29" t="s">
+      <c r="E37" s="14" t="s">
         <v>390</v>
       </c>
-      <c r="F37" s="30">
+      <c r="F37" s="37">
         <v>356000</v>
       </c>
-      <c r="G37" s="29" t="s">
+      <c r="G37" s="14" t="s">
         <v>391</v>
       </c>
-      <c r="H37" s="30">
+      <c r="H37" s="37">
         <v>473000</v>
       </c>
-      <c r="I37" s="22" t="s">
+      <c r="I37" s="13" t="s">
         <v>392</v>
       </c>
-      <c r="J37" s="56">
+      <c r="J37" s="71">
         <v>365000</v>
       </c>
       <c r="K37" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="L37" s="3">
+      <c r="L37" s="28">
         <v>1685000</v>
       </c>
     </row>
     <row r="38" spans="3:13">
-      <c r="C38" s="11" t="s">
+      <c r="C38" s="9" t="s">
         <v>394</v>
       </c>
-      <c r="E38" s="29" t="s">
+      <c r="E38" s="14" t="s">
         <v>395</v>
       </c>
-      <c r="F38" s="30">
+      <c r="F38" s="37">
         <v>369000</v>
       </c>
-      <c r="G38" s="29" t="s">
+      <c r="G38" s="14" t="s">
         <v>396</v>
       </c>
-      <c r="H38" s="30">
+      <c r="H38" s="37">
         <v>329000</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="J38" s="57">
+      <c r="J38" s="72">
         <v>501000</v>
       </c>
     </row>
     <row r="39" spans="3:13">
-      <c r="C39" s="11" t="s">
+      <c r="C39" s="9" t="s">
         <v>398</v>
       </c>
-      <c r="E39" s="29" t="s">
+      <c r="E39" s="14" t="s">
         <v>399</v>
       </c>
-      <c r="F39" s="30">
+      <c r="F39" s="37">
         <v>465000</v>
       </c>
-      <c r="G39" s="29" t="s">
+      <c r="G39" s="14" t="s">
         <v>400</v>
       </c>
-      <c r="H39" s="30">
+      <c r="H39" s="37">
         <v>385000</v>
       </c>
-      <c r="I39" s="29" t="s">
+      <c r="I39" s="14" t="s">
         <v>401</v>
       </c>
-      <c r="J39" s="58">
+      <c r="J39" s="73">
         <v>740000</v>
       </c>
     </row>
     <row r="40" spans="3:13">
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="9" t="s">
         <v>402</v>
       </c>
-      <c r="E40" s="29" t="s">
+      <c r="E40" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="F40" s="30">
+      <c r="F40" s="37">
         <v>543000</v>
       </c>
-      <c r="G40" s="29" t="s">
+      <c r="G40" s="14" t="s">
         <v>404</v>
       </c>
-      <c r="H40" s="30">
+      <c r="H40" s="37">
         <v>437000</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="J40" s="59">
+      <c r="J40" s="74">
         <v>278000</v>
       </c>
     </row>
     <row r="41" spans="3:13">
-      <c r="C41" s="11" t="s">
+      <c r="C41" s="9" t="s">
         <v>406</v>
       </c>
-      <c r="E41" s="29" t="s">
+      <c r="E41" s="14" t="s">
         <v>407</v>
       </c>
-      <c r="F41" s="30">
+      <c r="F41" s="37">
         <v>778000</v>
       </c>
-      <c r="G41" s="29" t="s">
+      <c r="G41" s="14" t="s">
         <v>408</v>
       </c>
-      <c r="H41" s="30">
+      <c r="H41" s="37">
         <v>566000</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="J41" s="31">
+      <c r="J41" s="56">
         <v>351000</v>
       </c>
     </row>
     <row r="42" spans="3:13">
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="9" t="s">
         <v>410</v>
       </c>
-      <c r="E42" s="29" t="s">
+      <c r="E42" s="14" t="s">
         <v>411</v>
       </c>
-      <c r="F42" s="30">
+      <c r="F42" s="37">
         <v>337000</v>
       </c>
-      <c r="G42" s="29" t="s">
+      <c r="G42" s="14" t="s">
         <v>412</v>
       </c>
-      <c r="H42" s="30">
+      <c r="H42" s="37">
         <v>636000</v>
       </c>
-      <c r="I42" s="20" t="s">
+      <c r="I42" s="12" t="s">
         <v>413</v>
       </c>
-      <c r="J42" s="60">
+      <c r="J42" s="75">
         <v>300000</v>
       </c>
     </row>
@@ -4766,22 +4810,22 @@
       <c r="C43" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E43" s="29" t="s">
+      <c r="E43" s="14" t="s">
         <v>415</v>
       </c>
-      <c r="F43" s="54">
+      <c r="F43" s="44">
         <v>440000</v>
       </c>
-      <c r="G43" s="29" t="s">
+      <c r="G43" s="14" t="s">
         <v>416</v>
       </c>
-      <c r="H43" s="30">
+      <c r="H43" s="37">
         <v>707000</v>
       </c>
-      <c r="I43" s="20" t="s">
+      <c r="I43" s="12" t="s">
         <v>417</v>
       </c>
-      <c r="J43" s="61">
+      <c r="J43" s="76">
         <v>322000</v>
       </c>
     </row>
@@ -4792,19 +4836,19 @@
       <c r="E44" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="F44" s="3">
+      <c r="F44" s="28">
         <v>335000</v>
       </c>
-      <c r="G44" s="29" t="s">
+      <c r="G44" s="14" t="s">
         <v>420</v>
       </c>
-      <c r="H44" s="30">
+      <c r="H44" s="37">
         <v>420000</v>
       </c>
-      <c r="I44" s="62" t="s">
+      <c r="I44" s="22" t="s">
         <v>421</v>
       </c>
-      <c r="J44" s="63">
+      <c r="J44" s="77">
         <v>329000</v>
       </c>
     </row>
@@ -4815,19 +4859,19 @@
       <c r="E45" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="F45" s="3">
+      <c r="F45" s="28">
         <v>448000</v>
       </c>
-      <c r="G45" s="29" t="s">
+      <c r="G45" s="14" t="s">
         <v>424</v>
       </c>
-      <c r="H45" s="30">
+      <c r="H45" s="37">
         <v>430000</v>
       </c>
-      <c r="I45" s="62" t="s">
+      <c r="I45" s="22" t="s">
         <v>425</v>
       </c>
-      <c r="J45" s="63">
+      <c r="J45" s="77">
         <v>445000</v>
       </c>
     </row>
@@ -4838,17 +4882,17 @@
       <c r="E46" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="F46" s="3">
+      <c r="F46" s="28">
         <v>402000</v>
       </c>
-      <c r="G46" s="29" t="s">
+      <c r="G46" s="14" t="s">
         <v>428</v>
       </c>
-      <c r="H46" s="30">
+      <c r="H46" s="37">
         <v>400000</v>
       </c>
-      <c r="I46" s="62"/>
-      <c r="J46" s="63"/>
+      <c r="I46" s="22"/>
+      <c r="J46" s="77"/>
     </row>
     <row r="47" spans="3:13">
       <c r="C47" s="2" t="s">
@@ -4857,58 +4901,58 @@
       <c r="E47" s="2" t="s">
         <v>430</v>
       </c>
-      <c r="F47" s="3">
+      <c r="F47" s="28">
         <v>469000</v>
       </c>
-      <c r="G47" s="29" t="s">
+      <c r="G47" s="14" t="s">
         <v>431</v>
       </c>
-      <c r="H47" s="30">
+      <c r="H47" s="37">
         <v>382000</v>
       </c>
     </row>
     <row r="48" spans="3:13">
-      <c r="C48" s="11" t="s">
+      <c r="C48" s="9" t="s">
         <v>432</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="F48" s="3">
+      <c r="F48" s="28">
         <v>537000</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="H48" s="3">
+      <c r="H48" s="28">
         <v>443000</v>
       </c>
     </row>
     <row r="49" spans="5:8">
-      <c r="E49" s="20" t="s">
+      <c r="E49" s="12" t="s">
         <v>435</v>
       </c>
-      <c r="F49" s="25">
+      <c r="F49" s="36">
         <v>180000</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="H49" s="3">
+      <c r="H49" s="28">
         <v>488000</v>
       </c>
     </row>
     <row r="50" spans="5:8">
-      <c r="E50" s="20" t="s">
+      <c r="E50" s="12" t="s">
         <v>437</v>
       </c>
-      <c r="F50" s="25">
+      <c r="F50" s="36">
         <v>230000</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="H50" s="3">
+      <c r="H50" s="28">
         <v>548000</v>
       </c>
     </row>
@@ -4916,13 +4960,13 @@
       <c r="E51" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="F51" s="3">
+      <c r="F51" s="28">
         <v>46000</v>
       </c>
-      <c r="G51" s="29" t="s">
+      <c r="G51" s="14" t="s">
         <v>440</v>
       </c>
-      <c r="H51" s="30">
+      <c r="H51" s="37">
         <v>446000</v>
       </c>
     </row>
@@ -4930,13 +4974,13 @@
       <c r="E52" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="F52" s="3">
+      <c r="F52" s="28">
         <v>48000</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="H52" s="3">
+      <c r="H52" s="28">
         <v>431000</v>
       </c>
     </row>
@@ -4944,13 +4988,13 @@
       <c r="E53" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="F53" s="3">
+      <c r="F53" s="28">
         <v>55000</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="H53" s="3">
+      <c r="H53" s="28">
         <v>483000</v>
       </c>
     </row>
@@ -4958,13 +5002,13 @@
       <c r="E54" s="2" t="s">
         <v>445</v>
       </c>
-      <c r="F54" s="3">
+      <c r="F54" s="28">
         <v>56000</v>
       </c>
       <c r="G54" s="2" t="s">
         <v>446</v>
       </c>
-      <c r="H54" s="3">
+      <c r="H54" s="28">
         <v>541000</v>
       </c>
     </row>
@@ -4972,13 +5016,13 @@
       <c r="E55" s="2" t="s">
         <v>447</v>
       </c>
-      <c r="F55" s="3">
+      <c r="F55" s="28">
         <v>56000</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>448</v>
       </c>
-      <c r="H55" s="3">
+      <c r="H55" s="28">
         <v>478000</v>
       </c>
     </row>
@@ -4986,13 +5030,13 @@
       <c r="E56" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="F56" s="3">
+      <c r="F56" s="28">
         <v>59000</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="H56" s="3">
+      <c r="H56" s="28">
         <v>589000</v>
       </c>
     </row>
@@ -5000,13 +5044,13 @@
       <c r="E57" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="F57" s="3">
+      <c r="F57" s="28">
         <v>60000</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>452</v>
       </c>
-      <c r="H57" s="3">
+      <c r="H57" s="28">
         <v>637000</v>
       </c>
     </row>
@@ -5014,13 +5058,13 @@
       <c r="E58" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="F58" s="3">
+      <c r="F58" s="28">
         <v>358000</v>
       </c>
-      <c r="G58" s="29" t="s">
+      <c r="G58" s="14" t="s">
         <v>454</v>
       </c>
-      <c r="H58" s="30">
+      <c r="H58" s="37">
         <v>541000</v>
       </c>
     </row>
@@ -5028,45 +5072,45 @@
       <c r="E59" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="F59" s="3">
+      <c r="F59" s="28">
         <v>320000</v>
       </c>
-      <c r="G59" s="47" t="s">
+      <c r="G59" s="19" t="s">
         <v>456</v>
       </c>
-      <c r="H59" s="48">
+      <c r="H59" s="39">
         <v>515000</v>
       </c>
     </row>
     <row r="60" spans="5:8">
-      <c r="G60" s="64" t="s">
+      <c r="G60" s="23" t="s">
         <v>457</v>
       </c>
-      <c r="H60" s="65">
+      <c r="H60" s="40">
         <v>701000</v>
       </c>
     </row>
     <row r="61" spans="5:8">
-      <c r="G61" s="64" t="s">
+      <c r="G61" s="23" t="s">
         <v>458</v>
       </c>
-      <c r="H61" s="65">
+      <c r="H61" s="40">
         <v>794000</v>
       </c>
     </row>
     <row r="62" spans="5:8">
-      <c r="G62" s="38" t="s">
+      <c r="G62" s="17" t="s">
         <v>459</v>
       </c>
-      <c r="H62" s="39">
+      <c r="H62" s="38">
         <v>628000</v>
       </c>
     </row>
     <row r="63" spans="5:8">
-      <c r="G63" s="38" t="s">
+      <c r="G63" s="17" t="s">
         <v>460</v>
       </c>
-      <c r="H63" s="39">
+      <c r="H63" s="38">
         <v>747000</v>
       </c>
     </row>
@@ -5074,7 +5118,7 @@
       <c r="G64" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="H64" s="3">
+      <c r="H64" s="28">
         <v>563000</v>
       </c>
     </row>
@@ -5082,7 +5126,7 @@
       <c r="G65" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="H65" s="3">
+      <c r="H65" s="28">
         <v>682000</v>
       </c>
     </row>
@@ -5090,7 +5134,7 @@
       <c r="G66" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="H66" s="3">
+      <c r="H66" s="28">
         <v>647000</v>
       </c>
     </row>
@@ -5098,7 +5142,7 @@
       <c r="G67" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="H67" s="3">
+      <c r="H67" s="28">
         <v>511000</v>
       </c>
     </row>
@@ -5106,7 +5150,7 @@
       <c r="G68" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="H68" s="3">
+      <c r="H68" s="28">
         <v>503000</v>
       </c>
     </row>
@@ -5114,7 +5158,7 @@
       <c r="G69" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="H69" s="3">
+      <c r="H69" s="28">
         <v>802000</v>
       </c>
     </row>
@@ -5122,7 +5166,7 @@
       <c r="G70" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="H70" s="18">
+      <c r="H70" s="34">
         <v>903000</v>
       </c>
     </row>
@@ -5130,300 +5174,300 @@
       <c r="G71" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="H71" s="3">
+      <c r="H71" s="28">
         <v>823000</v>
       </c>
     </row>
     <row r="72" spans="7:8">
-      <c r="G72" s="49" t="s">
+      <c r="G72" s="20" t="s">
         <v>469</v>
       </c>
-      <c r="H72" s="66">
+      <c r="H72" s="41">
         <v>268000</v>
       </c>
     </row>
     <row r="73" spans="7:8">
-      <c r="G73" s="49" t="s">
+      <c r="G73" s="20" t="s">
         <v>470</v>
       </c>
-      <c r="H73" s="66">
+      <c r="H73" s="41">
         <v>325000</v>
       </c>
     </row>
     <row r="74" spans="7:8">
-      <c r="G74" s="67" t="s">
+      <c r="G74" s="24" t="s">
         <v>471</v>
       </c>
-      <c r="H74" s="66">
+      <c r="H74" s="41">
         <v>297000</v>
       </c>
     </row>
     <row r="75" spans="7:8">
-      <c r="G75" s="67" t="s">
+      <c r="G75" s="24" t="s">
         <v>472</v>
       </c>
-      <c r="H75" s="66">
+      <c r="H75" s="41">
         <v>359000</v>
       </c>
     </row>
     <row r="76" spans="7:8">
-      <c r="G76" s="29" t="s">
+      <c r="G76" s="14" t="s">
         <v>473</v>
       </c>
-      <c r="H76" s="30">
+      <c r="H76" s="37">
         <v>297000</v>
       </c>
     </row>
     <row r="77" spans="7:8">
-      <c r="G77" s="29" t="s">
+      <c r="G77" s="14" t="s">
         <v>474</v>
       </c>
-      <c r="H77" s="30">
+      <c r="H77" s="37">
         <v>394000</v>
       </c>
     </row>
     <row r="78" spans="7:8">
-      <c r="G78" s="68" t="s">
+      <c r="G78" s="25" t="s">
         <v>475</v>
       </c>
-      <c r="H78" s="18">
+      <c r="H78" s="34">
         <v>446000</v>
       </c>
     </row>
     <row r="79" spans="7:8">
-      <c r="G79" s="38" t="s">
+      <c r="G79" s="17" t="s">
         <v>476</v>
       </c>
-      <c r="H79" s="39">
+      <c r="H79" s="38">
         <v>337000</v>
       </c>
     </row>
     <row r="80" spans="7:8">
-      <c r="G80" s="38" t="s">
+      <c r="G80" s="17" t="s">
         <v>477</v>
       </c>
-      <c r="H80" s="39">
+      <c r="H80" s="38">
         <v>358000</v>
       </c>
     </row>
     <row r="81" spans="7:8">
-      <c r="G81" s="38" t="s">
+      <c r="G81" s="17" t="s">
         <v>478</v>
       </c>
-      <c r="H81" s="39">
+      <c r="H81" s="38">
         <v>435000</v>
       </c>
     </row>
     <row r="82" spans="7:8">
-      <c r="G82" s="38" t="s">
+      <c r="G82" s="17" t="s">
         <v>479</v>
       </c>
-      <c r="H82" s="39">
+      <c r="H82" s="38">
         <v>497000</v>
       </c>
     </row>
     <row r="83" spans="7:8">
-      <c r="G83" s="47" t="s">
+      <c r="G83" s="19" t="s">
         <v>480</v>
       </c>
-      <c r="H83" s="48">
+      <c r="H83" s="39">
         <v>433000</v>
       </c>
     </row>
     <row r="84" spans="7:8">
-      <c r="G84" s="47" t="s">
+      <c r="G84" s="19" t="s">
         <v>481</v>
       </c>
-      <c r="H84" s="48">
+      <c r="H84" s="39">
         <v>610000</v>
       </c>
     </row>
     <row r="85" spans="7:8">
-      <c r="G85" s="47" t="s">
+      <c r="G85" s="19" t="s">
         <v>482</v>
       </c>
-      <c r="H85" s="48">
+      <c r="H85" s="39">
         <v>145000</v>
       </c>
     </row>
     <row r="86" spans="7:8">
-      <c r="G86" s="47" t="s">
+      <c r="G86" s="19" t="s">
         <v>483</v>
       </c>
-      <c r="H86" s="48">
+      <c r="H86" s="39">
         <v>178000</v>
       </c>
     </row>
     <row r="87" spans="7:8">
-      <c r="G87" s="47" t="s">
+      <c r="G87" s="19" t="s">
         <v>484</v>
       </c>
-      <c r="H87" s="48">
+      <c r="H87" s="39">
         <v>259000</v>
       </c>
     </row>
     <row r="88" spans="7:8">
-      <c r="G88" s="47" t="s">
+      <c r="G88" s="19" t="s">
         <v>485</v>
       </c>
-      <c r="H88" s="48">
+      <c r="H88" s="39">
         <v>176000</v>
       </c>
     </row>
     <row r="89" spans="7:8">
-      <c r="G89" s="47" t="s">
+      <c r="G89" s="19" t="s">
         <v>486</v>
       </c>
-      <c r="H89" s="48">
+      <c r="H89" s="39">
         <v>180000</v>
       </c>
     </row>
     <row r="90" spans="7:8">
-      <c r="G90" s="47" t="s">
+      <c r="G90" s="19" t="s">
         <v>487</v>
       </c>
-      <c r="H90" s="48">
+      <c r="H90" s="39">
         <v>240000</v>
       </c>
     </row>
     <row r="91" spans="7:8">
-      <c r="G91" s="47" t="s">
+      <c r="G91" s="19" t="s">
         <v>488</v>
       </c>
-      <c r="H91" s="48">
+      <c r="H91" s="39">
         <v>288000</v>
       </c>
     </row>
     <row r="92" spans="7:8">
-      <c r="G92" s="47" t="s">
+      <c r="G92" s="19" t="s">
         <v>489</v>
       </c>
-      <c r="H92" s="48">
+      <c r="H92" s="39">
         <v>568000</v>
       </c>
     </row>
     <row r="93" spans="7:8">
-      <c r="G93" s="47" t="s">
+      <c r="G93" s="19" t="s">
         <v>490</v>
       </c>
-      <c r="H93" s="48">
+      <c r="H93" s="39">
         <v>579000</v>
       </c>
     </row>
     <row r="94" spans="7:8">
-      <c r="G94" s="47" t="s">
+      <c r="G94" s="19" t="s">
         <v>491</v>
       </c>
-      <c r="H94" s="48">
+      <c r="H94" s="39">
         <v>473000</v>
       </c>
     </row>
     <row r="95" spans="7:8">
-      <c r="G95" s="69" t="s">
+      <c r="G95" s="26" t="s">
         <v>492</v>
       </c>
-      <c r="H95" s="70">
+      <c r="H95" s="42">
         <v>43000</v>
       </c>
     </row>
     <row r="96" spans="7:8">
-      <c r="G96" s="69" t="s">
+      <c r="G96" s="26" t="s">
         <v>493</v>
       </c>
-      <c r="H96" s="70">
+      <c r="H96" s="42">
         <v>48000</v>
       </c>
     </row>
     <row r="97" spans="2:8">
-      <c r="G97" s="71" t="s">
+      <c r="G97" s="27" t="s">
         <v>494</v>
       </c>
-      <c r="H97" s="72">
+      <c r="H97" s="43">
         <v>47000</v>
       </c>
     </row>
     <row r="98" spans="2:8">
-      <c r="G98" s="69" t="s">
+      <c r="G98" s="26" t="s">
         <v>495</v>
       </c>
-      <c r="H98" s="70">
+      <c r="H98" s="42">
         <v>53000</v>
       </c>
     </row>
     <row r="99" spans="2:8">
-      <c r="G99" s="69" t="s">
+      <c r="G99" s="26" t="s">
         <v>496</v>
       </c>
-      <c r="H99" s="70">
+      <c r="H99" s="42">
         <v>54000</v>
       </c>
     </row>
     <row r="100" spans="2:8">
-      <c r="G100" s="69" t="s">
+      <c r="G100" s="26" t="s">
         <v>497</v>
       </c>
-      <c r="H100" s="70">
+      <c r="H100" s="42">
         <v>56000</v>
       </c>
     </row>
     <row r="101" spans="2:8">
-      <c r="G101" s="69" t="s">
+      <c r="G101" s="26" t="s">
         <v>498</v>
       </c>
-      <c r="H101" s="70">
+      <c r="H101" s="42">
         <v>54000</v>
       </c>
     </row>
     <row r="102" spans="2:8">
-      <c r="G102" s="38" t="s">
+      <c r="G102" s="17" t="s">
         <v>499</v>
       </c>
-      <c r="H102" s="39">
+      <c r="H102" s="38">
         <v>250000</v>
       </c>
     </row>
     <row r="103" spans="2:8">
-      <c r="G103" s="38" t="s">
+      <c r="G103" s="17" t="s">
         <v>500</v>
       </c>
-      <c r="H103" s="39">
+      <c r="H103" s="38">
         <v>303000</v>
       </c>
     </row>
     <row r="104" spans="2:8">
-      <c r="G104" s="38" t="s">
+      <c r="G104" s="17" t="s">
         <v>501</v>
       </c>
-      <c r="H104" s="39">
+      <c r="H104" s="38">
         <v>330000</v>
       </c>
     </row>
     <row r="105" spans="2:8">
-      <c r="G105" s="38" t="s">
+      <c r="G105" s="17" t="s">
         <v>502</v>
       </c>
-      <c r="H105" s="39">
+      <c r="H105" s="38">
         <v>387000</v>
       </c>
     </row>
     <row r="106" spans="2:8">
-      <c r="G106" s="38" t="s">
+      <c r="G106" s="17" t="s">
         <v>503</v>
       </c>
-      <c r="H106" s="39">
+      <c r="H106" s="38">
         <v>578000</v>
       </c>
     </row>
     <row r="107" spans="2:8">
-      <c r="G107" s="38" t="s">
+      <c r="G107" s="17" t="s">
         <v>504</v>
       </c>
-      <c r="H107" s="39">
+      <c r="H107" s="38">
         <v>722000</v>
       </c>
     </row>
     <row r="110" spans="2:8">
-      <c r="B110" s="3">
+      <c r="B110" s="28">
         <v>1000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement price group functionality: load price groups from Excel, integrate with OrderController, and update UI with price group buttons; add GiaDacBiet.xlsx data file and update version to 1.1.4
</commit_message>
<xml_diff>
--- a/app/data/BangGia.xlsx
+++ b/app/data/BangGia.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20730"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thotr\OneDrive\Desktop\Toa Hang\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\Toa Hang\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB6A82C-6513-4991-AB5D-34D9FDB5ED72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D5F48D5-8C46-4933-B886-05014203A0F6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tổng Quát" sheetId="1" r:id="rId1"/>
@@ -31,12 +31,12 @@
     <definedName name="THANHDAT_NAME">'Tổng Quát'!$AA$2:$AA$1048576</definedName>
     <definedName name="YOKO_NAME">'Tổng Quát'!$I$2:$I$1048576</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="179021"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="510">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="515">
   <si>
     <t>GS</t>
   </si>
@@ -1295,9 +1295,6 @@
     <t>HB GS 95D31R</t>
   </si>
   <si>
-    <t>100/90-10 TL 009</t>
-  </si>
-  <si>
     <t>100/90-10 Atila MX</t>
   </si>
   <si>
@@ -1566,6 +1563,24 @@
   </si>
   <si>
     <t>90/80-17 DURO</t>
+  </si>
+  <si>
+    <t>CLICL.S IN</t>
+  </si>
+  <si>
+    <t>90/90-12 V6 CSIN</t>
+  </si>
+  <si>
+    <t>100/90-10 V6 CSIN</t>
+  </si>
+  <si>
+    <t>110/70-14 TL IN</t>
+  </si>
+  <si>
+    <t>80/90-14 HD</t>
+  </si>
+  <si>
+    <t>90/90-14 HD</t>
   </si>
 </sst>
 </file>
@@ -1730,7 +1745,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1770,6 +1785,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.39991454817346722"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2017,7 +2038,7 @@
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -2049,12 +2070,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="13" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -2159,6 +2174,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="12" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="12" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2438,46 +2462,46 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AD110"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.88671875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" style="28" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="34.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" style="28" customWidth="1"/>
-    <col min="7" max="7" width="25.33203125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" style="28" customWidth="1"/>
-    <col min="9" max="9" width="31.5546875" style="2" customWidth="1"/>
-    <col min="10" max="10" width="13" style="78" customWidth="1"/>
-    <col min="11" max="11" width="28.109375" style="2" customWidth="1"/>
-    <col min="12" max="12" width="10.6640625" style="28" customWidth="1"/>
-    <col min="13" max="13" width="29.5546875" style="2" customWidth="1"/>
-    <col min="14" max="14" width="10.6640625" style="3" customWidth="1"/>
-    <col min="15" max="15" width="17.33203125" style="2" customWidth="1"/>
-    <col min="16" max="16" width="10.6640625" style="3" customWidth="1"/>
-    <col min="17" max="17" width="19.6640625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="10.6640625" style="28" customWidth="1"/>
-    <col min="19" max="19" width="28.33203125" style="2" customWidth="1"/>
-    <col min="20" max="20" width="10.6640625" style="28" customWidth="1"/>
-    <col min="21" max="21" width="20.5546875" style="2" customWidth="1"/>
-    <col min="22" max="22" width="10.6640625" style="28" customWidth="1"/>
-    <col min="23" max="23" width="21.5546875" style="2" customWidth="1"/>
-    <col min="24" max="24" width="10.6640625" style="28" customWidth="1"/>
-    <col min="25" max="25" width="26.6640625" style="2" customWidth="1"/>
-    <col min="26" max="26" width="10.6640625" style="28" customWidth="1"/>
-    <col min="27" max="27" width="33.44140625" style="2" customWidth="1"/>
-    <col min="28" max="28" width="22.5546875" style="28" customWidth="1"/>
-    <col min="29" max="29" width="19.44140625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="28" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="4" customWidth="1"/>
+    <col min="5" max="5" width="34.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" style="28" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" style="28" customWidth="1"/>
+    <col min="9" max="9" width="31.5703125" style="2" customWidth="1"/>
+    <col min="10" max="10" width="13" style="76" customWidth="1"/>
+    <col min="11" max="11" width="28.140625" style="2" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" style="28" customWidth="1"/>
+    <col min="13" max="13" width="29.5703125" style="2" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" style="3" customWidth="1"/>
+    <col min="15" max="15" width="17.28515625" style="2" customWidth="1"/>
+    <col min="16" max="16" width="10.7109375" style="3" customWidth="1"/>
+    <col min="17" max="17" width="19.7109375" style="2" customWidth="1"/>
+    <col min="18" max="18" width="10.7109375" style="28" customWidth="1"/>
+    <col min="19" max="19" width="28.28515625" style="2" customWidth="1"/>
+    <col min="20" max="20" width="10.7109375" style="28" customWidth="1"/>
+    <col min="21" max="21" width="20.5703125" style="2" customWidth="1"/>
+    <col min="22" max="22" width="10.7109375" style="28" customWidth="1"/>
+    <col min="23" max="23" width="21.5703125" style="2" customWidth="1"/>
+    <col min="24" max="24" width="10.7109375" style="28" customWidth="1"/>
+    <col min="25" max="25" width="26.7109375" style="2" customWidth="1"/>
+    <col min="26" max="26" width="10.7109375" style="28" customWidth="1"/>
+    <col min="27" max="27" width="33.42578125" style="2" customWidth="1"/>
+    <col min="28" max="28" width="22.5703125" style="28" customWidth="1"/>
+    <col min="29" max="29" width="19.42578125" style="2" customWidth="1"/>
     <col min="30" max="30" width="18" style="28" customWidth="1"/>
-    <col min="31" max="16384" width="9.109375" style="2"/>
+    <col min="31" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="1" customFormat="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
+      <c r="B1" s="43"/>
       <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
@@ -2485,19 +2509,19 @@
       <c r="E1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="32"/>
+      <c r="F1" s="30"/>
       <c r="G1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="32"/>
+      <c r="H1" s="30"/>
       <c r="I1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="47"/>
+      <c r="J1" s="45"/>
       <c r="K1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="32"/>
+      <c r="L1" s="30"/>
       <c r="M1" s="7" t="s">
         <v>6</v>
       </c>
@@ -2509,31 +2533,31 @@
       <c r="Q1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="R1" s="32"/>
+      <c r="R1" s="30"/>
       <c r="S1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="T1" s="32"/>
+      <c r="T1" s="30"/>
       <c r="U1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="V1" s="32"/>
+      <c r="V1" s="30"/>
       <c r="W1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="X1" s="32"/>
+      <c r="X1" s="30"/>
       <c r="Y1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="Z1" s="32"/>
+      <c r="Z1" s="30"/>
       <c r="AA1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="AB1" s="32"/>
-      <c r="AC1" s="29" t="s">
+      <c r="AB1" s="30"/>
+      <c r="AC1" s="80" t="s">
         <v>14</v>
       </c>
-      <c r="AD1" s="30"/>
+      <c r="AD1" s="81"/>
     </row>
     <row r="2" spans="1:30">
       <c r="A2" s="9" t="s">
@@ -2561,7 +2585,7 @@
       <c r="I2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="48">
+      <c r="J2" s="46">
         <v>152000</v>
       </c>
       <c r="K2" s="2" t="s">
@@ -2645,7 +2669,7 @@
       <c r="I3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J3" s="49">
+      <c r="J3" s="47">
         <v>204000</v>
       </c>
       <c r="K3" s="2" t="s">
@@ -2729,7 +2753,7 @@
       <c r="I4" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="J4" s="50">
+      <c r="J4" s="48">
         <v>151000</v>
       </c>
       <c r="K4" s="2" t="s">
@@ -2813,7 +2837,7 @@
       <c r="I5" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="J5" s="51">
+      <c r="J5" s="49">
         <v>192000</v>
       </c>
       <c r="K5" s="2" t="s">
@@ -2897,7 +2921,7 @@
       <c r="I6" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="J6" s="48">
+      <c r="J6" s="46">
         <v>177000</v>
       </c>
       <c r="K6" s="2" t="s">
@@ -2976,12 +3000,12 @@
         <v>93</v>
       </c>
       <c r="H7" s="28">
-        <v>231000</v>
+        <v>226000</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="J7" s="49">
+      <c r="J7" s="47">
         <v>228000</v>
       </c>
       <c r="K7" s="2" t="s">
@@ -3054,18 +3078,18 @@
         <v>107</v>
       </c>
       <c r="F8" s="28">
-        <v>226000</v>
+        <v>230000</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="H8" s="34">
-        <v>286000</v>
+      <c r="H8" s="32">
+        <v>281000</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J8" s="48">
+      <c r="J8" s="46">
         <v>212000</v>
       </c>
       <c r="K8" s="2" t="s">
@@ -3138,18 +3162,18 @@
         <v>122</v>
       </c>
       <c r="F9" s="28">
-        <v>228000</v>
+        <v>232000</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>123</v>
       </c>
       <c r="H9" s="28">
-        <v>275000</v>
+        <v>272000</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="J9" s="49">
+      <c r="J9" s="47">
         <v>287000</v>
       </c>
       <c r="K9" s="2" t="s">
@@ -3173,7 +3197,7 @@
       <c r="S9" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="T9" s="33">
+      <c r="T9" s="31">
         <v>260000</v>
       </c>
       <c r="U9" s="2" t="s">
@@ -3222,18 +3246,18 @@
         <v>137</v>
       </c>
       <c r="F10" s="28">
-        <v>282000</v>
+        <v>294000</v>
       </c>
       <c r="G10" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="H10" s="35">
-        <v>348000</v>
+      <c r="H10" s="33">
+        <v>344000</v>
       </c>
       <c r="I10" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="J10" s="52">
+      <c r="J10" s="50">
         <v>218000</v>
       </c>
       <c r="K10" s="2" t="s">
@@ -3306,18 +3330,18 @@
         <v>152</v>
       </c>
       <c r="F11" s="28">
-        <v>235000</v>
+        <v>246000</v>
       </c>
       <c r="G11" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="H11" s="35">
-        <v>370000</v>
+      <c r="H11" s="33">
+        <v>367000</v>
       </c>
       <c r="I11" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="J11" s="53">
+      <c r="J11" s="51">
         <v>270000</v>
       </c>
       <c r="K11" s="2" t="s">
@@ -3390,18 +3414,18 @@
         <v>167</v>
       </c>
       <c r="F12" s="28">
-        <v>289000</v>
+        <v>303000</v>
       </c>
       <c r="G12" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="H12" s="36">
-        <v>348000</v>
+      <c r="H12" s="34">
+        <v>344000</v>
       </c>
       <c r="I12" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="J12" s="54">
+      <c r="J12" s="52">
         <v>395000</v>
       </c>
       <c r="K12" s="2" t="s">
@@ -3460,7 +3484,7 @@
       </c>
     </row>
     <row r="13" spans="1:30">
-      <c r="B13" s="46" t="s">
+      <c r="B13" s="44" t="s">
         <v>180</v>
       </c>
       <c r="C13" s="9" t="s">
@@ -3470,19 +3494,19 @@
       <c r="E13" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="F13" s="33">
-        <v>254000</v>
+      <c r="F13" s="31">
+        <v>266000</v>
       </c>
       <c r="G13" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="H13" s="36">
-        <v>370000</v>
+      <c r="H13" s="34">
+        <v>367000</v>
       </c>
       <c r="I13" s="11" t="s">
         <v>184</v>
       </c>
-      <c r="J13" s="55">
+      <c r="J13" s="53">
         <v>431000</v>
       </c>
       <c r="K13" s="2" t="s">
@@ -3546,21 +3570,21 @@
       </c>
       <c r="D14" s="10"/>
       <c r="E14" s="13" t="s">
-        <v>195</v>
-      </c>
-      <c r="F14" s="33">
-        <v>291000</v>
+        <v>509</v>
+      </c>
+      <c r="F14" s="31">
+        <v>306000</v>
       </c>
       <c r="G14" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="H14" s="37">
+      <c r="H14" s="35">
         <v>281000</v>
       </c>
       <c r="I14" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="J14" s="51">
+      <c r="J14" s="49">
         <v>286000</v>
       </c>
       <c r="K14" s="2" t="s">
@@ -3627,18 +3651,18 @@
         <v>209</v>
       </c>
       <c r="F15" s="28">
-        <v>214000</v>
+        <v>225000</v>
       </c>
       <c r="G15" s="14" t="s">
         <v>210</v>
       </c>
-      <c r="H15" s="37">
-        <v>358000</v>
+      <c r="H15" s="35">
+        <v>349000</v>
       </c>
       <c r="I15" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="J15" s="50">
+      <c r="J15" s="48">
         <v>334000</v>
       </c>
       <c r="K15" s="2" t="s">
@@ -3696,18 +3720,18 @@
         <v>221</v>
       </c>
       <c r="F16" s="28">
-        <v>266000</v>
+        <v>280000</v>
       </c>
       <c r="G16" s="14" t="s">
         <v>222</v>
       </c>
-      <c r="H16" s="37">
+      <c r="H16" s="35">
         <v>442000</v>
       </c>
       <c r="I16" s="11" t="s">
         <v>223</v>
       </c>
-      <c r="J16" s="51">
+      <c r="J16" s="49">
         <v>269000</v>
       </c>
       <c r="K16" s="2" t="s">
@@ -3765,18 +3789,18 @@
         <v>233</v>
       </c>
       <c r="F17" s="28">
-        <v>235000</v>
+        <v>246000</v>
       </c>
       <c r="G17" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="H17" s="37">
-        <v>374000</v>
+      <c r="H17" s="35">
+        <v>352000</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="J17" s="48">
+      <c r="J17" s="46">
         <v>312000</v>
       </c>
       <c r="K17" s="2" t="s">
@@ -3834,18 +3858,18 @@
         <v>245</v>
       </c>
       <c r="F18" s="28">
-        <v>293000</v>
+        <v>307000</v>
       </c>
       <c r="G18" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="H18" s="37">
-        <v>374000</v>
+      <c r="H18" s="35">
+        <v>365000</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="J18" s="56">
+      <c r="J18" s="54">
         <v>375000</v>
       </c>
       <c r="K18" s="2" t="s">
@@ -3903,18 +3927,18 @@
         <v>257</v>
       </c>
       <c r="F19" s="28">
-        <v>267000</v>
+        <v>283000</v>
       </c>
       <c r="G19" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="H19" s="37">
-        <v>298000</v>
+      <c r="H19" s="35">
+        <v>292000</v>
       </c>
       <c r="I19" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="J19" s="53">
+      <c r="J19" s="51">
         <v>317000</v>
       </c>
       <c r="K19" s="2" t="s">
@@ -3972,18 +3996,18 @@
         <v>269</v>
       </c>
       <c r="F20" s="28">
-        <v>340000</v>
+        <v>373000</v>
       </c>
       <c r="G20" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="H20" s="37">
-        <v>366000</v>
+      <c r="H20" s="35">
+        <v>356000</v>
       </c>
       <c r="I20" s="15" t="s">
         <v>271</v>
       </c>
-      <c r="J20" s="57">
+      <c r="J20" s="55">
         <v>417000</v>
       </c>
       <c r="K20" s="2" t="s">
@@ -4004,7 +4028,7 @@
       <c r="S20" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="T20" s="33">
+      <c r="T20" s="31">
         <v>431000</v>
       </c>
       <c r="U20" s="2" t="s">
@@ -4044,18 +4068,18 @@
         <v>281</v>
       </c>
       <c r="F21" s="28">
-        <v>411000</v>
+        <v>440000</v>
       </c>
       <c r="G21" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="H21" s="37">
+      <c r="H21" s="35">
         <v>330000</v>
       </c>
       <c r="I21" s="15" t="s">
         <v>283</v>
       </c>
-      <c r="J21" s="58">
+      <c r="J21" s="56">
         <v>373000</v>
       </c>
       <c r="K21" s="2" t="s">
@@ -4086,7 +4110,7 @@
         <v>104000</v>
       </c>
       <c r="AC21" s="2" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="AD21" s="28">
         <v>350000</v>
@@ -4101,18 +4125,18 @@
         <v>290</v>
       </c>
       <c r="F22" s="28">
-        <v>320000</v>
+        <v>341000</v>
       </c>
       <c r="G22" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="H22" s="37">
+      <c r="H22" s="35">
         <v>340000</v>
       </c>
       <c r="I22" s="15" t="s">
         <v>292</v>
       </c>
-      <c r="J22" s="59">
+      <c r="J22" s="57">
         <v>467000</v>
       </c>
       <c r="K22" s="2" t="s">
@@ -4137,7 +4161,7 @@
         <v>91000</v>
       </c>
       <c r="AC22" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AD22" s="28">
         <v>480000</v>
@@ -4152,18 +4176,18 @@
         <v>299</v>
       </c>
       <c r="F23" s="28">
-        <v>345000</v>
+        <v>369000</v>
       </c>
       <c r="G23" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="H23" s="37">
-        <v>360000</v>
+      <c r="H23" s="35">
+        <v>352000</v>
       </c>
       <c r="I23" s="16" t="s">
         <v>301</v>
       </c>
-      <c r="J23" s="60">
+      <c r="J23" s="58">
         <v>299000</v>
       </c>
       <c r="K23" s="2" t="s">
@@ -4188,7 +4212,7 @@
         <v>25000</v>
       </c>
       <c r="AC23" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="AD23" s="28">
         <v>380000</v>
@@ -4199,22 +4223,22 @@
         <v>306</v>
       </c>
       <c r="D24" s="10"/>
-      <c r="E24" s="12" t="s">
+      <c r="E24" s="14" t="s">
         <v>307</v>
       </c>
-      <c r="F24" s="36">
-        <v>309000</v>
+      <c r="F24" s="35">
+        <v>323000</v>
       </c>
       <c r="G24" s="17" t="s">
         <v>308</v>
       </c>
-      <c r="H24" s="38">
+      <c r="H24" s="36">
         <v>269000</v>
       </c>
       <c r="I24" s="16" t="s">
         <v>309</v>
       </c>
-      <c r="J24" s="61">
+      <c r="J24" s="59">
         <v>321000</v>
       </c>
       <c r="K24" s="2" t="s">
@@ -4238,8 +4262,8 @@
       <c r="AB24" s="28">
         <v>30000</v>
       </c>
-      <c r="AC24" s="31" t="s">
-        <v>508</v>
+      <c r="AC24" s="29" t="s">
+        <v>507</v>
       </c>
       <c r="AD24" s="28">
         <v>330000</v>
@@ -4253,19 +4277,19 @@
       <c r="E25" s="12" t="s">
         <v>315</v>
       </c>
-      <c r="F25" s="36">
-        <v>369000</v>
+      <c r="F25" s="34">
+        <v>387000</v>
       </c>
       <c r="G25" s="14" t="s">
         <v>316</v>
       </c>
-      <c r="H25" s="37">
-        <v>396000</v>
+      <c r="H25" s="35">
+        <v>387000</v>
       </c>
       <c r="I25" s="18" t="s">
         <v>317</v>
       </c>
-      <c r="J25" s="62">
+      <c r="J25" s="60">
         <v>329000</v>
       </c>
       <c r="K25" s="2" t="s">
@@ -4289,8 +4313,8 @@
       <c r="AB25" s="28">
         <v>17000</v>
       </c>
-      <c r="AC25" s="31" t="s">
-        <v>509</v>
+      <c r="AC25" s="29" t="s">
+        <v>508</v>
       </c>
       <c r="AD25" s="28">
         <v>380000</v>
@@ -4301,22 +4325,22 @@
         <v>322</v>
       </c>
       <c r="D26" s="10"/>
-      <c r="E26" s="12" t="s">
+      <c r="E26" s="14" t="s">
         <v>323</v>
       </c>
-      <c r="F26" s="36">
-        <v>372000</v>
+      <c r="F26" s="35">
+        <v>387000</v>
       </c>
       <c r="G26" s="14" t="s">
         <v>324</v>
       </c>
-      <c r="H26" s="37">
-        <v>441000</v>
+      <c r="H26" s="35">
+        <v>431000</v>
       </c>
       <c r="I26" s="18" t="s">
         <v>325</v>
       </c>
-      <c r="J26" s="63">
+      <c r="J26" s="61">
         <v>349000</v>
       </c>
       <c r="K26" s="2" t="s">
@@ -4340,22 +4364,22 @@
         <v>329</v>
       </c>
       <c r="D27" s="10"/>
-      <c r="E27" s="12" t="s">
+      <c r="E27" s="14" t="s">
         <v>330</v>
       </c>
-      <c r="F27" s="36">
-        <v>425000</v>
+      <c r="F27" s="35">
+        <v>442000</v>
       </c>
       <c r="G27" s="14" t="s">
         <v>331</v>
       </c>
-      <c r="H27" s="37">
+      <c r="H27" s="35">
         <v>697000</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="J27" s="64">
+      <c r="J27" s="62">
         <v>280000</v>
       </c>
       <c r="K27" s="2" t="s">
@@ -4373,22 +4397,22 @@
         <v>335</v>
       </c>
       <c r="D28" s="10"/>
-      <c r="E28" s="12" t="s">
+      <c r="E28" s="14" t="s">
         <v>336</v>
       </c>
-      <c r="F28" s="36">
-        <v>522000</v>
+      <c r="F28" s="35">
+        <v>542000</v>
       </c>
       <c r="G28" s="14" t="s">
         <v>337</v>
       </c>
-      <c r="H28" s="37">
-        <v>494000</v>
+      <c r="H28" s="35">
+        <v>488000</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="J28" s="65">
+      <c r="J28" s="63">
         <v>426000</v>
       </c>
       <c r="K28" s="2" t="s">
@@ -4409,19 +4433,19 @@
       <c r="E29" s="14" t="s">
         <v>342</v>
       </c>
-      <c r="F29" s="37">
-        <v>398000</v>
+      <c r="F29" s="35">
+        <v>421000</v>
       </c>
       <c r="G29" s="14" t="s">
         <v>343</v>
       </c>
-      <c r="H29" s="37">
+      <c r="H29" s="35">
         <v>173000</v>
       </c>
       <c r="I29" s="12" t="s">
         <v>344</v>
       </c>
-      <c r="J29" s="66">
+      <c r="J29" s="64">
         <v>207000</v>
       </c>
       <c r="K29" s="2" t="s">
@@ -4439,22 +4463,22 @@
         <v>347</v>
       </c>
       <c r="D30" s="10"/>
-      <c r="E30" s="14" t="s">
+      <c r="E30" s="12" t="s">
         <v>348</v>
       </c>
-      <c r="F30" s="37">
-        <v>777000</v>
+      <c r="F30" s="34">
+        <v>819000</v>
       </c>
       <c r="G30" s="14" t="s">
         <v>349</v>
       </c>
-      <c r="H30" s="37">
+      <c r="H30" s="35">
         <v>207000</v>
       </c>
       <c r="I30" s="12" t="s">
         <v>350</v>
       </c>
-      <c r="J30" s="66">
+      <c r="J30" s="64">
         <v>257000</v>
       </c>
       <c r="K30" s="2" t="s">
@@ -4472,22 +4496,22 @@
         <v>353</v>
       </c>
       <c r="D31" s="10"/>
-      <c r="E31" s="19" t="s">
+      <c r="E31" s="77" t="s">
         <v>354</v>
       </c>
-      <c r="F31" s="39">
-        <v>341000</v>
+      <c r="F31" s="33">
+        <v>348000</v>
       </c>
       <c r="G31" s="14" t="s">
         <v>355</v>
       </c>
-      <c r="H31" s="37">
+      <c r="H31" s="35">
         <v>302000</v>
       </c>
       <c r="I31" s="20" t="s">
         <v>356</v>
       </c>
-      <c r="J31" s="67">
+      <c r="J31" s="65">
         <v>295000</v>
       </c>
       <c r="K31" s="2" t="s">
@@ -4505,22 +4529,22 @@
         <v>359</v>
       </c>
       <c r="D32" s="10"/>
-      <c r="E32" s="19" t="s">
+      <c r="E32" s="77" t="s">
         <v>360</v>
       </c>
-      <c r="F32" s="39">
-        <v>388000</v>
+      <c r="F32" s="33">
+        <v>401000</v>
       </c>
       <c r="G32" s="17" t="s">
         <v>361</v>
       </c>
-      <c r="H32" s="38">
-        <v>381000</v>
+      <c r="H32" s="36">
+        <v>377000</v>
       </c>
       <c r="I32" s="20" t="s">
         <v>362</v>
       </c>
-      <c r="J32" s="67">
+      <c r="J32" s="65">
         <v>405000</v>
       </c>
       <c r="K32" s="2" t="s">
@@ -4541,19 +4565,19 @@
       <c r="E33" s="14" t="s">
         <v>366</v>
       </c>
-      <c r="F33" s="37">
-        <v>648000</v>
+      <c r="F33" s="35">
+        <v>692000</v>
       </c>
       <c r="G33" s="14" t="s">
         <v>367</v>
       </c>
-      <c r="H33" s="39">
-        <v>388000</v>
+      <c r="H33" s="37">
+        <v>378000</v>
       </c>
       <c r="I33" s="14" t="s">
         <v>368</v>
       </c>
-      <c r="J33" s="68">
+      <c r="J33" s="66">
         <v>641000</v>
       </c>
       <c r="K33" s="2" t="s">
@@ -4573,19 +4597,19 @@
       <c r="E34" s="14" t="s">
         <v>372</v>
       </c>
-      <c r="F34" s="37">
-        <v>793000</v>
+      <c r="F34" s="35">
+        <v>819000</v>
       </c>
       <c r="G34" s="14" t="s">
         <v>373</v>
       </c>
-      <c r="H34" s="39">
-        <v>413000</v>
+      <c r="H34" s="37">
+        <v>403000</v>
       </c>
       <c r="I34" s="14" t="s">
         <v>374</v>
       </c>
-      <c r="J34" s="69">
+      <c r="J34" s="67">
         <v>754000</v>
       </c>
       <c r="K34" s="2" t="s">
@@ -4605,19 +4629,19 @@
       <c r="E35" s="14" t="s">
         <v>378</v>
       </c>
-      <c r="F35" s="44">
-        <v>747000</v>
+      <c r="F35" s="42">
+        <v>760000</v>
       </c>
       <c r="G35" s="14" t="s">
         <v>379</v>
       </c>
-      <c r="H35" s="37">
+      <c r="H35" s="35">
         <v>309000</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="J35" s="70">
+      <c r="J35" s="68">
         <v>312000</v>
       </c>
       <c r="K35" s="2" t="s">
@@ -4637,19 +4661,19 @@
       <c r="E36" s="14" t="s">
         <v>384</v>
       </c>
-      <c r="F36" s="44">
-        <v>882000</v>
+      <c r="F36" s="42">
+        <v>895000</v>
       </c>
       <c r="G36" s="14" t="s">
         <v>385</v>
       </c>
-      <c r="H36" s="37">
-        <v>411000</v>
+      <c r="H36" s="35">
+        <v>405000</v>
       </c>
       <c r="I36" s="11" t="s">
         <v>386</v>
       </c>
-      <c r="J36" s="70">
+      <c r="J36" s="68">
         <v>381000</v>
       </c>
       <c r="K36" s="2" t="s">
@@ -4669,19 +4693,19 @@
       <c r="E37" s="14" t="s">
         <v>390</v>
       </c>
-      <c r="F37" s="37">
-        <v>356000</v>
+      <c r="F37" s="35">
+        <v>377000</v>
       </c>
       <c r="G37" s="14" t="s">
         <v>391</v>
       </c>
-      <c r="H37" s="37">
+      <c r="H37" s="35">
         <v>473000</v>
       </c>
       <c r="I37" s="13" t="s">
         <v>392</v>
       </c>
-      <c r="J37" s="71">
+      <c r="J37" s="69">
         <v>365000</v>
       </c>
       <c r="K37" s="2" t="s">
@@ -4698,19 +4722,19 @@
       <c r="E38" s="14" t="s">
         <v>395</v>
       </c>
-      <c r="F38" s="37">
-        <v>369000</v>
+      <c r="F38" s="35">
+        <v>319000</v>
       </c>
       <c r="G38" s="14" t="s">
         <v>396</v>
       </c>
-      <c r="H38" s="37">
-        <v>329000</v>
+      <c r="H38" s="35">
+        <v>322000</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="J38" s="72">
+      <c r="J38" s="70">
         <v>501000</v>
       </c>
     </row>
@@ -4718,22 +4742,22 @@
       <c r="C39" s="9" t="s">
         <v>398</v>
       </c>
-      <c r="E39" s="14" t="s">
+      <c r="E39" s="12" t="s">
         <v>399</v>
       </c>
-      <c r="F39" s="37">
-        <v>465000</v>
+      <c r="F39" s="34">
+        <v>492000</v>
       </c>
       <c r="G39" s="14" t="s">
         <v>400</v>
       </c>
-      <c r="H39" s="37">
-        <v>385000</v>
+      <c r="H39" s="35">
+        <v>375000</v>
       </c>
       <c r="I39" s="14" t="s">
         <v>401</v>
       </c>
-      <c r="J39" s="73">
+      <c r="J39" s="71">
         <v>740000</v>
       </c>
     </row>
@@ -4744,19 +4768,19 @@
       <c r="E40" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="F40" s="37">
-        <v>543000</v>
+      <c r="F40" s="35">
+        <v>577000</v>
       </c>
       <c r="G40" s="14" t="s">
         <v>404</v>
       </c>
-      <c r="H40" s="37">
+      <c r="H40" s="35">
         <v>437000</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="J40" s="74">
+      <c r="J40" s="72">
         <v>278000</v>
       </c>
     </row>
@@ -4767,19 +4791,19 @@
       <c r="E41" s="14" t="s">
         <v>407</v>
       </c>
-      <c r="F41" s="37">
-        <v>778000</v>
+      <c r="F41" s="35">
+        <v>825000</v>
       </c>
       <c r="G41" s="14" t="s">
         <v>408</v>
       </c>
-      <c r="H41" s="37">
-        <v>566000</v>
+      <c r="H41" s="35">
+        <v>564000</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="J41" s="56">
+      <c r="J41" s="54">
         <v>351000</v>
       </c>
     </row>
@@ -4790,19 +4814,19 @@
       <c r="E42" s="14" t="s">
         <v>411</v>
       </c>
-      <c r="F42" s="37">
-        <v>337000</v>
+      <c r="F42" s="35">
+        <v>357000</v>
       </c>
       <c r="G42" s="14" t="s">
         <v>412</v>
       </c>
-      <c r="H42" s="37">
+      <c r="H42" s="35">
         <v>636000</v>
       </c>
       <c r="I42" s="12" t="s">
         <v>413</v>
       </c>
-      <c r="J42" s="75">
+      <c r="J42" s="73">
         <v>300000</v>
       </c>
     </row>
@@ -4813,19 +4837,19 @@
       <c r="E43" s="14" t="s">
         <v>415</v>
       </c>
-      <c r="F43" s="44">
-        <v>440000</v>
+      <c r="F43" s="42">
+        <v>461000</v>
       </c>
       <c r="G43" s="14" t="s">
         <v>416</v>
       </c>
-      <c r="H43" s="37">
+      <c r="H43" s="35">
         <v>707000</v>
       </c>
       <c r="I43" s="12" t="s">
         <v>417</v>
       </c>
-      <c r="J43" s="76">
+      <c r="J43" s="74">
         <v>322000</v>
       </c>
     </row>
@@ -4834,151 +4858,151 @@
         <v>418</v>
       </c>
       <c r="E44" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="F44" s="28">
+        <v>344000</v>
+      </c>
+      <c r="G44" s="14" t="s">
         <v>419</v>
       </c>
-      <c r="F44" s="28">
-        <v>335000</v>
-      </c>
-      <c r="G44" s="14" t="s">
+      <c r="H44" s="35">
+        <v>413000</v>
+      </c>
+      <c r="I44" s="22" t="s">
         <v>420</v>
       </c>
-      <c r="H44" s="37">
-        <v>420000</v>
-      </c>
-      <c r="I44" s="22" t="s">
-        <v>421</v>
-      </c>
-      <c r="J44" s="77">
+      <c r="J44" s="75">
         <v>329000</v>
       </c>
     </row>
     <row r="45" spans="3:13">
       <c r="C45" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E45" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="F45" s="28">
+        <v>439000</v>
+      </c>
+      <c r="G45" s="14" t="s">
         <v>423</v>
       </c>
-      <c r="F45" s="28">
-        <v>448000</v>
-      </c>
-      <c r="G45" s="14" t="s">
+      <c r="H45" s="35">
+        <v>430000</v>
+      </c>
+      <c r="I45" s="22" t="s">
         <v>424</v>
       </c>
-      <c r="H45" s="37">
-        <v>430000</v>
-      </c>
-      <c r="I45" s="22" t="s">
-        <v>425</v>
-      </c>
-      <c r="J45" s="77">
+      <c r="J45" s="75">
         <v>445000</v>
       </c>
     </row>
     <row r="46" spans="3:13">
       <c r="C46" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E46" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="F46" s="28">
+        <v>448000</v>
+      </c>
+      <c r="G46" s="14" t="s">
         <v>427</v>
       </c>
-      <c r="F46" s="28">
-        <v>402000</v>
-      </c>
-      <c r="G46" s="14" t="s">
-        <v>428</v>
-      </c>
-      <c r="H46" s="37">
+      <c r="H46" s="35">
         <v>400000</v>
       </c>
       <c r="I46" s="22"/>
-      <c r="J46" s="77"/>
+      <c r="J46" s="75"/>
     </row>
     <row r="47" spans="3:13">
       <c r="C47" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="E47" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="F47" s="28">
+        <v>428000</v>
+      </c>
+      <c r="G47" s="14" t="s">
         <v>430</v>
       </c>
-      <c r="F47" s="28">
-        <v>469000</v>
-      </c>
-      <c r="G47" s="14" t="s">
-        <v>431</v>
-      </c>
-      <c r="H47" s="37">
+      <c r="H47" s="35">
         <v>382000</v>
       </c>
     </row>
     <row r="48" spans="3:13">
       <c r="C48" s="9" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E48" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="F48" s="28">
+        <v>495000</v>
+      </c>
+      <c r="G48" s="2" t="s">
         <v>433</v>
-      </c>
-      <c r="F48" s="28">
-        <v>537000</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>434</v>
       </c>
       <c r="H48" s="28">
         <v>443000</v>
       </c>
     </row>
     <row r="49" spans="5:8">
-      <c r="E49" s="12" t="s">
+      <c r="E49" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="F49" s="28">
+        <v>547000</v>
+      </c>
+      <c r="G49" s="2" t="s">
         <v>435</v>
-      </c>
-      <c r="F49" s="36">
-        <v>180000</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>436</v>
       </c>
       <c r="H49" s="28">
         <v>488000</v>
       </c>
     </row>
     <row r="50" spans="5:8">
-      <c r="E50" s="12" t="s">
+      <c r="E50" s="14" t="s">
+        <v>434</v>
+      </c>
+      <c r="F50" s="35">
+        <v>180000</v>
+      </c>
+      <c r="G50" s="2" t="s">
         <v>437</v>
-      </c>
-      <c r="F50" s="36">
-        <v>230000</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>438</v>
       </c>
       <c r="H50" s="28">
         <v>548000</v>
       </c>
     </row>
     <row r="51" spans="5:8">
-      <c r="E51" s="2" t="s">
+      <c r="E51" s="14" t="s">
+        <v>436</v>
+      </c>
+      <c r="F51" s="35">
+        <v>230000</v>
+      </c>
+      <c r="G51" s="14" t="s">
         <v>439</v>
       </c>
-      <c r="F51" s="28">
-        <v>46000</v>
-      </c>
-      <c r="G51" s="14" t="s">
-        <v>440</v>
-      </c>
-      <c r="H51" s="37">
-        <v>446000</v>
+      <c r="H51" s="35">
+        <v>447000</v>
       </c>
     </row>
     <row r="52" spans="5:8">
       <c r="E52" s="2" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="F52" s="28">
         <v>48000</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="H52" s="28">
         <v>431000</v>
@@ -4986,13 +5010,13 @@
     </row>
     <row r="53" spans="5:8">
       <c r="E53" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="F53" s="28">
+        <v>50000</v>
+      </c>
+      <c r="G53" s="2" t="s">
         <v>443</v>
-      </c>
-      <c r="F53" s="28">
-        <v>55000</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>444</v>
       </c>
       <c r="H53" s="28">
         <v>483000</v>
@@ -5000,13 +5024,13 @@
     </row>
     <row r="54" spans="5:8">
       <c r="E54" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="F54" s="28">
+        <v>58000</v>
+      </c>
+      <c r="G54" s="2" t="s">
         <v>445</v>
-      </c>
-      <c r="F54" s="28">
-        <v>56000</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>446</v>
       </c>
       <c r="H54" s="28">
         <v>541000</v>
@@ -5014,13 +5038,13 @@
     </row>
     <row r="55" spans="5:8">
       <c r="E55" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="F55" s="28">
+        <v>59000</v>
+      </c>
+      <c r="G55" s="2" t="s">
         <v>447</v>
-      </c>
-      <c r="F55" s="28">
-        <v>56000</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>448</v>
       </c>
       <c r="H55" s="28">
         <v>478000</v>
@@ -5028,13 +5052,13 @@
     </row>
     <row r="56" spans="5:8">
       <c r="E56" s="2" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="F56" s="28">
         <v>59000</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="H56" s="28">
         <v>589000</v>
@@ -5042,13 +5066,13 @@
     </row>
     <row r="57" spans="5:8">
       <c r="E57" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="F57" s="28">
+        <v>61000</v>
+      </c>
+      <c r="G57" s="2" t="s">
         <v>451</v>
-      </c>
-      <c r="F57" s="28">
-        <v>60000</v>
-      </c>
-      <c r="G57" s="2" t="s">
-        <v>452</v>
       </c>
       <c r="H57" s="28">
         <v>637000</v>
@@ -5056,67 +5080,79 @@
     </row>
     <row r="58" spans="5:8">
       <c r="E58" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="F58" s="28">
+        <v>60000</v>
+      </c>
+      <c r="G58" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="F58" s="28">
-        <v>358000</v>
-      </c>
-      <c r="G58" s="14" t="s">
-        <v>454</v>
-      </c>
-      <c r="H58" s="37">
-        <v>541000</v>
+      <c r="H58" s="35">
+        <v>537000</v>
       </c>
     </row>
     <row r="59" spans="5:8">
       <c r="E59" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="F59" s="28">
+        <v>358000</v>
+      </c>
+      <c r="G59" s="19" t="s">
         <v>455</v>
       </c>
-      <c r="F59" s="28">
-        <v>320000</v>
-      </c>
-      <c r="G59" s="19" t="s">
+      <c r="H59" s="37">
+        <v>507000</v>
+      </c>
+    </row>
+    <row r="60" spans="5:8">
+      <c r="E60" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="F60" s="28">
+        <v>357000</v>
+      </c>
+      <c r="G60" s="23" t="s">
         <v>456</v>
       </c>
-      <c r="H59" s="39">
-        <v>515000</v>
-      </c>
-    </row>
-    <row r="60" spans="5:8">
-      <c r="G60" s="23" t="s">
+      <c r="H60" s="38">
+        <v>701000</v>
+      </c>
+    </row>
+    <row r="61" spans="5:8">
+      <c r="E61" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="F61" s="28">
+        <v>492000</v>
+      </c>
+      <c r="G61" s="23" t="s">
         <v>457</v>
       </c>
-      <c r="H60" s="40">
-        <v>701000</v>
-      </c>
-    </row>
-    <row r="61" spans="5:8">
-      <c r="G61" s="23" t="s">
-        <v>458</v>
-      </c>
-      <c r="H61" s="40">
+      <c r="H61" s="38">
         <v>794000</v>
       </c>
     </row>
     <row r="62" spans="5:8">
       <c r="G62" s="17" t="s">
-        <v>459</v>
-      </c>
-      <c r="H62" s="38">
-        <v>628000</v>
+        <v>458</v>
+      </c>
+      <c r="H62" s="36">
+        <v>618000</v>
       </c>
     </row>
     <row r="63" spans="5:8">
       <c r="G63" s="17" t="s">
-        <v>460</v>
-      </c>
-      <c r="H63" s="38">
-        <v>747000</v>
+        <v>459</v>
+      </c>
+      <c r="H63" s="36">
+        <v>737000</v>
       </c>
     </row>
     <row r="64" spans="5:8">
       <c r="G64" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="H64" s="28">
         <v>563000</v>
@@ -5124,7 +5160,7 @@
     </row>
     <row r="65" spans="7:8">
       <c r="G65" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="H65" s="28">
         <v>682000</v>
@@ -5132,7 +5168,7 @@
     </row>
     <row r="66" spans="7:8">
       <c r="G66" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="H66" s="28">
         <v>647000</v>
@@ -5140,7 +5176,7 @@
     </row>
     <row r="67" spans="7:8">
       <c r="G67" s="2" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="H67" s="28">
         <v>511000</v>
@@ -5148,7 +5184,7 @@
     </row>
     <row r="68" spans="7:8">
       <c r="G68" s="2" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="H68" s="28">
         <v>503000</v>
@@ -5156,7 +5192,7 @@
     </row>
     <row r="69" spans="7:8">
       <c r="G69" s="2" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="H69" s="28">
         <v>802000</v>
@@ -5164,15 +5200,15 @@
     </row>
     <row r="70" spans="7:8">
       <c r="G70" s="2" t="s">
-        <v>467</v>
-      </c>
-      <c r="H70" s="34">
+        <v>466</v>
+      </c>
+      <c r="H70" s="32">
         <v>903000</v>
       </c>
     </row>
     <row r="71" spans="7:8">
       <c r="G71" s="2" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="H71" s="28">
         <v>823000</v>
@@ -5180,293 +5216,310 @@
     </row>
     <row r="72" spans="7:8">
       <c r="G72" s="20" t="s">
-        <v>469</v>
-      </c>
-      <c r="H72" s="41">
-        <v>268000</v>
+        <v>468</v>
+      </c>
+      <c r="H72" s="39">
+        <v>266000</v>
       </c>
     </row>
     <row r="73" spans="7:8">
       <c r="G73" s="20" t="s">
-        <v>470</v>
-      </c>
-      <c r="H73" s="41">
-        <v>325000</v>
+        <v>469</v>
+      </c>
+      <c r="H73" s="39">
+        <v>323000</v>
       </c>
     </row>
     <row r="74" spans="7:8">
       <c r="G74" s="24" t="s">
-        <v>471</v>
-      </c>
-      <c r="H74" s="41">
-        <v>297000</v>
+        <v>470</v>
+      </c>
+      <c r="H74" s="39">
+        <v>293000</v>
       </c>
     </row>
     <row r="75" spans="7:8">
       <c r="G75" s="24" t="s">
-        <v>472</v>
-      </c>
-      <c r="H75" s="41">
-        <v>359000</v>
+        <v>471</v>
+      </c>
+      <c r="H75" s="39">
+        <v>351000</v>
       </c>
     </row>
     <row r="76" spans="7:8">
       <c r="G76" s="14" t="s">
-        <v>473</v>
-      </c>
-      <c r="H76" s="37">
-        <v>297000</v>
+        <v>472</v>
+      </c>
+      <c r="H76" s="35">
+        <v>298000</v>
       </c>
     </row>
     <row r="77" spans="7:8">
       <c r="G77" s="14" t="s">
-        <v>474</v>
-      </c>
-      <c r="H77" s="37">
-        <v>394000</v>
+        <v>473</v>
+      </c>
+      <c r="H77" s="35">
+        <v>395000</v>
       </c>
     </row>
     <row r="78" spans="7:8">
       <c r="G78" s="25" t="s">
-        <v>475</v>
-      </c>
-      <c r="H78" s="34">
+        <v>474</v>
+      </c>
+      <c r="H78" s="32">
         <v>446000</v>
       </c>
     </row>
     <row r="79" spans="7:8">
       <c r="G79" s="17" t="s">
-        <v>476</v>
-      </c>
-      <c r="H79" s="38">
-        <v>337000</v>
+        <v>475</v>
+      </c>
+      <c r="H79" s="36">
+        <v>330000</v>
       </c>
     </row>
     <row r="80" spans="7:8">
       <c r="G80" s="17" t="s">
-        <v>477</v>
-      </c>
-      <c r="H80" s="38">
-        <v>358000</v>
+        <v>476</v>
+      </c>
+      <c r="H80" s="36">
+        <v>352000</v>
       </c>
     </row>
     <row r="81" spans="7:8">
       <c r="G81" s="17" t="s">
-        <v>478</v>
-      </c>
-      <c r="H81" s="38">
+        <v>477</v>
+      </c>
+      <c r="H81" s="36">
         <v>435000</v>
       </c>
     </row>
     <row r="82" spans="7:8">
       <c r="G82" s="17" t="s">
-        <v>479</v>
-      </c>
-      <c r="H82" s="38">
+        <v>478</v>
+      </c>
+      <c r="H82" s="36">
         <v>497000</v>
       </c>
     </row>
     <row r="83" spans="7:8">
       <c r="G83" s="19" t="s">
-        <v>480</v>
-      </c>
-      <c r="H83" s="39">
+        <v>479</v>
+      </c>
+      <c r="H83" s="37">
         <v>433000</v>
       </c>
     </row>
     <row r="84" spans="7:8">
       <c r="G84" s="19" t="s">
-        <v>481</v>
-      </c>
-      <c r="H84" s="39">
+        <v>480</v>
+      </c>
+      <c r="H84" s="37">
         <v>610000</v>
       </c>
     </row>
     <row r="85" spans="7:8">
       <c r="G85" s="19" t="s">
-        <v>482</v>
-      </c>
-      <c r="H85" s="39">
+        <v>481</v>
+      </c>
+      <c r="H85" s="37">
         <v>145000</v>
       </c>
     </row>
     <row r="86" spans="7:8">
       <c r="G86" s="19" t="s">
-        <v>483</v>
-      </c>
-      <c r="H86" s="39">
+        <v>482</v>
+      </c>
+      <c r="H86" s="37">
         <v>178000</v>
       </c>
     </row>
     <row r="87" spans="7:8">
       <c r="G87" s="19" t="s">
-        <v>484</v>
-      </c>
-      <c r="H87" s="39">
+        <v>483</v>
+      </c>
+      <c r="H87" s="37">
         <v>259000</v>
       </c>
     </row>
     <row r="88" spans="7:8">
       <c r="G88" s="19" t="s">
-        <v>485</v>
-      </c>
-      <c r="H88" s="39">
-        <v>176000</v>
+        <v>484</v>
+      </c>
+      <c r="H88" s="37">
+        <v>173000</v>
       </c>
     </row>
     <row r="89" spans="7:8">
       <c r="G89" s="19" t="s">
-        <v>486</v>
-      </c>
-      <c r="H89" s="39">
-        <v>180000</v>
+        <v>485</v>
+      </c>
+      <c r="H89" s="37">
+        <v>177000</v>
       </c>
     </row>
     <row r="90" spans="7:8">
       <c r="G90" s="19" t="s">
-        <v>487</v>
-      </c>
-      <c r="H90" s="39">
-        <v>240000</v>
+        <v>486</v>
+      </c>
+      <c r="H90" s="37">
+        <v>236000</v>
       </c>
     </row>
     <row r="91" spans="7:8">
       <c r="G91" s="19" t="s">
-        <v>488</v>
-      </c>
-      <c r="H91" s="39">
+        <v>487</v>
+      </c>
+      <c r="H91" s="37">
         <v>288000</v>
       </c>
     </row>
     <row r="92" spans="7:8">
       <c r="G92" s="19" t="s">
-        <v>489</v>
-      </c>
-      <c r="H92" s="39">
+        <v>488</v>
+      </c>
+      <c r="H92" s="37">
         <v>568000</v>
       </c>
     </row>
     <row r="93" spans="7:8">
       <c r="G93" s="19" t="s">
-        <v>490</v>
-      </c>
-      <c r="H93" s="39">
+        <v>489</v>
+      </c>
+      <c r="H93" s="37">
         <v>579000</v>
       </c>
     </row>
     <row r="94" spans="7:8">
       <c r="G94" s="19" t="s">
-        <v>491</v>
-      </c>
-      <c r="H94" s="39">
+        <v>490</v>
+      </c>
+      <c r="H94" s="37">
         <v>473000</v>
       </c>
     </row>
     <row r="95" spans="7:8">
       <c r="G95" s="26" t="s">
-        <v>492</v>
-      </c>
-      <c r="H95" s="42">
+        <v>491</v>
+      </c>
+      <c r="H95" s="40">
         <v>43000</v>
       </c>
     </row>
     <row r="96" spans="7:8">
       <c r="G96" s="26" t="s">
+        <v>492</v>
+      </c>
+      <c r="H96" s="40">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="97" spans="2:9">
+      <c r="G97" s="27" t="s">
         <v>493</v>
       </c>
-      <c r="H96" s="42">
-        <v>48000</v>
-      </c>
-    </row>
-    <row r="97" spans="2:8">
-      <c r="G97" s="27" t="s">
+      <c r="H97" s="41">
+        <v>47000</v>
+      </c>
+    </row>
+    <row r="98" spans="2:9">
+      <c r="G98" s="26" t="s">
         <v>494</v>
       </c>
-      <c r="H97" s="43">
-        <v>47000</v>
-      </c>
-    </row>
-    <row r="98" spans="2:8">
-      <c r="G98" s="26" t="s">
+      <c r="H98" s="40">
+        <v>53000</v>
+      </c>
+    </row>
+    <row r="99" spans="2:9">
+      <c r="G99" s="26" t="s">
         <v>495</v>
       </c>
-      <c r="H98" s="42">
-        <v>53000</v>
-      </c>
-    </row>
-    <row r="99" spans="2:8">
-      <c r="G99" s="26" t="s">
+      <c r="H99" s="40">
+        <v>54000</v>
+      </c>
+    </row>
+    <row r="100" spans="2:9">
+      <c r="G100" s="26" t="s">
         <v>496</v>
       </c>
-      <c r="H99" s="42">
+      <c r="H100" s="40">
+        <v>56000</v>
+      </c>
+      <c r="I100" s="14"/>
+    </row>
+    <row r="101" spans="2:9">
+      <c r="G101" s="26" t="s">
+        <v>497</v>
+      </c>
+      <c r="H101" s="40">
         <v>54000</v>
       </c>
     </row>
-    <row r="100" spans="2:8">
-      <c r="G100" s="26" t="s">
-        <v>497</v>
-      </c>
-      <c r="H100" s="42">
-        <v>56000</v>
-      </c>
-    </row>
-    <row r="101" spans="2:8">
-      <c r="G101" s="26" t="s">
+    <row r="102" spans="2:9">
+      <c r="G102" s="14" t="s">
         <v>498</v>
       </c>
-      <c r="H101" s="42">
-        <v>54000</v>
-      </c>
-    </row>
-    <row r="102" spans="2:8">
-      <c r="G102" s="17" t="s">
+      <c r="H102" s="35">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="103" spans="2:9">
+      <c r="G103" s="14" t="s">
         <v>499</v>
       </c>
-      <c r="H102" s="38">
-        <v>250000</v>
-      </c>
-    </row>
-    <row r="103" spans="2:8">
-      <c r="G103" s="17" t="s">
+      <c r="H103" s="35">
+        <v>303000</v>
+      </c>
+    </row>
+    <row r="104" spans="2:9">
+      <c r="G104" s="14" t="s">
         <v>500</v>
       </c>
-      <c r="H103" s="38">
-        <v>303000</v>
-      </c>
-    </row>
-    <row r="104" spans="2:8">
-      <c r="G104" s="17" t="s">
+      <c r="H104" s="35">
+        <v>324000</v>
+      </c>
+    </row>
+    <row r="105" spans="2:9">
+      <c r="G105" s="14" t="s">
         <v>501</v>
       </c>
-      <c r="H104" s="38">
-        <v>330000</v>
-      </c>
-    </row>
-    <row r="105" spans="2:8">
-      <c r="G105" s="17" t="s">
+      <c r="H105" s="35">
+        <v>380000</v>
+      </c>
+    </row>
+    <row r="106" spans="2:9">
+      <c r="G106" s="14" t="s">
         <v>502</v>
       </c>
-      <c r="H105" s="38">
-        <v>387000</v>
-      </c>
-    </row>
-    <row r="106" spans="2:8">
-      <c r="G106" s="17" t="s">
+      <c r="H106" s="35">
+        <v>573000</v>
+      </c>
+    </row>
+    <row r="107" spans="2:9">
+      <c r="G107" s="14" t="s">
         <v>503</v>
       </c>
-      <c r="H106" s="38">
-        <v>578000</v>
-      </c>
-    </row>
-    <row r="107" spans="2:8">
-      <c r="G107" s="17" t="s">
-        <v>504</v>
-      </c>
-      <c r="H107" s="38">
-        <v>722000</v>
-      </c>
-    </row>
-    <row r="110" spans="2:8">
+      <c r="H107" s="35">
+        <v>7180000</v>
+      </c>
+    </row>
+    <row r="108" spans="2:9">
+      <c r="G108" s="78" t="s">
+        <v>510</v>
+      </c>
+      <c r="H108" s="79">
+        <v>310000</v>
+      </c>
+    </row>
+    <row r="109" spans="2:9">
+      <c r="G109" s="78" t="s">
+        <v>511</v>
+      </c>
+      <c r="H109" s="79">
+        <v>344000</v>
+      </c>
+    </row>
+    <row r="110" spans="2:9">
       <c r="B110" s="28">
         <v>1000</v>
       </c>

</xml_diff>